<commit_message>
Bug list: PT-33 (CI runner pinned to ubuntu-24.04, actions on Node 24)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1063" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="701">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1255,6 +1255,39 @@
     <t xml:space="preserve">b96269a</t>
   </si>
   <si>
+    <t xml:space="preserve">PT-33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI / GitHub Actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.github/workflows/ci.yml (4 job), .github/workflows/apk-device.yml (2 job): runs-on và phiên bản action</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Actions từ 19/10/2026 (ubuntu-latest chuyển sang Ubuntu 26)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quy trình CI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi lần chạy CI có cảnh báo "The ubuntu-latest label will migrate to Ubuntu 26 beginning October 19, 2026" và "Node.js 20 is deprecated" cho checkout/setup-node/setup-java/upload-artifact@v4. Chưa hỏng, nhưng từ 19/10 mọi job (Android SDK, Java, Chromium cho E2E, emulator) sẽ chạy trên image chưa thử mà không ai đổi gì; hỏng thì không deploy được bản sửa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">runs-on: ubuntu-latest là nhãn trôi: GitHub tự đổi image bên dưới theo lịch của họ. Các action @v4 chạy trên Node 20 đã bị khai tử. Cảnh báo chỉ nằm trong annotation, CI vẫn xanh nên không ai đọc.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ghim runs-on: ubuntu-24.04 cho cả 6 job (đúng image ubuntu-latest đang dùng); checkout, setup-node, setup-java lên v5, upload-artifact lên v6, setup-python lên v6.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI nhánh online-v1.7 run 37278811859 và main run 37279049646 xanh, không còn annotation cảnh báo; APK on Android emulator run 37278843002 xanh (release-apk: 1.7.60 → 1.7.62 trên Android 11, WebView 83; test-build: luồng đầy đủ).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ghim phiên bản image runner và action, đổi có chủ đích. Sau mỗi lần chạy đọc cả annotation cảnh báo, không chỉ xanh/đỏ. Repo lotus-pos-saas mới ghim ci.yml (SAAS-25); apk-device.yml bên đó vẫn ubuntu-latest.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5706299; cùng hướng sửa SAAS-25 (lotus-pos-saas 34b760d)</t>
+  </si>
+  <si>
     <t xml:space="preserve">SAAS-01</t>
   </si>
   <si>
@@ -1737,9 +1770,6 @@
   </si>
   <si>
     <t xml:space="preserve">GitHub Actions (job e2e)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quy trình CI</t>
   </si>
   <si>
     <t xml:space="preserve">4 lần push liên tiếp (317e13e → d7414f1) đều đỏ ở job e2e; deploy bị bỏ qua. Không ai biết cho tới khi GitHub gửi email.</t>
@@ -2576,7 +2606,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2621,15 +2651,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2755,8 +2789,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O65" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O65"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O66"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3019,7 +3053,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O65"/>
+  <dimension ref="A1:O66"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -4595,43 +4629,43 @@
         <v>357</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="F34" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="G34" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H34" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="I34" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="G34" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H34" s="6" t="s">
+      <c r="J34" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="I34" s="6" t="s">
+      <c r="K34" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="J34" s="6" t="s">
+      <c r="L34" s="6" t="s">
         <v>365</v>
       </c>
-      <c r="K34" s="6" t="s">
+      <c r="M34" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="L34" s="6" t="s">
+      <c r="N34" s="6" t="s">
         <v>367</v>
-      </c>
-      <c r="M34" s="6" t="s">
-        <v>368</v>
-      </c>
-      <c r="N34" s="6" t="s">
-        <v>369</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>37</v>
@@ -4639,28 +4673,28 @@
     </row>
     <row r="35" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C35" s="6" t="s">
+      <c r="D35" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="E35" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="G35" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H35" s="6" t="s">
         <v>374</v>
-      </c>
-      <c r="G35" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H35" s="6" t="s">
-        <v>363</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>375</v>
@@ -4678,7 +4712,7 @@
         <v>379</v>
       </c>
       <c r="N35" s="6" t="s">
-        <v>369</v>
+        <v>380</v>
       </c>
       <c r="O35" s="6" t="s">
         <v>37</v>
@@ -4686,46 +4720,46 @@
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>386</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>387</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="M36" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="N36" s="6" t="s">
         <v>380</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>381</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>383</v>
-      </c>
-      <c r="G36" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>363</v>
-      </c>
-      <c r="I36" s="6" t="s">
-        <v>384</v>
-      </c>
-      <c r="J36" s="6" t="s">
-        <v>385</v>
-      </c>
-      <c r="K36" s="6" t="s">
-        <v>386</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>387</v>
-      </c>
-      <c r="M36" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="N36" s="6" t="s">
-        <v>389</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>37</v>
@@ -4733,46 +4767,46 @@
     </row>
     <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>146</v>
+        <v>392</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G37" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H37" s="6" t="s">
-        <v>393</v>
+        <v>374</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="K37" s="6" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L37" s="6" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="M37" s="6" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="N37" s="6" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="O37" s="6" t="s">
         <v>37</v>
@@ -4780,46 +4814,46 @@
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>401</v>
+        <v>146</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>402</v>
       </c>
       <c r="F38" s="6" t="s">
-        <v>392</v>
+        <v>403</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="I38" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="L38" s="6" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="M38" s="6" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>399</v>
+        <v>410</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>37</v>
@@ -4827,46 +4861,46 @@
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="E39" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>403</v>
+      </c>
+      <c r="G39" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="J39" s="6" t="s">
+        <v>415</v>
+      </c>
+      <c r="K39" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="L39" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="M39" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="N39" s="6" t="s">
         <v>410</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>411</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H39" s="6" t="s">
-        <v>393</v>
-      </c>
-      <c r="I39" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="J39" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="K39" s="6" t="s">
-        <v>414</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>415</v>
-      </c>
-      <c r="M39" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="N39" s="6" t="s">
-        <v>399</v>
       </c>
       <c r="O39" s="6" t="s">
         <v>37</v>
@@ -4874,46 +4908,46 @@
     </row>
     <row r="40" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>80</v>
+        <v>420</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>392</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>52</v>
+        <v>422</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="L40" s="6" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="M40" s="6" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>399</v>
+        <v>410</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>37</v>
@@ -4921,46 +4955,46 @@
     </row>
     <row r="41" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>425</v>
+        <v>80</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>427</v>
-      </c>
-      <c r="G41" s="9" t="s">
-        <v>73</v>
+        <v>403</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>428</v>
+        <v>404</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="N41" s="6" t="s">
-        <v>434</v>
+        <v>410</v>
       </c>
       <c r="O41" s="6" t="s">
         <v>37</v>
@@ -4971,10 +5005,10 @@
         <v>435</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D42" s="6" t="s">
         <v>436</v>
@@ -5007,7 +5041,7 @@
         <v>444</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>434</v>
+        <v>445</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>37</v>
@@ -5015,46 +5049,46 @@
     </row>
     <row r="43" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>53</v>
+        <v>450</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>454</v>
+        <v>445</v>
       </c>
       <c r="O43" s="6" t="s">
         <v>37</v>
@@ -5062,46 +5096,46 @@
     </row>
     <row r="44" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G44" s="7" t="s">
-        <v>29</v>
+        <v>459</v>
+      </c>
+      <c r="G44" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="K44" s="6" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="L44" s="6" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="M44" s="6" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>454</v>
+        <v>465</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>37</v>
@@ -5109,46 +5143,46 @@
     </row>
     <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>463</v>
+        <v>457</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F45" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I45" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="K45" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="L45" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="M45" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="N45" s="6" t="s">
         <v>465</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>363</v>
-      </c>
-      <c r="I45" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="J45" s="6" t="s">
-        <v>467</v>
-      </c>
-      <c r="K45" s="6" t="s">
-        <v>468</v>
-      </c>
-      <c r="L45" s="6" t="s">
-        <v>469</v>
-      </c>
-      <c r="M45" s="6" t="s">
-        <v>470</v>
-      </c>
-      <c r="N45" s="6" t="s">
-        <v>434</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>37</v>
@@ -5156,46 +5190,46 @@
     </row>
     <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>475</v>
+        <v>374</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>481</v>
+        <v>445</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
@@ -5206,43 +5240,43 @@
         <v>482</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>338</v>
+        <v>483</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G47" s="8" t="s">
-        <v>52</v>
+        <v>485</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>149</v>
+        <v>486</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="M47" s="6" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
@@ -5250,22 +5284,22 @@
     </row>
     <row r="48" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>359</v>
+        <v>382</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>492</v>
+        <v>211</v>
       </c>
       <c r="G48" s="8" t="s">
         <v>52</v>
@@ -5274,22 +5308,22 @@
         <v>149</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>452</v>
+        <v>498</v>
       </c>
       <c r="M48" s="6" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
@@ -5297,46 +5331,46 @@
     </row>
     <row r="49" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>307</v>
+        <v>502</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>73</v>
+        <v>503</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>503</v>
+        <v>463</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
@@ -5344,28 +5378,28 @@
     </row>
     <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>507</v>
+        <v>306</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>508</v>
+        <v>307</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>509</v>
-      </c>
-      <c r="G50" s="8" t="s">
-        <v>52</v>
+        <v>510</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>510</v>
+        <v>309</v>
       </c>
       <c r="I50" s="6" t="s">
         <v>511</v>
@@ -5394,10 +5428,10 @@
         <v>517</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D51" s="6" t="s">
         <v>518</v>
@@ -5412,7 +5446,7 @@
         <v>52</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>393</v>
+        <v>361</v>
       </c>
       <c r="I51" s="6" t="s">
         <v>521</v>
@@ -5430,7 +5464,7 @@
         <v>525</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>516</v>
+        <v>526</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
@@ -5438,28 +5472,28 @@
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>529</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>29</v>
+        <v>530</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>530</v>
+        <v>404</v>
       </c>
       <c r="I52" s="6" t="s">
         <v>531</v>
@@ -5477,7 +5511,7 @@
         <v>535</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>536</v>
+        <v>526</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
@@ -5485,46 +5519,46 @@
     </row>
     <row r="53" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="D53" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="B53" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="D53" s="6" t="s">
+      <c r="E53" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="E53" s="6" t="s">
+      <c r="F53" s="6" t="s">
         <v>539</v>
-      </c>
-      <c r="F53" s="6" t="s">
-        <v>540</v>
       </c>
       <c r="G53" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H53" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="I53" s="6" t="s">
         <v>541</v>
       </c>
-      <c r="I53" s="6" t="s">
+      <c r="J53" s="6" t="s">
         <v>542</v>
       </c>
-      <c r="J53" s="6" t="s">
+      <c r="K53" s="6" t="s">
         <v>543</v>
       </c>
-      <c r="K53" s="6" t="s">
+      <c r="L53" s="6" t="s">
         <v>544</v>
       </c>
-      <c r="L53" s="6" t="s">
+      <c r="M53" s="6" t="s">
         <v>545</v>
       </c>
-      <c r="M53" s="6" t="s">
+      <c r="N53" s="6" t="s">
         <v>546</v>
-      </c>
-      <c r="N53" s="6" t="s">
-        <v>547</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
@@ -5532,46 +5566,46 @@
     </row>
     <row r="54" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
+        <v>547</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="D54" s="6" t="s">
         <v>548</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="D54" s="6" t="s">
+      <c r="E54" s="6" t="s">
         <v>549</v>
       </c>
-      <c r="E54" s="6" t="s">
+      <c r="F54" s="6" t="s">
         <v>550</v>
       </c>
-      <c r="F54" s="6" t="s">
+      <c r="G54" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H54" s="6" t="s">
         <v>551</v>
       </c>
-      <c r="G54" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H54" s="6" t="s">
+      <c r="I54" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="I54" s="6" t="s">
+      <c r="J54" s="6" t="s">
         <v>553</v>
       </c>
-      <c r="J54" s="6" t="s">
+      <c r="K54" s="6" t="s">
         <v>554</v>
       </c>
-      <c r="K54" s="6" t="s">
+      <c r="L54" s="6" t="s">
         <v>555</v>
       </c>
-      <c r="L54" s="6" t="s">
+      <c r="M54" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="M54" s="6" t="s">
+      <c r="N54" s="6" t="s">
         <v>557</v>
-      </c>
-      <c r="N54" s="6" t="s">
-        <v>558</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
@@ -5579,28 +5613,28 @@
     </row>
     <row r="55" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
+        <v>558</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>559</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>371</v>
-      </c>
-      <c r="D55" s="6" t="s">
+      <c r="E55" s="6" t="s">
         <v>560</v>
       </c>
-      <c r="E55" s="6" t="s">
+      <c r="F55" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="F55" s="6" t="s">
+      <c r="G55" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H55" s="6" t="s">
         <v>562</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>552</v>
       </c>
       <c r="I55" s="6" t="s">
         <v>563</v>
@@ -5618,7 +5652,7 @@
         <v>567</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>547</v>
+        <v>568</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
@@ -5626,46 +5660,46 @@
     </row>
     <row r="56" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>295</v>
+        <v>570</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>296</v>
+        <v>571</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>29</v>
+        <v>572</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>298</v>
+        <v>562</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>299</v>
+        <v>573</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>300</v>
+        <v>574</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>569</v>
+        <v>575</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>570</v>
+        <v>576</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>571</v>
+        <v>577</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>547</v>
+        <v>557</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
@@ -5673,46 +5707,46 @@
     </row>
     <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>572</v>
+        <v>578</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>573</v>
+        <v>295</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>574</v>
+        <v>296</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>575</v>
+        <v>297</v>
       </c>
       <c r="G57" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>552</v>
+        <v>298</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>576</v>
+        <v>299</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>577</v>
+        <v>300</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>581</v>
+        <v>557</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
@@ -5723,63 +5757,63 @@
         <v>582</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>507</v>
+        <v>583</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>508</v>
+        <v>584</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="G58" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>510</v>
+        <v>562</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>590</v>
+        <v>37</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>573</v>
+        <v>518</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>592</v>
+        <v>519</v>
       </c>
       <c r="F59" s="6" t="s">
         <v>593</v>
@@ -5788,7 +5822,7 @@
         <v>29</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>552</v>
+        <v>361</v>
       </c>
       <c r="I59" s="6" t="s">
         <v>594</v>
@@ -5809,21 +5843,21 @@
         <v>599</v>
       </c>
       <c r="O59" s="6" t="s">
-        <v>37</v>
+        <v>600</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>371</v>
+        <v>382</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>601</v>
+        <v>583</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>602</v>
@@ -5831,29 +5865,29 @@
       <c r="F60" s="6" t="s">
         <v>603</v>
       </c>
-      <c r="G60" s="8" t="s">
-        <v>52</v>
+      <c r="G60" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H60" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="I60" s="6" t="s">
         <v>604</v>
       </c>
-      <c r="I60" s="6" t="s">
+      <c r="J60" s="6" t="s">
         <v>605</v>
       </c>
-      <c r="J60" s="6" t="s">
+      <c r="K60" s="6" t="s">
         <v>606</v>
       </c>
-      <c r="K60" s="6" t="s">
+      <c r="L60" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="L60" s="6" t="s">
+      <c r="M60" s="6" t="s">
         <v>608</v>
       </c>
-      <c r="M60" s="6" t="s">
+      <c r="N60" s="6" t="s">
         <v>609</v>
-      </c>
-      <c r="N60" s="6" t="s">
-        <v>610</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
@@ -5861,28 +5895,28 @@
     </row>
     <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>382</v>
+      </c>
+      <c r="D61" s="6" t="s">
         <v>611</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>358</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D61" s="6" t="s">
+      <c r="E61" s="6" t="s">
         <v>612</v>
       </c>
-      <c r="E61" s="6" t="s">
+      <c r="F61" s="6" t="s">
         <v>613</v>
-      </c>
-      <c r="F61" s="6" t="s">
-        <v>614</v>
       </c>
       <c r="G61" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>255</v>
+        <v>614</v>
       </c>
       <c r="I61" s="6" t="s">
         <v>615</v>
@@ -5900,7 +5934,7 @@
         <v>619</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>610</v>
+        <v>620</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
@@ -5908,46 +5942,46 @@
     </row>
     <row r="62" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>623</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>73</v>
+        <v>624</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>268</v>
+        <v>626</v>
       </c>
       <c r="K62" s="6" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>271</v>
+        <v>629</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>610</v>
+        <v>620</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
@@ -5955,46 +5989,46 @@
     </row>
     <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>371</v>
+        <v>25</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>630</v>
-      </c>
-      <c r="G63" s="7" t="s">
-        <v>29</v>
+        <v>633</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>632</v>
+        <v>268</v>
       </c>
       <c r="K63" s="6" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="M63" s="6" t="s">
-        <v>635</v>
+        <v>271</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>610</v>
+        <v>620</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
@@ -6002,46 +6036,46 @@
     </row>
     <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>25</v>
+        <v>382</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>639</v>
-      </c>
-      <c r="G64" s="8" t="s">
-        <v>52</v>
+        <v>640</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="M64" s="6" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>645</v>
+        <v>620</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
@@ -6052,45 +6086,92 @@
         <v>646</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>358</v>
+        <v>369</v>
       </c>
       <c r="C65" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D65" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="G65" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I65" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="J65" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="K65" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="L65" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="M65" s="6" t="s">
+        <v>654</v>
+      </c>
+      <c r="N65" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="O65" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5" t="s">
+        <v>656</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D66" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E65" s="6" t="s">
-        <v>647</v>
-      </c>
-      <c r="F65" s="6" t="s">
-        <v>648</v>
-      </c>
-      <c r="G65" s="7" t="s">
+      <c r="E66" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="G66" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H65" s="6" t="s">
+      <c r="H66" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I65" s="6" t="s">
-        <v>649</v>
-      </c>
-      <c r="J65" s="6" t="s">
-        <v>650</v>
-      </c>
-      <c r="K65" s="6" t="s">
-        <v>651</v>
-      </c>
-      <c r="L65" s="6" t="s">
-        <v>652</v>
-      </c>
-      <c r="M65" s="6" t="s">
-        <v>653</v>
-      </c>
-      <c r="N65" s="6" t="s">
-        <v>645</v>
-      </c>
-      <c r="O65" s="6" t="s">
+      <c r="I66" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="N66" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6148,12 +6229,12 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>428</v>
+        <v>439</v>
       </c>
       <c r="B2" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A2,'Bug List'!$G:$G,"Cao")</f>
@@ -6195,7 +6276,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>393</v>
+        <v>404</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -6216,7 +6297,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>439</v>
+        <v>450</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -6237,7 +6318,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>530</v>
+        <v>540</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -6321,7 +6402,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>363</v>
+        <v>374</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -6384,7 +6465,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>604</v>
+        <v>614</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -6426,7 +6507,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>541</v>
+        <v>551</v>
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A15,'Bug List'!$G:$G,"Cao")</f>
@@ -6531,7 +6612,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>552</v>
+        <v>562</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Cao")</f>
@@ -6615,7 +6696,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>510</v>
+        <v>361</v>
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Cao")</f>
@@ -6623,7 +6704,7 @@
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Thấp")</f>
@@ -6631,7 +6712,7 @@
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">SUM(B24:D24)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6699,7 +6780,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>475</v>
+        <v>486</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Cao")</f>
@@ -6804,7 +6885,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>654</v>
+        <v>664</v>
       </c>
       <c r="B33" s="12" t="n">
         <f aca="false">SUM(B2:B32)</f>
@@ -6812,7 +6893,7 @@
       </c>
       <c r="C33" s="12" t="n">
         <f aca="false">SUM(C2:C32)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D33" s="12" t="n">
         <f aca="false">SUM(D2:D32)</f>
@@ -6820,7 +6901,7 @@
       </c>
       <c r="E33" s="12" t="n">
         <f aca="false">SUM(E2:E32)</f>
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6829,12 +6910,12 @@
         <v>22</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>655</v>
+        <v>665</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>656</v>
+        <v>666</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A36)</f>
@@ -6843,7 +6924,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>590</v>
+        <v>600</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A37)</f>
@@ -6856,12 +6937,12 @@
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A38)</f>
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>657</v>
+        <v>667</v>
       </c>
       <c r="B39" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A39)</f>
@@ -6871,7 +6952,7 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>658</v>
+        <v>668</v>
       </c>
     </row>
   </sheetData>
@@ -6899,146 +6980,146 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>659</v>
+        <v>669</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>660</v>
+        <v>670</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>661</v>
+        <v>671</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>662</v>
+        <v>672</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>663</v>
+      <c r="A4" s="14" t="s">
+        <v>673</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>664</v>
+        <v>674</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>665</v>
+        <v>675</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>666</v>
+      <c r="A6" s="14" t="s">
+        <v>676</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>667</v>
+        <v>677</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>668</v>
+      <c r="A7" s="14" t="s">
+        <v>678</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>670</v>
+      <c r="A8" s="14" t="s">
+        <v>680</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>671</v>
+        <v>681</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>672</v>
+      <c r="A9" s="14" t="s">
+        <v>682</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>673</v>
+        <v>683</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>674</v>
+      <c r="A10" s="14" t="s">
+        <v>684</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>675</v>
+        <v>685</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>676</v>
+      <c r="A11" s="14" t="s">
+        <v>686</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>677</v>
+        <v>687</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>678</v>
+      <c r="A12" s="14" t="s">
+        <v>688</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>679</v>
+        <v>689</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>680</v>
+      <c r="A13" s="14" t="s">
+        <v>690</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>681</v>
+        <v>691</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>682</v>
+      <c r="A14" s="14" t="s">
+        <v>692</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>683</v>
+        <v>693</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>684</v>
+      <c r="A15" s="14" t="s">
+        <v>694</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>685</v>
+        <v>695</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>686</v>
+      <c r="A16" s="14" t="s">
+        <v>696</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>687</v>
+        <v>697</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>688</v>
+        <v>698</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>689</v>
+      <c r="A18" s="14" t="s">
+        <v>699</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>690</v>
+        <v>700</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-34..PT-38 from the handover simulation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1078" uniqueCount="701">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="751">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1288,6 +1288,197 @@
     <t xml:space="preserve">5706299; cùng hướng sửa SAAS-25 (lotus-pos-saas 34b760d)</t>
   </si>
   <si>
+    <t xml:space="preserve">PT-34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worker / Hội viên, đơn QR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/worker.js (register, login, logout, getOrder, body()); src/staff.js (overview, deps.register/login); src/ops.js (inventory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mọi request lỗi định dạng tới đăng ký/đăng nhập hội viên (QR và máy cầm tay), đăng xuất, xem trạng thái đơn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Async</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gửi JSON hỏng tới /api/member/register, /api/member/login, /api/staff/members/register: Worker ném lỗi ra ngoài, Cloudflare trả trang lỗi 1101 dạng HTML thay vì JSON 400; body là null thì trả 503 "máy chủ gián đoạn".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trong khối try, hàm async được trả về trực tiếp (return register(env,request), ?overview(env,…)) mà không await, nên lỗi của promise không đi qua catch của try. body() chấp nhận JSON null/số rồi code đọc b.x gây TypeError → 503.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">await mọi lời gọi async được return trong try (register, login, logout, getOrder, overview ×13, inventory ×5, deps.register/login); body() từ chối JSON không phải object bằng BAD_JSON.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v179-sim-worker.test.mjs: "SIM robustness /api/…: broken JSON, wrong content type and a huge body get a 4xx JSON answer, never a crash" (7 endpoint, đỏ trên code cũ); tests/phattai-v179-ui.test.mjs: "PT-34 every async call returned from inside a try block is awaited…".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trong try/catch luôn return await; grep "return f(" và "?f(" của hàm async. Test robustness phải gửi body hỏng tới mọi endpoint POST và yêu cầu JSON 4xx.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">afef54d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web QR / Gửi đơn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/assets/app.js submit(), dock gửi đơn, thẻ demoBadge trong giỏ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Điện thoại khách mất Wi-Fi/4G lúc bấm gửi đơn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách mất mạng bấm "Xác nhận gọi món" thì thấy màn "DEMO · Không có đơn thật · Chỉ là bản xem thử"; nút gửi đổi thành "Xem trước (DEMO)". Khách tưởng quán chưa nhận đơn thật.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">isReady() gộp "mất mạng" với "quán chưa bật nhận đơn"; mọi trường hợp !isReady() đều đưa sang màn xem thử DEMO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">offlineNow() tách riêng: mất mạng hoặc không gọi được server thì báo "Mất kết nối…" và giữ giỏ, nút ghi "Mất kết nối – chưa gửi được", không hiện huy hiệu DEMO; DEMO chỉ còn khi server bảo chưa nhận đơn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs: "QR offline: sending is refused with a message and no order is made; back online it goes through" (đỏ trên code cũ); tests/phattai-v179-ui.test.mjs: "PT-35 …".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi trạng thái lỗi (mất mạng, server lỗi, quán đóng) phải có câu riêng; không gộp vào một nhánh "chưa sẵn sàng".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staff UI / Đăng nhập</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js renderLogin()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máy cầm tay/quầy dùng tài khoản nhân viên khác "huang"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thu ngân gõ tên đăng nhập và sai mật khẩu: thông báo lỗi hiện ra thì ô tên đăng nhập quay về "huang". Lần thử sau là đăng nhập tài khoản chủ tiệm với mật khẩu thu ngân, lại báo sai.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">renderLogin() dựng lại form bằng innerHTML với value="huang" mặc định mỗi khi có thông báo (message() → render()); không giữ giá trị đã gõ. Cùng loại PT-01/PT-32 nhưng màn đăng nhập dùng hàm render riêng nên không được bản sửa PT-32 che.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">renderLogin() giữ bản nháp form và ô đang gõ (keepDrafts/keepTyping) như render(); mật khẩu không lưu vào bản nháp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs: "Handheld: after a wrong password the cashier's user name stays filled in" (đỏ trên code cũ); tests/phattai-v179-ui.test.mjs: "PT-36 …".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mọi hàm vẽ màn hình (không chỉ render chính) phải giữ dữ liệu đang nhập. Giá trị mặc định trong ô nhập (value="huang") nguy hiểm khi form bị vẽ lại.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staff UI / Kết nối</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js connection(), vòng auto print</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máy cầm tay mất mạng rồi có mạng lại</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sau khi Wi-Fi có lại, máy vẫn hiện "Không kiểm tra được lệnh in bếp: Không kết nối được Worker: Failed to fetch" trên mọi màn hình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vòng kiểm tra in bếp ghi lỗi vào st.error (không hẹn giờ xóa); khi kết nối trở lại không ai xóa lỗi này nên render nào cũng vẽ lại.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">connection() nhận ra lúc chuyển từ mất mạng sang có mạng và xóa thông báo lỗi mạng còn treo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs: "Handheld: network loss shows offline, then recovers by itself" (kiểm không còn lỗi mạng sau khi có lại; đỏ trên code cũ); tests/phattai-v179-ui.test.mjs: "PT-37 …".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lỗi tạm thời (mạng) phải có điều kiện tự xóa; thông báo không hẹn giờ phải có người dọn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web QR / Tùy chọn món</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/assets/app.js modal()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trang QR, món một cỡ (canh, combo)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Bảng chọn tùy chọn của canh và combo vẫn có mục "Phần ăn: Tô thường / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">中碗</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" dù món không có cỡ.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">modal() luôn vẽ nhóm cỡ, với món không có cỡ thì vẫn vẽ một nút "Tô thường" (optsSize=['</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">中</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">']); nhóm cay thì đã có điều kiện p.spicy.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Chỉ vẽ nhóm cỡ khi p.size; Worker vốn đã không lưu cỡ cho món không có cỡ (PT-26).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs: "QR dish 113..119: the option sheet shows no bowl size…" (6 món đỏ trên code cũ); tests/phattai-v179-ui.test.mjs: "PT-38 the QR option sheet offers a bowl size only for dishes that have one".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mọi tùy chọn món trên mọi giao diện (QR, máy cầm tay, phiếu in) phải theo cùng cờ size/spicy của món.</t>
+  </si>
+  <si>
     <t xml:space="preserve">SAAS-01</t>
   </si>
   <si>
@@ -1499,9 +1690,6 @@
   </si>
   <si>
     <t xml:space="preserve">Quán chỉ có key chưa kích hoạt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Async</t>
   </si>
   <si>
     <t xml:space="preserve">Quán chỉ có license PENDING lại báo "chưa có license" (NONE).</t>
@@ -2444,6 +2632,18 @@
   </si>
   <si>
     <t xml:space="preserve">Lỗi sửa ở lotus-pos-saas đã đối chiếu với pos-phattai (và ngược lại) chưa? Ghi dòng PT-/SAAS- tương ứng.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Async trong try</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hàm async return trong try/catch có await không (return await f())? Body hỏng/null tới mọi endpoint POST có ra JSON 4xx không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mất mạng ≠ chưa mở</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Màn hình phân biệt mất mạng, server lỗi, quán chưa nhận đơn bằng câu riêng; lỗi mạng tự xóa khi có mạng lại?</t>
   </si>
 </sst>
 </file>
@@ -2789,8 +2989,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O66" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O66"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O71"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3053,7 +3253,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -4676,43 +4876,43 @@
         <v>368</v>
       </c>
       <c r="B35" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="E35" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="G35" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H35" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="I35" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="G35" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H35" s="6" t="s">
+      <c r="J35" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="I35" s="6" t="s">
+      <c r="K35" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="J35" s="6" t="s">
+      <c r="L35" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="K35" s="6" t="s">
+      <c r="M35" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="L35" s="6" t="s">
+      <c r="N35" s="6" t="s">
         <v>378</v>
-      </c>
-      <c r="M35" s="6" t="s">
-        <v>379</v>
-      </c>
-      <c r="N35" s="6" t="s">
-        <v>380</v>
       </c>
       <c r="O35" s="6" t="s">
         <v>37</v>
@@ -4720,46 +4920,46 @@
     </row>
     <row r="36" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C36" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>382</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>383</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>384</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>385</v>
       </c>
       <c r="G36" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>374</v>
+        <v>298</v>
       </c>
       <c r="I36" s="6" t="s">
+        <v>383</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>384</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="L36" s="6" t="s">
         <v>386</v>
       </c>
-      <c r="J36" s="6" t="s">
+      <c r="M36" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="K36" s="6" t="s">
-        <v>388</v>
-      </c>
-      <c r="L36" s="6" t="s">
-        <v>389</v>
-      </c>
-      <c r="M36" s="6" t="s">
-        <v>390</v>
-      </c>
       <c r="N36" s="6" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="O36" s="6" t="s">
         <v>37</v>
@@ -4767,46 +4967,46 @@
     </row>
     <row r="37" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
+        <v>388</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>389</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>390</v>
+      </c>
+      <c r="F37" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D37" s="6" t="s">
+      <c r="G37" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I37" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="J37" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="F37" s="6" t="s">
+      <c r="K37" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="G37" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H37" s="6" t="s">
-        <v>374</v>
-      </c>
-      <c r="I37" s="6" t="s">
+      <c r="L37" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="J37" s="6" t="s">
+      <c r="M37" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="K37" s="6" t="s">
-        <v>397</v>
-      </c>
-      <c r="L37" s="6" t="s">
-        <v>398</v>
-      </c>
-      <c r="M37" s="6" t="s">
-        <v>399</v>
-      </c>
       <c r="N37" s="6" t="s">
-        <v>400</v>
+        <v>378</v>
       </c>
       <c r="O37" s="6" t="s">
         <v>37</v>
@@ -4814,46 +5014,46 @@
     </row>
     <row r="38" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>399</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>400</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="I38" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="E38" s="6" t="s">
+      <c r="J38" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="F38" s="6" t="s">
+      <c r="K38" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="G38" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H38" s="6" t="s">
+      <c r="L38" s="6" t="s">
         <v>404</v>
       </c>
-      <c r="I38" s="6" t="s">
+      <c r="M38" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="J38" s="6" t="s">
-        <v>406</v>
-      </c>
-      <c r="K38" s="6" t="s">
-        <v>407</v>
-      </c>
-      <c r="L38" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="M38" s="6" t="s">
-        <v>409</v>
-      </c>
       <c r="N38" s="6" t="s">
-        <v>410</v>
+        <v>378</v>
       </c>
       <c r="O38" s="6" t="s">
         <v>37</v>
@@ -4861,46 +5061,46 @@
     </row>
     <row r="39" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="G39" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>298</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="J39" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D39" s="6" t="s">
+      <c r="K39" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="L39" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>403</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H39" s="6" t="s">
-        <v>404</v>
-      </c>
-      <c r="I39" s="6" t="s">
+      <c r="M39" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="J39" s="6" t="s">
-        <v>415</v>
-      </c>
-      <c r="K39" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="L39" s="6" t="s">
-        <v>417</v>
-      </c>
-      <c r="M39" s="6" t="s">
-        <v>418</v>
-      </c>
       <c r="N39" s="6" t="s">
-        <v>410</v>
+        <v>378</v>
       </c>
       <c r="O39" s="6" t="s">
         <v>37</v>
@@ -4908,46 +5108,46 @@
     </row>
     <row r="40" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>417</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="B40" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D40" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="G40" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="I40" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="G40" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>404</v>
-      </c>
-      <c r="I40" s="6" t="s">
+      <c r="J40" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="J40" s="6" t="s">
+      <c r="K40" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="K40" s="6" t="s">
+      <c r="L40" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="L40" s="6" t="s">
+      <c r="M40" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="M40" s="6" t="s">
+      <c r="N40" s="6" t="s">
         <v>427</v>
-      </c>
-      <c r="N40" s="6" t="s">
-        <v>410</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>37</v>
@@ -4958,43 +5158,43 @@
         <v>428</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>80</v>
+        <v>430</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>403</v>
-      </c>
-      <c r="G41" s="8" t="s">
-        <v>52</v>
+        <v>432</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H41" s="6" t="s">
-        <v>404</v>
+        <v>421</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="L41" s="6" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="M41" s="6" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="N41" s="6" t="s">
-        <v>410</v>
+        <v>427</v>
       </c>
       <c r="O41" s="6" t="s">
         <v>37</v>
@@ -5002,46 +5202,46 @@
     </row>
     <row r="42" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>438</v>
-      </c>
-      <c r="G42" s="9" t="s">
-        <v>73</v>
+        <v>441</v>
+      </c>
+      <c r="G42" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>439</v>
+        <v>421</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="L42" s="6" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="M42" s="6" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>37</v>
@@ -5049,46 +5249,46 @@
     </row>
     <row r="43" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>447</v>
+        <v>146</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>449</v>
-      </c>
-      <c r="G43" s="9" t="s">
-        <v>73</v>
+        <v>450</v>
+      </c>
+      <c r="G43" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="L43" s="6" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="M43" s="6" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="O43" s="6" t="s">
         <v>37</v>
@@ -5096,46 +5296,46 @@
     </row>
     <row r="44" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D44" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="G44" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="M44" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="N44" s="6" t="s">
         <v>457</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="G44" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="I44" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="J44" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="K44" s="6" t="s">
-        <v>462</v>
-      </c>
-      <c r="L44" s="6" t="s">
-        <v>463</v>
-      </c>
-      <c r="M44" s="6" t="s">
-        <v>464</v>
-      </c>
-      <c r="N44" s="6" t="s">
-        <v>465</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>37</v>
@@ -5146,43 +5346,43 @@
         <v>466</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>457</v>
+        <v>467</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>28</v>
+        <v>469</v>
       </c>
       <c r="G45" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>30</v>
+        <v>451</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>37</v>
@@ -5190,28 +5390,28 @@
     </row>
     <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>474</v>
+        <v>80</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>476</v>
-      </c>
-      <c r="G46" s="9" t="s">
-        <v>73</v>
+        <v>450</v>
+      </c>
+      <c r="G46" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>374</v>
+        <v>451</v>
       </c>
       <c r="I46" s="6" t="s">
         <v>477</v>
@@ -5229,7 +5429,7 @@
         <v>481</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>445</v>
+        <v>457</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
@@ -5240,10 +5440,10 @@
         <v>482</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D47" s="6" t="s">
         <v>483</v>
@@ -5258,25 +5458,25 @@
         <v>73</v>
       </c>
       <c r="H47" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="I47" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="J47" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="J47" s="6" t="s">
+      <c r="K47" s="6" t="s">
         <v>488</v>
       </c>
-      <c r="K47" s="6" t="s">
+      <c r="L47" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="L47" s="6" t="s">
+      <c r="M47" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="M47" s="6" t="s">
+      <c r="N47" s="6" t="s">
         <v>491</v>
-      </c>
-      <c r="N47" s="6" t="s">
-        <v>492</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
@@ -5284,46 +5484,46 @@
     </row>
     <row r="48" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>493</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>338</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>494</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>52</v>
+        <v>495</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>149</v>
+        <v>496</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="M48" s="6" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>500</v>
+        <v>491</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
@@ -5331,46 +5531,46 @@
     </row>
     <row r="49" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>370</v>
+        <v>429</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>146</v>
+        <v>503</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>503</v>
-      </c>
-      <c r="G49" s="8" t="s">
-        <v>52</v>
+        <v>505</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>149</v>
+        <v>53</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>463</v>
+        <v>509</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
@@ -5378,46 +5578,46 @@
     </row>
     <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>306</v>
+        <v>503</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>307</v>
+        <v>513</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>510</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>73</v>
+        <v>28</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>309</v>
+        <v>30</v>
       </c>
       <c r="I50" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="M50" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="N50" s="6" t="s">
         <v>511</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>512</v>
-      </c>
-      <c r="K50" s="6" t="s">
-        <v>513</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="M50" s="6" t="s">
-        <v>515</v>
-      </c>
-      <c r="N50" s="6" t="s">
-        <v>516</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
@@ -5425,46 +5625,46 @@
     </row>
     <row r="51" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="G51" s="8" t="s">
-        <v>52</v>
+        <v>522</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>361</v>
+        <v>421</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>526</v>
+        <v>491</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
@@ -5472,46 +5672,46 @@
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>530</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>52</v>
+        <v>531</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>404</v>
+        <v>532</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>526</v>
+        <v>538</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
@@ -5519,28 +5719,28 @@
     </row>
     <row r="53" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>537</v>
+        <v>338</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>539</v>
-      </c>
-      <c r="G53" s="7" t="s">
-        <v>29</v>
+        <v>211</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>540</v>
+        <v>149</v>
       </c>
       <c r="I53" s="6" t="s">
         <v>541</v>
@@ -5569,43 +5769,43 @@
         <v>547</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>382</v>
+        <v>417</v>
       </c>
       <c r="D54" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>548</v>
       </c>
-      <c r="E54" s="6" t="s">
+      <c r="F54" s="6" t="s">
         <v>549</v>
       </c>
-      <c r="F54" s="6" t="s">
+      <c r="G54" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="I54" s="6" t="s">
         <v>550</v>
       </c>
-      <c r="G54" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H54" s="6" t="s">
+      <c r="J54" s="6" t="s">
         <v>551</v>
       </c>
-      <c r="I54" s="6" t="s">
+      <c r="K54" s="6" t="s">
         <v>552</v>
       </c>
-      <c r="J54" s="6" t="s">
+      <c r="L54" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="M54" s="6" t="s">
         <v>553</v>
       </c>
-      <c r="K54" s="6" t="s">
+      <c r="N54" s="6" t="s">
         <v>554</v>
-      </c>
-      <c r="L54" s="6" t="s">
-        <v>555</v>
-      </c>
-      <c r="M54" s="6" t="s">
-        <v>556</v>
-      </c>
-      <c r="N54" s="6" t="s">
-        <v>557</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
@@ -5613,46 +5813,46 @@
     </row>
     <row r="55" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
+        <v>555</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="J55" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D55" s="6" t="s">
+      <c r="K55" s="6" t="s">
         <v>559</v>
       </c>
-      <c r="E55" s="6" t="s">
+      <c r="L55" s="6" t="s">
         <v>560</v>
       </c>
-      <c r="F55" s="6" t="s">
+      <c r="M55" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="G55" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H55" s="6" t="s">
+      <c r="N55" s="6" t="s">
         <v>562</v>
-      </c>
-      <c r="I55" s="6" t="s">
-        <v>563</v>
-      </c>
-      <c r="J55" s="6" t="s">
-        <v>564</v>
-      </c>
-      <c r="K55" s="6" t="s">
-        <v>565</v>
-      </c>
-      <c r="L55" s="6" t="s">
-        <v>566</v>
-      </c>
-      <c r="M55" s="6" t="s">
-        <v>567</v>
-      </c>
-      <c r="N55" s="6" t="s">
-        <v>568</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
@@ -5660,46 +5860,46 @@
     </row>
     <row r="56" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
+        <v>563</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="F56" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="J56" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="K56" s="6" t="s">
         <v>569</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D56" s="6" t="s">
+      <c r="L56" s="6" t="s">
         <v>570</v>
       </c>
-      <c r="E56" s="6" t="s">
+      <c r="M56" s="6" t="s">
         <v>571</v>
       </c>
-      <c r="F56" s="6" t="s">
+      <c r="N56" s="6" t="s">
         <v>572</v>
-      </c>
-      <c r="G56" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>562</v>
-      </c>
-      <c r="I56" s="6" t="s">
-        <v>573</v>
-      </c>
-      <c r="J56" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="K56" s="6" t="s">
-        <v>575</v>
-      </c>
-      <c r="L56" s="6" t="s">
-        <v>576</v>
-      </c>
-      <c r="M56" s="6" t="s">
-        <v>577</v>
-      </c>
-      <c r="N56" s="6" t="s">
-        <v>557</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
@@ -5707,34 +5907,34 @@
     </row>
     <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="F57" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="J57" s="6" t="s">
         <v>578</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>382</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="F57" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G57" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H57" s="6" t="s">
-        <v>298</v>
-      </c>
-      <c r="I57" s="6" t="s">
-        <v>299</v>
-      </c>
-      <c r="J57" s="6" t="s">
-        <v>300</v>
       </c>
       <c r="K57" s="6" t="s">
         <v>579</v>
@@ -5746,7 +5946,7 @@
         <v>581</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>557</v>
+        <v>572</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
@@ -5757,10 +5957,10 @@
         <v>582</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>583</v>
@@ -5775,25 +5975,25 @@
         <v>29</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>562</v>
+        <v>586</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
@@ -5801,93 +6001,93 @@
     </row>
     <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>518</v>
+        <v>594</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>519</v>
+        <v>595</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G59" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>361</v>
+        <v>597</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="M59" s="6" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="O59" s="6" t="s">
-        <v>600</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>583</v>
+        <v>605</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>603</v>
-      </c>
-      <c r="G60" s="7" t="s">
-        <v>29</v>
+        <v>607</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>562</v>
+        <v>608</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>609</v>
+        <v>614</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
@@ -5895,46 +6095,46 @@
     </row>
     <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>610</v>
+        <v>615</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>612</v>
+        <v>617</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>613</v>
-      </c>
-      <c r="G61" s="8" t="s">
-        <v>52</v>
+        <v>618</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>614</v>
+        <v>608</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="K61" s="6" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>620</v>
+        <v>603</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
@@ -5942,46 +6142,46 @@
     </row>
     <row r="62" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>25</v>
+        <v>429</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>622</v>
+        <v>295</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>623</v>
+        <v>296</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>624</v>
-      </c>
-      <c r="G62" s="8" t="s">
-        <v>52</v>
+        <v>297</v>
+      </c>
+      <c r="G62" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>255</v>
+        <v>298</v>
       </c>
       <c r="I62" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="J62" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="K62" s="6" t="s">
         <v>625</v>
       </c>
-      <c r="J62" s="6" t="s">
+      <c r="L62" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="K62" s="6" t="s">
+      <c r="M62" s="6" t="s">
         <v>627</v>
       </c>
-      <c r="L62" s="6" t="s">
-        <v>628</v>
-      </c>
-      <c r="M62" s="6" t="s">
-        <v>629</v>
-      </c>
       <c r="N62" s="6" t="s">
-        <v>620</v>
+        <v>603</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
@@ -5989,46 +6189,46 @@
     </row>
     <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
+        <v>628</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="E63" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>369</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D63" s="6" t="s">
+      <c r="F63" s="6" t="s">
         <v>631</v>
       </c>
-      <c r="E63" s="6" t="s">
+      <c r="G63" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H63" s="6" t="s">
+        <v>608</v>
+      </c>
+      <c r="I63" s="6" t="s">
         <v>632</v>
       </c>
-      <c r="F63" s="6" t="s">
+      <c r="J63" s="6" t="s">
         <v>633</v>
       </c>
-      <c r="G63" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H63" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="I63" s="6" t="s">
+      <c r="K63" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="J63" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="K63" s="6" t="s">
+      <c r="L63" s="6" t="s">
         <v>635</v>
       </c>
-      <c r="L63" s="6" t="s">
+      <c r="M63" s="6" t="s">
         <v>636</v>
       </c>
-      <c r="M63" s="6" t="s">
-        <v>271</v>
-      </c>
       <c r="N63" s="6" t="s">
-        <v>620</v>
+        <v>637</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
@@ -6036,63 +6236,63 @@
     </row>
     <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>382</v>
+        <v>429</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>638</v>
+        <v>564</v>
       </c>
       <c r="E64" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="F64" s="6" t="s">
         <v>639</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>640</v>
       </c>
       <c r="G64" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>276</v>
+        <v>361</v>
       </c>
       <c r="I64" s="6" t="s">
+        <v>640</v>
+      </c>
+      <c r="J64" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="J64" s="6" t="s">
+      <c r="K64" s="6" t="s">
         <v>642</v>
       </c>
-      <c r="K64" s="6" t="s">
+      <c r="L64" s="6" t="s">
         <v>643</v>
       </c>
-      <c r="L64" s="6" t="s">
+      <c r="M64" s="6" t="s">
         <v>644</v>
       </c>
-      <c r="M64" s="6" t="s">
+      <c r="N64" s="6" t="s">
         <v>645</v>
       </c>
-      <c r="N64" s="6" t="s">
-        <v>620</v>
-      </c>
       <c r="O64" s="6" t="s">
-        <v>37</v>
+        <v>646</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>25</v>
+        <v>429</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>647</v>
+        <v>629</v>
       </c>
       <c r="E65" s="6" t="s">
         <v>648</v>
@@ -6100,11 +6300,11 @@
       <c r="F65" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="G65" s="8" t="s">
-        <v>52</v>
+      <c r="G65" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>330</v>
+        <v>608</v>
       </c>
       <c r="I65" s="6" t="s">
         <v>650</v>
@@ -6128,50 +6328,285 @@
         <v>37</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
         <v>656</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>369</v>
+        <v>416</v>
       </c>
       <c r="C66" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="F66" s="6" t="s">
+        <v>659</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>661</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="N66" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="O66" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="s">
+        <v>667</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C67" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D66" s="6" t="s">
+      <c r="D67" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="F67" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I67" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="J67" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="K67" s="6" t="s">
+        <v>673</v>
+      </c>
+      <c r="L67" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="M67" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="N67" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="O67" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="5" t="s">
+        <v>676</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="J68" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>681</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="N68" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="O68" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>684</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="M69" s="6" t="s">
+        <v>691</v>
+      </c>
+      <c r="N69" s="6" t="s">
+        <v>666</v>
+      </c>
+      <c r="O69" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I70" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="J70" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="K70" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="L70" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="M70" s="6" t="s">
+        <v>700</v>
+      </c>
+      <c r="N70" s="6" t="s">
+        <v>701</v>
+      </c>
+      <c r="O70" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>416</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D71" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E66" s="6" t="s">
-        <v>657</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>658</v>
-      </c>
-      <c r="G66" s="7" t="s">
+      <c r="E71" s="6" t="s">
+        <v>703</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>704</v>
+      </c>
+      <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H66" s="6" t="s">
+      <c r="H71" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I66" s="6" t="s">
-        <v>659</v>
-      </c>
-      <c r="J66" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="K66" s="6" t="s">
-        <v>661</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>662</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>663</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>655</v>
-      </c>
-      <c r="O66" s="6" t="s">
+      <c r="I71" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>707</v>
+      </c>
+      <c r="L71" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="M71" s="6" t="s">
+        <v>709</v>
+      </c>
+      <c r="N71" s="6" t="s">
+        <v>701</v>
+      </c>
+      <c r="O71" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6229,12 +6664,12 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>664</v>
+        <v>710</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>439</v>
+        <v>372</v>
       </c>
       <c r="B2" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A2,'Bug List'!$G:$G,"Cao")</f>
@@ -6242,7 +6677,7 @@
       </c>
       <c r="C2" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A2,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A2,'Bug List'!$G:$G,"Thấp")</f>
@@ -6250,7 +6685,7 @@
       </c>
       <c r="E2" s="12" t="n">
         <f aca="false">SUM(B2:D2)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6276,7 +6711,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>404</v>
+        <v>451</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -6297,7 +6732,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>450</v>
+        <v>496</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -6318,7 +6753,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>540</v>
+        <v>586</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -6402,7 +6837,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>374</v>
+        <v>421</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -6431,15 +6866,15 @@
       </c>
       <c r="C11" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A11,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A11,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="12" t="n">
         <f aca="false">SUM(B11:D11)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6465,7 +6900,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>614</v>
+        <v>660</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -6507,7 +6942,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>551</v>
+        <v>597</v>
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A15,'Bug List'!$G:$G,"Cao")</f>
@@ -6612,7 +7047,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>562</v>
+        <v>608</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Cao")</f>
@@ -6746,7 +7181,7 @@
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Trung")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Thấp")</f>
@@ -6754,7 +7189,7 @@
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">SUM(B26:D26)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6780,7 +7215,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>486</v>
+        <v>532</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Cao")</f>
@@ -6885,7 +7320,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>664</v>
+        <v>710</v>
       </c>
       <c r="B33" s="12" t="n">
         <f aca="false">SUM(B2:B32)</f>
@@ -6893,15 +7328,15 @@
       </c>
       <c r="C33" s="12" t="n">
         <f aca="false">SUM(C2:C32)</f>
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D33" s="12" t="n">
         <f aca="false">SUM(D2:D32)</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E33" s="12" t="n">
         <f aca="false">SUM(E2:E32)</f>
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -6910,12 +7345,12 @@
         <v>22</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>665</v>
+        <v>711</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>666</v>
+        <v>712</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A36)</f>
@@ -6924,7 +7359,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>600</v>
+        <v>646</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A37)</f>
@@ -6937,12 +7372,12 @@
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A38)</f>
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>667</v>
+        <v>713</v>
       </c>
       <c r="B39" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A39)</f>
@@ -6952,7 +7387,7 @@
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>668</v>
+        <v>714</v>
       </c>
     </row>
   </sheetData>
@@ -6971,7 +7406,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
@@ -6980,10 +7415,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>669</v>
+        <v>715</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>670</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6991,7 +7426,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>671</v>
+        <v>717</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6999,15 +7434,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>672</v>
+        <v>718</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>673</v>
+        <v>719</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>674</v>
+        <v>720</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7015,95 +7450,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>675</v>
+        <v>721</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>676</v>
+        <v>722</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>677</v>
+        <v>723</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>678</v>
+        <v>724</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>679</v>
+        <v>725</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>680</v>
+        <v>726</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>681</v>
+        <v>727</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>682</v>
+        <v>728</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>683</v>
+        <v>729</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>684</v>
+        <v>730</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>685</v>
+        <v>731</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>686</v>
+        <v>732</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>687</v>
+        <v>733</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>688</v>
+        <v>734</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>689</v>
+        <v>735</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>690</v>
+        <v>736</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>691</v>
+        <v>737</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>692</v>
+        <v>738</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>693</v>
+        <v>739</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>694</v>
+        <v>740</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>695</v>
+        <v>741</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>696</v>
+        <v>742</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>697</v>
+        <v>743</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7111,15 +7546,31 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>698</v>
+        <v>744</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>699</v>
+        <v>745</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>700</v>
+        <v>746</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>747</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="14" t="s">
+        <v>749</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>750</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-39 (+86 mobiles), PT-40 (kitchen account sees dishes only)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1157" uniqueCount="751">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="771">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1479,6 +1479,63 @@
     <t xml:space="preserve">Mọi tùy chọn món trên mọi giao diện (QR, máy cầm tay, phiếu in) phải theo cùng cờ size/spicy của món.</t>
   </si>
   <si>
+    <t xml:space="preserve">PT-39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/worker.js phone(); public/assets/app.js, public/staff/staff.js memberPhone(); public/staff/scanner.js; câu báo lỗi SĐT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách dùng số di động Trung Quốc đại lục (+86)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khách có số +86 138 xxxx xxxx không đăng ký được hội viên (báo thông tin hội viên không hợp lệ). Phát hiện bằng bộ giả lập 05/10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quy tắc số quốc tế đặt ở 12–13 ký tự (\+[1-9]\d{10,11}); số di động +86 có 11 chữ số nên dài 14 ký tự.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm quyết định 05/10: số có mã nước dài 12–14 ký tự (\+[1-9]\d{10,12}); sửa đồng thời Worker, hai bản client, máy quét và mọi câu báo lỗi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v180-kitchen-view.test.mjs: "PT-39 a mainland China mobile (+86, 11 digits, 14 characters) can register"; tests/phattai-v177-members-cpu-phone.test.mjs (bảng CASES có +86 hợp lệ, 15 ký tự bị từ chối; client = Worker); tests/phattai-v179-sim-worker.test.mjs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi đặt giới hạn độ dài, thử với số thật của nhóm khách chính (VN, Đài Loan, Trung Quốc đại lục); chuẩn E.164 cho tới 15 chữ số.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b07efa6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worker + Staff UI / Quyền tài khoản bếp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/ops.js kitchenOnly/kitchenOrder; src/staff.js (danh sách đơn, chi tiết đơn, paid-labels, summary, tra hội viên, service-requests); src/customers.js; public/staff/staff.js (nav, kitchenDetail, itemsHtml)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tài khoản vai trò KITCHEN trên máy cầm tay/quầy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phân quyền dữ liệu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tài khoản bếp xem được danh sách khách hàng (SĐT, tổng chi tiêu, điểm), giá từng món, tổng tiền, cách thanh toán và tra cứu hội viên.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mọi API đọc đơn và khách chỉ kiểm quyền ORDER_VIEW (bếp có quyền này để in phiếu) rồi trả nguyên dữ liệu; giao diện cũng chỉ dựa vào ORDER_VIEW.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm quyết định 05/10: bếp chỉ thấy tên khách, mã đơn, món đã gọi (giữ bàn để giao món). Worker lọc dữ liệu cho tài khoản không có PAYMENT_CONFIRM và ORDER_EDIT: đơn chỉ còn mã, bàn, tên khách, ghi chú, món không giá; ẩn đơn đã trả; chặn 403 danh sách/chi tiết khách, tra hội viên, tổng quan ngày. Giao diện ẩn Khách hàng, Dashboard, QR Order và hiện màn chi tiết chỉ có món.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v180-kitchen-view.test.mjs: 6 test PT-40 (không trường tiền/thanh toán nào trong phản hồi, 403 khách hàng/hội viên/tổng quan, thu ngân vẫn thấy giá); scripts/sim-browser.mjs: "Handheld kitchen: …" (mọi màn của tài khoản bếp không có số tiền, mở đơn chỉ thấy món).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phân quyền phải lọc ở server, không chỉ ẩn trên giao diện. Mỗi vai trò mới: liệt kê trường dữ liệu nó được thấy và có test quét phản hồi không lộ trường khác.</t>
+  </si>
+  <si>
     <t xml:space="preserve">SAAS-01</t>
   </si>
   <si>
@@ -2644,6 +2701,9 @@
   </si>
   <si>
     <t xml:space="preserve">Màn hình phân biệt mất mạng, server lỗi, quán chưa nhận đơn bằng câu riêng; lỗi mạng tự xóa khi có mạng lại?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi vai trò được thấy trường nào? Server có lọc (không chỉ giao diện ẩn) và có test quét phản hồi không lộ tiền, SĐT, khách hàng không?</t>
   </si>
 </sst>
 </file>
@@ -2989,8 +3049,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O71" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O71"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O73"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3253,7 +3313,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O73"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -5111,43 +5171,43 @@
         <v>415</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E40" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="C40" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="G40" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="I40" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="J40" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="K40" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="G40" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H40" s="6" t="s">
+      <c r="L40" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="I40" s="6" t="s">
+      <c r="M40" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="J40" s="6" t="s">
+      <c r="N40" s="6" t="s">
         <v>423</v>
-      </c>
-      <c r="K40" s="6" t="s">
-        <v>424</v>
-      </c>
-      <c r="L40" s="6" t="s">
-        <v>425</v>
-      </c>
-      <c r="M40" s="6" t="s">
-        <v>426</v>
-      </c>
-      <c r="N40" s="6" t="s">
-        <v>427</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>37</v>
@@ -5155,46 +5215,46 @@
     </row>
     <row r="41" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>426</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H41" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="B41" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C41" s="6" t="s">
+      <c r="I41" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="J41" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="E41" s="6" t="s">
+      <c r="K41" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="L41" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="G41" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H41" s="6" t="s">
-        <v>421</v>
-      </c>
-      <c r="I41" s="6" t="s">
+      <c r="M41" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="J41" s="6" t="s">
-        <v>434</v>
-      </c>
-      <c r="K41" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="L41" s="6" t="s">
-        <v>436</v>
-      </c>
-      <c r="M41" s="6" t="s">
-        <v>437</v>
-      </c>
       <c r="N41" s="6" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
       <c r="O41" s="6" t="s">
         <v>37</v>
@@ -5202,46 +5262,46 @@
     </row>
     <row r="42" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
+        <v>434</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>436</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>437</v>
+      </c>
+      <c r="E42" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="B42" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D42" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>439</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>441</v>
       </c>
       <c r="G42" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>421</v>
+        <v>440</v>
       </c>
       <c r="I42" s="6" t="s">
+        <v>441</v>
+      </c>
+      <c r="J42" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="J42" s="6" t="s">
+      <c r="K42" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="K42" s="6" t="s">
+      <c r="L42" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="L42" s="6" t="s">
+      <c r="M42" s="6" t="s">
         <v>445</v>
       </c>
-      <c r="M42" s="6" t="s">
+      <c r="N42" s="6" t="s">
         <v>446</v>
-      </c>
-      <c r="N42" s="6" t="s">
-        <v>447</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>37</v>
@@ -5249,28 +5309,28 @@
     </row>
     <row r="43" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>429</v>
-      </c>
       <c r="D43" s="6" t="s">
-        <v>146</v>
+        <v>449</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>450</v>
-      </c>
-      <c r="G43" s="8" t="s">
-        <v>52</v>
+        <v>451</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H43" s="6" t="s">
-        <v>451</v>
+        <v>440</v>
       </c>
       <c r="I43" s="6" t="s">
         <v>452</v>
@@ -5288,7 +5348,7 @@
         <v>456</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>457</v>
+        <v>446</v>
       </c>
       <c r="O43" s="6" t="s">
         <v>37</v>
@@ -5296,28 +5356,28 @@
     </row>
     <row r="44" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D44" s="6" t="s">
+      <c r="E44" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="F44" s="6" t="s">
         <v>460</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>450</v>
       </c>
       <c r="G44" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>451</v>
+        <v>440</v>
       </c>
       <c r="I44" s="6" t="s">
         <v>461</v>
@@ -5335,7 +5395,7 @@
         <v>465</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>37</v>
@@ -5343,16 +5403,16 @@
     </row>
     <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>467</v>
+        <v>146</v>
       </c>
       <c r="E45" s="6" t="s">
         <v>468</v>
@@ -5360,29 +5420,29 @@
       <c r="F45" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="G45" s="7" t="s">
-        <v>29</v>
+      <c r="G45" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>457</v>
+        <v>476</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>37</v>
@@ -5390,46 +5450,46 @@
     </row>
     <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>80</v>
+        <v>478</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="G46" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>457</v>
+        <v>476</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
@@ -5437,46 +5497,46 @@
     </row>
     <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="G47" s="9" t="s">
-        <v>73</v>
+        <v>488</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>372</v>
+        <v>470</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="M47" s="6" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>491</v>
+        <v>476</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
@@ -5484,46 +5544,46 @@
     </row>
     <row r="48" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>493</v>
+        <v>80</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>495</v>
-      </c>
-      <c r="G48" s="9" t="s">
-        <v>73</v>
+        <v>469</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H48" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="I48" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="I48" s="6" t="s">
+      <c r="J48" s="6" t="s">
         <v>497</v>
       </c>
-      <c r="J48" s="6" t="s">
+      <c r="K48" s="6" t="s">
         <v>498</v>
       </c>
-      <c r="K48" s="6" t="s">
+      <c r="L48" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="L48" s="6" t="s">
+      <c r="M48" s="6" t="s">
         <v>500</v>
       </c>
-      <c r="M48" s="6" t="s">
-        <v>501</v>
-      </c>
       <c r="N48" s="6" t="s">
-        <v>491</v>
+        <v>476</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
@@ -5531,46 +5591,46 @@
     </row>
     <row r="49" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
+        <v>501</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D49" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="B49" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D49" s="6" t="s">
+      <c r="E49" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="F49" s="6" t="s">
         <v>504</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>505</v>
       </c>
       <c r="G49" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>53</v>
+        <v>372</v>
       </c>
       <c r="I49" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="J49" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="J49" s="6" t="s">
+      <c r="K49" s="6" t="s">
         <v>507</v>
       </c>
-      <c r="K49" s="6" t="s">
+      <c r="L49" s="6" t="s">
         <v>508</v>
       </c>
-      <c r="L49" s="6" t="s">
+      <c r="M49" s="6" t="s">
         <v>509</v>
       </c>
-      <c r="M49" s="6" t="s">
+      <c r="N49" s="6" t="s">
         <v>510</v>
-      </c>
-      <c r="N49" s="6" t="s">
-        <v>511</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
@@ -5578,46 +5638,46 @@
     </row>
     <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>512</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>503</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>513</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>29</v>
+        <v>514</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>30</v>
+        <v>515</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
@@ -5625,46 +5685,46 @@
     </row>
     <row r="51" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>421</v>
+        <v>53</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>491</v>
+        <v>530</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
@@ -5672,28 +5732,28 @@
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>531</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>73</v>
+        <v>28</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>532</v>
+        <v>30</v>
       </c>
       <c r="I52" s="6" t="s">
         <v>533</v>
@@ -5711,7 +5771,7 @@
         <v>537</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>538</v>
+        <v>530</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
@@ -5719,46 +5779,46 @@
     </row>
     <row r="53" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
+        <v>538</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D53" s="6" t="s">
         <v>539</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>338</v>
       </c>
       <c r="E53" s="6" t="s">
         <v>540</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G53" s="8" t="s">
-        <v>52</v>
+        <v>541</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>149</v>
+        <v>440</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="M53" s="6" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>546</v>
+        <v>510</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
@@ -5769,43 +5829,43 @@
         <v>547</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>417</v>
+        <v>448</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>146</v>
+        <v>548</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>549</v>
-      </c>
-      <c r="G54" s="8" t="s">
-        <v>52</v>
+        <v>550</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>149</v>
+        <v>551</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>509</v>
+        <v>555</v>
       </c>
       <c r="M54" s="6" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
@@ -5813,46 +5873,46 @@
     </row>
     <row r="55" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>306</v>
+        <v>338</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>307</v>
+        <v>559</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>556</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>73</v>
+        <v>211</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
@@ -5860,46 +5920,46 @@
     </row>
     <row r="56" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>564</v>
+        <v>146</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>361</v>
+        <v>149</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>570</v>
+        <v>528</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
@@ -5907,46 +5967,46 @@
     </row>
     <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>574</v>
+        <v>306</v>
       </c>
       <c r="E57" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F57" s="6" t="s">
         <v>575</v>
       </c>
-      <c r="F57" s="6" t="s">
+      <c r="G57" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="I57" s="6" t="s">
         <v>576</v>
       </c>
-      <c r="G57" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H57" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="I57" s="6" t="s">
+      <c r="J57" s="6" t="s">
         <v>577</v>
       </c>
-      <c r="J57" s="6" t="s">
+      <c r="K57" s="6" t="s">
         <v>578</v>
       </c>
-      <c r="K57" s="6" t="s">
+      <c r="L57" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="L57" s="6" t="s">
+      <c r="M57" s="6" t="s">
         <v>580</v>
       </c>
-      <c r="M57" s="6" t="s">
+      <c r="N57" s="6" t="s">
         <v>581</v>
-      </c>
-      <c r="N57" s="6" t="s">
-        <v>572</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
@@ -5957,10 +6017,10 @@
         <v>582</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D58" s="6" t="s">
         <v>583</v>
@@ -5971,29 +6031,29 @@
       <c r="F58" s="6" t="s">
         <v>585</v>
       </c>
-      <c r="G58" s="7" t="s">
-        <v>29</v>
+      <c r="G58" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H58" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="I58" s="6" t="s">
         <v>586</v>
       </c>
-      <c r="I58" s="6" t="s">
+      <c r="J58" s="6" t="s">
         <v>587</v>
       </c>
-      <c r="J58" s="6" t="s">
+      <c r="K58" s="6" t="s">
         <v>588</v>
       </c>
-      <c r="K58" s="6" t="s">
+      <c r="L58" s="6" t="s">
         <v>589</v>
       </c>
-      <c r="L58" s="6" t="s">
+      <c r="M58" s="6" t="s">
         <v>590</v>
       </c>
-      <c r="M58" s="6" t="s">
+      <c r="N58" s="6" t="s">
         <v>591</v>
-      </c>
-      <c r="N58" s="6" t="s">
-        <v>592</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
@@ -6001,46 +6061,46 @@
     </row>
     <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
+        <v>592</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D59" s="6" t="s">
+      <c r="E59" s="6" t="s">
         <v>594</v>
       </c>
-      <c r="E59" s="6" t="s">
+      <c r="F59" s="6" t="s">
         <v>595</v>
       </c>
-      <c r="F59" s="6" t="s">
+      <c r="G59" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>596</v>
       </c>
-      <c r="G59" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H59" s="6" t="s">
+      <c r="J59" s="6" t="s">
         <v>597</v>
       </c>
-      <c r="I59" s="6" t="s">
+      <c r="K59" s="6" t="s">
         <v>598</v>
       </c>
-      <c r="J59" s="6" t="s">
+      <c r="L59" s="6" t="s">
         <v>599</v>
       </c>
-      <c r="K59" s="6" t="s">
+      <c r="M59" s="6" t="s">
         <v>600</v>
       </c>
-      <c r="L59" s="6" t="s">
-        <v>601</v>
-      </c>
-      <c r="M59" s="6" t="s">
-        <v>602</v>
-      </c>
       <c r="N59" s="6" t="s">
-        <v>603</v>
+        <v>591</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
@@ -6048,46 +6108,46 @@
     </row>
     <row r="60" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
+        <v>601</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>602</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="F60" s="6" t="s">
         <v>604</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D60" s="6" t="s">
+      <c r="G60" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H60" s="6" t="s">
         <v>605</v>
       </c>
-      <c r="E60" s="6" t="s">
+      <c r="I60" s="6" t="s">
         <v>606</v>
       </c>
-      <c r="F60" s="6" t="s">
+      <c r="J60" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="G60" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H60" s="6" t="s">
+      <c r="K60" s="6" t="s">
         <v>608</v>
       </c>
-      <c r="I60" s="6" t="s">
+      <c r="L60" s="6" t="s">
         <v>609</v>
       </c>
-      <c r="J60" s="6" t="s">
+      <c r="M60" s="6" t="s">
         <v>610</v>
       </c>
-      <c r="K60" s="6" t="s">
+      <c r="N60" s="6" t="s">
         <v>611</v>
-      </c>
-      <c r="L60" s="6" t="s">
-        <v>612</v>
-      </c>
-      <c r="M60" s="6" t="s">
-        <v>613</v>
-      </c>
-      <c r="N60" s="6" t="s">
-        <v>614</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
@@ -6095,46 +6155,46 @@
     </row>
     <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
+        <v>612</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="F61" s="6" t="s">
         <v>615</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D61" s="6" t="s">
+      <c r="G61" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H61" s="6" t="s">
         <v>616</v>
       </c>
-      <c r="E61" s="6" t="s">
+      <c r="I61" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="F61" s="6" t="s">
+      <c r="J61" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="G61" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H61" s="6" t="s">
-        <v>608</v>
-      </c>
-      <c r="I61" s="6" t="s">
+      <c r="K61" s="6" t="s">
         <v>619</v>
       </c>
-      <c r="J61" s="6" t="s">
+      <c r="L61" s="6" t="s">
         <v>620</v>
       </c>
-      <c r="K61" s="6" t="s">
+      <c r="M61" s="6" t="s">
         <v>621</v>
       </c>
-      <c r="L61" s="6" t="s">
+      <c r="N61" s="6" t="s">
         <v>622</v>
-      </c>
-      <c r="M61" s="6" t="s">
-        <v>623</v>
-      </c>
-      <c r="N61" s="6" t="s">
-        <v>603</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
@@ -6142,46 +6202,46 @@
     </row>
     <row r="62" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
+        <v>623</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D62" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>429</v>
-      </c>
-      <c r="D62" s="6" t="s">
-        <v>295</v>
-      </c>
       <c r="E62" s="6" t="s">
-        <v>296</v>
+        <v>625</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G62" s="7" t="s">
-        <v>29</v>
+        <v>626</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>298</v>
+        <v>627</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>299</v>
+        <v>628</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>300</v>
+        <v>629</v>
       </c>
       <c r="K62" s="6" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>603</v>
+        <v>633</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
@@ -6189,46 +6249,46 @@
     </row>
     <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>628</v>
+        <v>634</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>629</v>
+        <v>635</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>630</v>
+        <v>636</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>631</v>
-      </c>
-      <c r="G63" s="7" t="s">
-        <v>29</v>
+        <v>637</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>632</v>
+        <v>638</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>633</v>
+        <v>639</v>
       </c>
       <c r="K63" s="6" t="s">
-        <v>634</v>
+        <v>640</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>635</v>
+        <v>641</v>
       </c>
       <c r="M63" s="6" t="s">
-        <v>636</v>
+        <v>642</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>637</v>
+        <v>622</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
@@ -6236,49 +6296,49 @@
     </row>
     <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>564</v>
+        <v>295</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>565</v>
+        <v>296</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>639</v>
+        <v>297</v>
       </c>
       <c r="G64" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>361</v>
+        <v>298</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>640</v>
+        <v>299</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>641</v>
+        <v>300</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="M64" s="6" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>645</v>
+        <v>622</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>646</v>
+        <v>37</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6286,43 +6346,43 @@
         <v>647</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>629</v>
+        <v>648</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
@@ -6330,283 +6390,377 @@
     </row>
     <row r="66" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>657</v>
+        <v>583</v>
       </c>
       <c r="E66" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="F66" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="F66" s="6" t="s">
+      <c r="G66" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="I66" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="G66" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H66" s="6" t="s">
+      <c r="J66" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="I66" s="6" t="s">
+      <c r="K66" s="6" t="s">
         <v>661</v>
       </c>
-      <c r="J66" s="6" t="s">
+      <c r="L66" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="K66" s="6" t="s">
+      <c r="M66" s="6" t="s">
         <v>663</v>
       </c>
-      <c r="L66" s="6" t="s">
+      <c r="N66" s="6" t="s">
         <v>664</v>
       </c>
-      <c r="M66" s="6" t="s">
+      <c r="O66" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="N66" s="6" t="s">
+    </row>
+    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="s">
         <v>666</v>
       </c>
-      <c r="O66" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="5" t="s">
+      <c r="B67" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>667</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D67" s="6" t="s">
+      <c r="F67" s="6" t="s">
         <v>668</v>
       </c>
-      <c r="E67" s="6" t="s">
+      <c r="G67" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="I67" s="6" t="s">
         <v>669</v>
       </c>
-      <c r="F67" s="6" t="s">
+      <c r="J67" s="6" t="s">
         <v>670</v>
       </c>
-      <c r="G67" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H67" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="I67" s="6" t="s">
+      <c r="K67" s="6" t="s">
         <v>671</v>
       </c>
-      <c r="J67" s="6" t="s">
+      <c r="L67" s="6" t="s">
         <v>672</v>
       </c>
-      <c r="K67" s="6" t="s">
+      <c r="M67" s="6" t="s">
         <v>673</v>
       </c>
-      <c r="L67" s="6" t="s">
+      <c r="N67" s="6" t="s">
         <v>674</v>
-      </c>
-      <c r="M67" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="N67" s="6" t="s">
-        <v>666</v>
       </c>
       <c r="O67" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
+        <v>675</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>448</v>
+      </c>
+      <c r="D68" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>416</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D68" s="6" t="s">
+      <c r="E68" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="F68" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="F68" s="6" t="s">
+      <c r="G68" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>679</v>
-      </c>
-      <c r="G68" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>266</v>
       </c>
       <c r="I68" s="6" t="s">
         <v>680</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>268</v>
+        <v>681</v>
       </c>
       <c r="K68" s="6" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="M68" s="6" t="s">
-        <v>271</v>
+        <v>684</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>666</v>
+        <v>685</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>429</v>
+        <v>25</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="E69" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="G69" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>691</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>692</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>693</v>
+      </c>
+      <c r="M69" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="N69" s="6" t="s">
         <v>685</v>
-      </c>
-      <c r="F69" s="6" t="s">
-        <v>686</v>
-      </c>
-      <c r="G69" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H69" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="I69" s="6" t="s">
-        <v>687</v>
-      </c>
-      <c r="J69" s="6" t="s">
-        <v>688</v>
-      </c>
-      <c r="K69" s="6" t="s">
-        <v>689</v>
-      </c>
-      <c r="L69" s="6" t="s">
-        <v>690</v>
-      </c>
-      <c r="M69" s="6" t="s">
-        <v>691</v>
-      </c>
-      <c r="N69" s="6" t="s">
-        <v>666</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>695</v>
-      </c>
-      <c r="G70" s="8" t="s">
-        <v>52</v>
+        <v>698</v>
+      </c>
+      <c r="G70" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>330</v>
+        <v>266</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>697</v>
+        <v>268</v>
       </c>
       <c r="K70" s="6" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="M70" s="6" t="s">
-        <v>700</v>
+        <v>271</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>701</v>
+        <v>685</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
         <v>702</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>25</v>
+        <v>448</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>317</v>
+        <v>703</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H71" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="I71" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="J71" s="6" t="s">
+        <v>707</v>
+      </c>
+      <c r="K71" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="L71" s="6" t="s">
+        <v>709</v>
+      </c>
+      <c r="M71" s="6" t="s">
+        <v>710</v>
+      </c>
+      <c r="N71" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="O71" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D72" s="6" t="s">
+        <v>712</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>713</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>714</v>
+      </c>
+      <c r="G72" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H72" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I72" s="6" t="s">
+        <v>715</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>716</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="L72" s="6" t="s">
+        <v>718</v>
+      </c>
+      <c r="M72" s="6" t="s">
+        <v>719</v>
+      </c>
+      <c r="N72" s="6" t="s">
+        <v>720</v>
+      </c>
+      <c r="O72" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="5" t="s">
+        <v>721</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>722</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>723</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H73" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I71" s="6" t="s">
-        <v>705</v>
-      </c>
-      <c r="J71" s="6" t="s">
-        <v>706</v>
-      </c>
-      <c r="K71" s="6" t="s">
-        <v>707</v>
-      </c>
-      <c r="L71" s="6" t="s">
-        <v>708</v>
-      </c>
-      <c r="M71" s="6" t="s">
-        <v>709</v>
-      </c>
-      <c r="N71" s="6" t="s">
-        <v>701</v>
-      </c>
-      <c r="O71" s="6" t="s">
+      <c r="I73" s="6" t="s">
+        <v>724</v>
+      </c>
+      <c r="J73" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>726</v>
+      </c>
+      <c r="L73" s="6" t="s">
+        <v>727</v>
+      </c>
+      <c r="M73" s="6" t="s">
+        <v>728</v>
+      </c>
+      <c r="N73" s="6" t="s">
+        <v>720</v>
+      </c>
+      <c r="O73" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6643,7 +6797,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -6664,7 +6818,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>710</v>
+        <v>729</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6711,7 +6865,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -6732,7 +6886,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>496</v>
+        <v>515</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -6753,7 +6907,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>586</v>
+        <v>605</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -6837,7 +6991,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>421</v>
+        <v>440</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -6900,7 +7054,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>660</v>
+        <v>679</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -6942,7 +7096,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>597</v>
+        <v>616</v>
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A15,'Bug List'!$G:$G,"Cao")</f>
@@ -7047,7 +7201,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Cao")</f>
@@ -7131,7 +7285,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>361</v>
+        <v>428</v>
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Cao")</f>
@@ -7139,7 +7293,7 @@
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Thấp")</f>
@@ -7147,12 +7301,12 @@
       </c>
       <c r="E24" s="12" t="n">
         <f aca="false">SUM(B24:D24)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>243</v>
+        <v>361</v>
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Cao")</f>
@@ -7160,7 +7314,7 @@
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Thấp")</f>
@@ -7168,20 +7322,20 @@
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">SUM(B25:D25)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>30</v>
+        <v>243</v>
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Trung")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Thấp")</f>
@@ -7189,37 +7343,37 @@
       </c>
       <c r="E26" s="12" t="n">
         <f aca="false">SUM(B26:D26)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="B27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">SUM(B27:D27)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>532</v>
+        <v>105</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Trung")</f>
@@ -7231,12 +7385,12 @@
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">SUM(B28:D28)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>222</v>
+        <v>551</v>
       </c>
       <c r="B29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Cao")</f>
@@ -7244,11 +7398,11 @@
       </c>
       <c r="C29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">SUM(B29:D29)</f>
@@ -7257,15 +7411,15 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="B30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Thấp")</f>
@@ -7278,7 +7432,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Cao")</f>
@@ -7286,7 +7440,7 @@
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Thấp")</f>
@@ -7294,16 +7448,16 @@
       </c>
       <c r="E31" s="12" t="n">
         <f aca="false">SUM(B31:D31)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>276</v>
+        <v>160</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Trung")</f>
@@ -7315,79 +7469,100 @@
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">SUM(B32:D32)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B33" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C33" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12" t="s">
-        <v>710</v>
-      </c>
-      <c r="B33" s="12" t="n">
-        <f aca="false">SUM(B2:B32)</f>
-        <v>23</v>
-      </c>
-      <c r="C33" s="12" t="n">
-        <f aca="false">SUM(C2:C32)</f>
-        <v>29</v>
-      </c>
-      <c r="D33" s="12" t="n">
-        <f aca="false">SUM(D2:D32)</f>
+      <c r="D33" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <f aca="false">SUM(B33:D33)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
+        <v>729</v>
+      </c>
+      <c r="B34" s="12" t="n">
+        <f aca="false">SUM(B2:B33)</f>
+        <v>24</v>
+      </c>
+      <c r="C34" s="12" t="n">
+        <f aca="false">SUM(C2:C33)</f>
+        <v>30</v>
+      </c>
+      <c r="D34" s="12" t="n">
+        <f aca="false">SUM(D2:D33)</f>
         <v>18</v>
       </c>
-      <c r="E33" s="12" t="n">
-        <f aca="false">SUM(E2:E32)</f>
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
+      <c r="E34" s="12" t="n">
+        <f aca="false">SUM(E2:E33)</f>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B35" s="12" t="s">
-        <v>711</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="11" t="s">
-        <v>712</v>
-      </c>
-      <c r="B36" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A36)</f>
-        <v>0</v>
+      <c r="B36" s="12" t="s">
+        <v>730</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>646</v>
+        <v>731</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A37)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>37</v>
+        <v>665</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A38)</f>
-        <v>69</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>713</v>
+        <v>37</v>
       </c>
       <c r="B39" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A39)</f>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>732</v>
+      </c>
+      <c r="B40" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A40)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>714</v>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>733</v>
       </c>
     </row>
   </sheetData>
@@ -7406,7 +7581,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
@@ -7415,10 +7590,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>715</v>
+        <v>734</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>716</v>
+        <v>735</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7426,7 +7601,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>717</v>
+        <v>736</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7434,15 +7609,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>718</v>
+        <v>737</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>719</v>
+        <v>738</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>720</v>
+        <v>739</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7450,95 +7625,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>721</v>
+        <v>740</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>722</v>
+        <v>741</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>723</v>
+        <v>742</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>724</v>
+        <v>743</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>725</v>
+        <v>744</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>726</v>
+        <v>745</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>727</v>
+        <v>746</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>728</v>
+        <v>747</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>729</v>
+        <v>748</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>730</v>
+        <v>749</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>731</v>
+        <v>750</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>732</v>
+        <v>751</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>733</v>
+        <v>752</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>734</v>
+        <v>753</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>735</v>
+        <v>754</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>736</v>
+        <v>755</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>737</v>
+        <v>756</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>738</v>
+        <v>757</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>739</v>
+        <v>758</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>740</v>
+        <v>759</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>741</v>
+        <v>760</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>742</v>
+        <v>761</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>743</v>
+        <v>762</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7546,31 +7721,39 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>744</v>
+        <v>763</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>745</v>
+        <v>764</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>746</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>747</v>
+        <v>766</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>748</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>749</v>
+        <v>768</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>750</v>
+        <v>769</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>428</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>770</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simulation: wait for the kitchen order view to open before reading it; bug list PT-41 (one-off CI E2E failure, open)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1190" uniqueCount="771">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="780">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1536,6 +1536,39 @@
     <t xml:space="preserve">Phân quyền phải lọc ở server, không chỉ ẩn trên giao diện. Mỗi vai trò mới: liệt kê trường dữ liệu nó được thấy và có test quét phản hồi không lộ trường khác.</t>
   </si>
   <si>
+    <t xml:space="preserve">PT-41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI / E2E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/e2e-staff.mjs (một lệnh fetch(...).json() của harness); GitHub Actions run 37293401352</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Actions job e2e (wrangler dev local, Google Chrome của runner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run 37293401352 (commit 4ee557c) đỏ ở job e2e với một dòng "Unexpected token 'E', \"Error: Net\"... is not valid JSON"; deploy bị chặn. Chạy lại cùng code trên CI (run 37294172954) và 3 lần local đều xanh ở bước e2e.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chưa xác định. Harness gọi fetch(...).json() và nhận văn bản "Error: Network connection lost." của workerd thay vì JSON, tức Worker local (wrangler dev) đã đứt kết nối hoặc khởi động lại giữa một request. Annotation lúc đó không có dòng script nên không biết bước nào.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annotation lỗi E2E giờ ghi kèm dòng script (line N) để lần sau đọc được ngay trên GitHub; không thêm retry để che lỗi.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Job e2e trong CI; lần đỏ sau phải đọc dòng script trong annotation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fail chỉ xảy ra trên CI thì không đóng bằng cách chạy lại cho xanh: ghi lại bằng chứng và tìm bước hỏng. Harness nên kiểm r.ok trước khi gọi .json() để báo rõ status và nội dung.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fcd0dcb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đang làm</t>
+  </si>
+  <si>
     <t xml:space="preserve">SAAS-01</t>
   </si>
   <si>
@@ -2006,9 +2039,6 @@
   </si>
   <si>
     <t xml:space="preserve">SAAS-17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CI / E2E</t>
   </si>
   <si>
     <t xml:space="preserve">scripts/e2e-staff.mjs; .github/workflows/ci.yml</t>
@@ -2361,9 +2391,6 @@
   </si>
   <si>
     <t xml:space="preserve">a65f8d5 + 34b760d (lotus-pos-saas; chưa rõ gốc)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đang làm</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-26</t>
@@ -3049,8 +3076,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O73" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O73"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O74"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3313,7 +3340,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O73"/>
+  <dimension ref="A1:O74"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -5265,72 +5292,72 @@
         <v>434</v>
       </c>
       <c r="B42" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D42" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="E42" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="G42" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="I42" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="J42" s="6" t="s">
         <v>439</v>
       </c>
-      <c r="G42" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H42" s="6" t="s">
+      <c r="K42" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="I42" s="6" t="s">
+      <c r="L42" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="J42" s="6" t="s">
+      <c r="M42" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="K42" s="6" t="s">
+      <c r="N42" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="L42" s="6" t="s">
+      <c r="O42" s="6" t="s">
         <v>444</v>
-      </c>
-      <c r="M42" s="6" t="s">
-        <v>445</v>
-      </c>
-      <c r="N42" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="O42" s="6" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="B43" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C43" s="6" t="s">
+      <c r="D43" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="E43" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="F43" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="F43" s="6" t="s">
+      <c r="G43" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H43" s="6" t="s">
         <v>451</v>
-      </c>
-      <c r="G43" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H43" s="6" t="s">
-        <v>440</v>
       </c>
       <c r="I43" s="6" t="s">
         <v>452</v>
@@ -5348,7 +5375,7 @@
         <v>456</v>
       </c>
       <c r="N43" s="6" t="s">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="O43" s="6" t="s">
         <v>37</v>
@@ -5356,46 +5383,46 @@
     </row>
     <row r="44" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H44" s="6" t="s">
+        <v>451</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="J44" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="K44" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="L44" s="6" t="s">
+        <v>466</v>
+      </c>
+      <c r="M44" s="6" t="s">
+        <v>467</v>
+      </c>
+      <c r="N44" s="6" t="s">
         <v>457</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>458</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="G44" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="I44" s="6" t="s">
-        <v>461</v>
-      </c>
-      <c r="J44" s="6" t="s">
-        <v>462</v>
-      </c>
-      <c r="K44" s="6" t="s">
-        <v>463</v>
-      </c>
-      <c r="L44" s="6" t="s">
-        <v>464</v>
-      </c>
-      <c r="M44" s="6" t="s">
-        <v>465</v>
-      </c>
-      <c r="N44" s="6" t="s">
-        <v>466</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>37</v>
@@ -5403,46 +5430,46 @@
     </row>
     <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>146</v>
+        <v>469</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="G45" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>470</v>
+        <v>451</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="L45" s="6" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="M45" s="6" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="N45" s="6" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>37</v>
@@ -5450,46 +5477,46 @@
     </row>
     <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>478</v>
+        <v>146</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>479</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>469</v>
+        <v>480</v>
       </c>
       <c r="G46" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
@@ -5497,46 +5524,46 @@
     </row>
     <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="E47" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="G47" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="M47" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="N47" s="6" t="s">
         <v>487</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>488</v>
-      </c>
-      <c r="G47" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H47" s="6" t="s">
-        <v>470</v>
-      </c>
-      <c r="I47" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="J47" s="6" t="s">
-        <v>490</v>
-      </c>
-      <c r="K47" s="6" t="s">
-        <v>491</v>
-      </c>
-      <c r="L47" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="M47" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="N47" s="6" t="s">
-        <v>476</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
@@ -5544,46 +5571,46 @@
     </row>
     <row r="48" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>80</v>
+        <v>497</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>469</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>52</v>
+        <v>499</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="M48" s="6" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>476</v>
+        <v>487</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
@@ -5591,46 +5618,46 @@
     </row>
     <row r="49" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>502</v>
+        <v>80</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>504</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>73</v>
+        <v>480</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>372</v>
+        <v>481</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>510</v>
+        <v>487</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
@@ -5638,28 +5665,28 @@
     </row>
     <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>515</v>
+        <v>372</v>
       </c>
       <c r="I50" s="6" t="s">
         <v>516</v>
@@ -5677,7 +5704,7 @@
         <v>520</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
@@ -5685,46 +5712,46 @@
     </row>
     <row r="51" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>53</v>
+        <v>526</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>530</v>
+        <v>521</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
@@ -5732,46 +5759,46 @@
     </row>
     <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>29</v>
+        <v>535</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
@@ -5779,46 +5806,46 @@
     </row>
     <row r="53" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>539</v>
+        <v>533</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="F53" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="M53" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="N53" s="6" t="s">
         <v>541</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H53" s="6" t="s">
-        <v>440</v>
-      </c>
-      <c r="I53" s="6" t="s">
-        <v>542</v>
-      </c>
-      <c r="J53" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="K53" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="L53" s="6" t="s">
-        <v>545</v>
-      </c>
-      <c r="M53" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="N53" s="6" t="s">
-        <v>510</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
@@ -5826,46 +5853,46 @@
     </row>
     <row r="54" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>551</v>
+        <v>451</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="M54" s="6" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>557</v>
+        <v>521</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
@@ -5876,43 +5903,43 @@
         <v>558</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>338</v>
+        <v>559</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G55" s="8" t="s">
-        <v>52</v>
+        <v>561</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>149</v>
+        <v>562</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
@@ -5920,22 +5947,22 @@
     </row>
     <row r="56" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>436</v>
+        <v>459</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>568</v>
+        <v>211</v>
       </c>
       <c r="G56" s="8" t="s">
         <v>52</v>
@@ -5944,22 +5971,22 @@
         <v>149</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>528</v>
+        <v>574</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
@@ -5967,46 +5994,46 @@
     </row>
     <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>307</v>
+        <v>578</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>575</v>
-      </c>
-      <c r="G57" s="9" t="s">
-        <v>73</v>
+        <v>579</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>579</v>
+        <v>539</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
@@ -6014,46 +6041,46 @@
     </row>
     <row r="58" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>583</v>
+        <v>306</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>584</v>
+        <v>307</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>585</v>
-      </c>
-      <c r="G58" s="8" t="s">
-        <v>52</v>
+        <v>586</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>361</v>
+        <v>309</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
@@ -6061,16 +6088,16 @@
     </row>
     <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B59" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D59" s="6" t="s">
         <v>435</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>593</v>
       </c>
       <c r="E59" s="6" t="s">
         <v>594</v>
@@ -6082,7 +6109,7 @@
         <v>52</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>470</v>
+        <v>361</v>
       </c>
       <c r="I59" s="6" t="s">
         <v>596</v>
@@ -6100,7 +6127,7 @@
         <v>600</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>591</v>
+        <v>601</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
@@ -6108,28 +6135,28 @@
     </row>
     <row r="60" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="G60" s="7" t="s">
-        <v>29</v>
+        <v>605</v>
+      </c>
+      <c r="G60" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>605</v>
+        <v>481</v>
       </c>
       <c r="I60" s="6" t="s">
         <v>606</v>
@@ -6147,7 +6174,7 @@
         <v>610</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>611</v>
+        <v>601</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
@@ -6155,46 +6182,46 @@
     </row>
     <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D61" s="6" t="s">
         <v>612</v>
       </c>
-      <c r="B61" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D61" s="6" t="s">
+      <c r="E61" s="6" t="s">
         <v>613</v>
       </c>
-      <c r="E61" s="6" t="s">
+      <c r="F61" s="6" t="s">
         <v>614</v>
-      </c>
-      <c r="F61" s="6" t="s">
-        <v>615</v>
       </c>
       <c r="G61" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H61" s="6" t="s">
+        <v>615</v>
+      </c>
+      <c r="I61" s="6" t="s">
         <v>616</v>
       </c>
-      <c r="I61" s="6" t="s">
+      <c r="J61" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="J61" s="6" t="s">
+      <c r="K61" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="K61" s="6" t="s">
+      <c r="L61" s="6" t="s">
         <v>619</v>
       </c>
-      <c r="L61" s="6" t="s">
+      <c r="M61" s="6" t="s">
         <v>620</v>
       </c>
-      <c r="M61" s="6" t="s">
+      <c r="N61" s="6" t="s">
         <v>621</v>
-      </c>
-      <c r="N61" s="6" t="s">
-        <v>622</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
@@ -6202,46 +6229,46 @@
     </row>
     <row r="62" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
+        <v>622</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D62" s="6" t="s">
         <v>623</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D62" s="6" t="s">
+      <c r="E62" s="6" t="s">
         <v>624</v>
       </c>
-      <c r="E62" s="6" t="s">
+      <c r="F62" s="6" t="s">
         <v>625</v>
       </c>
-      <c r="F62" s="6" t="s">
+      <c r="G62" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H62" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="G62" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H62" s="6" t="s">
+      <c r="I62" s="6" t="s">
         <v>627</v>
       </c>
-      <c r="I62" s="6" t="s">
+      <c r="J62" s="6" t="s">
         <v>628</v>
       </c>
-      <c r="J62" s="6" t="s">
+      <c r="K62" s="6" t="s">
         <v>629</v>
       </c>
-      <c r="K62" s="6" t="s">
+      <c r="L62" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="L62" s="6" t="s">
+      <c r="M62" s="6" t="s">
         <v>631</v>
       </c>
-      <c r="M62" s="6" t="s">
+      <c r="N62" s="6" t="s">
         <v>632</v>
-      </c>
-      <c r="N62" s="6" t="s">
-        <v>633</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
@@ -6249,28 +6276,28 @@
     </row>
     <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D63" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="B63" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D63" s="6" t="s">
+      <c r="E63" s="6" t="s">
         <v>635</v>
       </c>
-      <c r="E63" s="6" t="s">
+      <c r="F63" s="6" t="s">
         <v>636</v>
       </c>
-      <c r="F63" s="6" t="s">
+      <c r="G63" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H63" s="6" t="s">
         <v>637</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H63" s="6" t="s">
-        <v>627</v>
       </c>
       <c r="I63" s="6" t="s">
         <v>638</v>
@@ -6288,7 +6315,7 @@
         <v>642</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>622</v>
+        <v>643</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
@@ -6296,46 +6323,46 @@
     </row>
     <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>295</v>
+        <v>645</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>296</v>
+        <v>646</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G64" s="7" t="s">
-        <v>29</v>
+        <v>647</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>298</v>
+        <v>637</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>299</v>
+        <v>648</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>300</v>
+        <v>649</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
       <c r="M64" s="6" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>622</v>
+        <v>632</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
@@ -6343,46 +6370,46 @@
     </row>
     <row r="65" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>648</v>
+        <v>295</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>649</v>
+        <v>296</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>650</v>
+        <v>297</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>627</v>
+        <v>298</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>651</v>
+        <v>299</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>652</v>
+        <v>300</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>656</v>
+        <v>632</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
@@ -6393,63 +6420,63 @@
         <v>657</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>583</v>
+        <v>658</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>584</v>
+        <v>659</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="G66" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>361</v>
+        <v>637</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="M66" s="6" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="O66" s="6" t="s">
-        <v>665</v>
+        <v>37</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="B67" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D67" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="C67" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>648</v>
-      </c>
       <c r="E67" s="6" t="s">
-        <v>667</v>
+        <v>594</v>
       </c>
       <c r="F67" s="6" t="s">
         <v>668</v>
@@ -6458,7 +6485,7 @@
         <v>29</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>627</v>
+        <v>361</v>
       </c>
       <c r="I67" s="6" t="s">
         <v>669</v>
@@ -6479,7 +6506,7 @@
         <v>674</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6487,43 +6514,43 @@
         <v>675</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>448</v>
+        <v>459</v>
       </c>
       <c r="D68" s="6" t="s">
+        <v>658</v>
+      </c>
+      <c r="E68" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="F68" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="F68" s="6" t="s">
+      <c r="G68" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>637</v>
+      </c>
+      <c r="I68" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="G68" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H68" s="6" t="s">
+      <c r="J68" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="I68" s="6" t="s">
+      <c r="K68" s="6" t="s">
         <v>680</v>
       </c>
-      <c r="J68" s="6" t="s">
+      <c r="L68" s="6" t="s">
         <v>681</v>
       </c>
-      <c r="K68" s="6" t="s">
+      <c r="M68" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="L68" s="6" t="s">
+      <c r="N68" s="6" t="s">
         <v>683</v>
-      </c>
-      <c r="M68" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="N68" s="6" t="s">
-        <v>685</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
@@ -6531,46 +6558,46 @@
     </row>
     <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>459</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="E69" s="6" t="s">
         <v>686</v>
       </c>
-      <c r="B69" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D69" s="6" t="s">
+      <c r="F69" s="6" t="s">
         <v>687</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>688</v>
-      </c>
-      <c r="F69" s="6" t="s">
-        <v>689</v>
       </c>
       <c r="G69" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>255</v>
+        <v>688</v>
       </c>
       <c r="I69" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="J69" s="6" t="s">
         <v>690</v>
       </c>
-      <c r="J69" s="6" t="s">
+      <c r="K69" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="K69" s="6" t="s">
+      <c r="L69" s="6" t="s">
         <v>692</v>
       </c>
-      <c r="L69" s="6" t="s">
+      <c r="M69" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="M69" s="6" t="s">
+      <c r="N69" s="6" t="s">
         <v>694</v>
-      </c>
-      <c r="N69" s="6" t="s">
-        <v>685</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
@@ -6581,7 +6608,7 @@
         <v>695</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C70" s="6" t="s">
         <v>25</v>
@@ -6595,29 +6622,29 @@
       <c r="F70" s="6" t="s">
         <v>698</v>
       </c>
-      <c r="G70" s="9" t="s">
-        <v>73</v>
+      <c r="G70" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="I70" s="6" t="s">
         <v>699</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>268</v>
+        <v>700</v>
       </c>
       <c r="K70" s="6" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="M70" s="6" t="s">
-        <v>271</v>
+        <v>703</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>685</v>
+        <v>694</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>37</v>
@@ -6625,60 +6652,60 @@
     </row>
     <row r="71" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>448</v>
+        <v>25</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>705</v>
-      </c>
-      <c r="G71" s="7" t="s">
-        <v>29</v>
+        <v>707</v>
+      </c>
+      <c r="G71" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>707</v>
+        <v>268</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>710</v>
+        <v>271</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>685</v>
+        <v>694</v>
       </c>
       <c r="O71" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
         <v>711</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>25</v>
+        <v>459</v>
       </c>
       <c r="D72" s="6" t="s">
         <v>712</v>
@@ -6689,11 +6716,11 @@
       <c r="F72" s="6" t="s">
         <v>714</v>
       </c>
-      <c r="G72" s="8" t="s">
-        <v>52</v>
+      <c r="G72" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="I72" s="6" t="s">
         <v>715</v>
@@ -6711,24 +6738,24 @@
         <v>719</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>720</v>
+        <v>694</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>435</v>
+        <v>446</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>317</v>
+        <v>721</v>
       </c>
       <c r="E73" s="6" t="s">
         <v>722</v>
@@ -6736,11 +6763,11 @@
       <c r="F73" s="6" t="s">
         <v>723</v>
       </c>
-      <c r="G73" s="7" t="s">
-        <v>29</v>
+      <c r="G73" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="I73" s="6" t="s">
         <v>724</v>
@@ -6758,9 +6785,56 @@
         <v>728</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>720</v>
+        <v>729</v>
       </c>
       <c r="O73" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="5" t="s">
+        <v>730</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>731</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="G74" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="J74" s="6" t="s">
+        <v>734</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>735</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>736</v>
+      </c>
+      <c r="M74" s="6" t="s">
+        <v>737</v>
+      </c>
+      <c r="N74" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="O74" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6818,7 +6892,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>729</v>
+        <v>738</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6865,7 +6939,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>470</v>
+        <v>481</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -6886,7 +6960,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>515</v>
+        <v>526</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -6907,7 +6981,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>605</v>
+        <v>615</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -6991,7 +7065,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>440</v>
+        <v>451</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7054,7 +7128,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>679</v>
+        <v>688</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7096,7 +7170,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>616</v>
+        <v>626</v>
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A15,'Bug List'!$G:$G,"Cao")</f>
@@ -7201,7 +7275,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>627</v>
+        <v>637</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Cao")</f>
@@ -7314,7 +7388,7 @@
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Thấp")</f>
@@ -7322,7 +7396,7 @@
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">SUM(B25:D25)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7390,7 +7464,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="B29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Cao")</f>
@@ -7495,7 +7569,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>729</v>
+        <v>738</v>
       </c>
       <c r="B34" s="12" t="n">
         <f aca="false">SUM(B2:B33)</f>
@@ -7503,7 +7577,7 @@
       </c>
       <c r="C34" s="12" t="n">
         <f aca="false">SUM(C2:C33)</f>
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D34" s="12" t="n">
         <f aca="false">SUM(D2:D33)</f>
@@ -7511,7 +7585,7 @@
       </c>
       <c r="E34" s="12" t="n">
         <f aca="false">SUM(E2:E33)</f>
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -7520,12 +7594,12 @@
         <v>22</v>
       </c>
       <c r="B36" s="12" t="s">
-        <v>730</v>
+        <v>739</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>731</v>
+        <v>740</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A37)</f>
@@ -7534,11 +7608,11 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>665</v>
+        <v>444</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A38)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7552,7 +7626,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>732</v>
+        <v>741</v>
       </c>
       <c r="B40" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A40)</f>
@@ -7560,9 +7634,9 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>733</v>
+        <v>742</v>
       </c>
     </row>
   </sheetData>
@@ -7590,10 +7664,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>734</v>
+        <v>743</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>735</v>
+        <v>744</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7601,7 +7675,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>736</v>
+        <v>745</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7609,15 +7683,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>737</v>
+        <v>746</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>738</v>
+        <v>747</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>739</v>
+        <v>748</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7625,95 +7699,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>740</v>
+        <v>749</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>741</v>
+        <v>750</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>742</v>
+        <v>751</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>743</v>
+        <v>752</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>744</v>
+        <v>753</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>745</v>
+        <v>754</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>746</v>
+        <v>755</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>747</v>
+        <v>756</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>748</v>
+        <v>757</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>749</v>
+        <v>758</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>750</v>
+        <v>759</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>751</v>
+        <v>760</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>752</v>
+        <v>761</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>753</v>
+        <v>762</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>754</v>
+        <v>763</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>755</v>
+        <v>764</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>756</v>
+        <v>765</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>757</v>
+        <v>766</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>758</v>
+        <v>767</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>759</v>
+        <v>768</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>760</v>
+        <v>769</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>761</v>
+        <v>770</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>762</v>
+        <v>771</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7721,39 +7795,39 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>763</v>
+        <v>772</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>764</v>
+        <v>773</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>765</v>
+        <v>774</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>766</v>
+        <v>775</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>767</v>
+        <v>776</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>768</v>
+        <v>777</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>769</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>770</v>
+        <v>779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-42 refunded orders not marked in the order list, PT-43 phone menu loses its scroll, PT-44 duplicate Món & giá entry
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1205" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="811">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -2605,6 +2605,141 @@
   </si>
   <si>
     <t xml:space="preserve">Chữ trên giấy in là cam kết với khách và thuế: đặt ở một nơi (payload), các máy in chỉ trình bày.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm (ảnh chụp web nhân viên)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn hàng / Hoàn tiền</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/staff.js GET /api/staff/orders; public/staff/staff.js orderList(); public/staff/staff.css</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.../staff/ trên điện thoại, máy SUNMI, trang quầy (Lịch sử đơn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiển thị trạng thái</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn đã hoàn tiền toàn bộ vẫn hiện "POS · PAID" và "Đã thanh toán" trong danh sách đơn, giống hệt đơn bình thường; phải mở từng đơn mới thấy đã hoàn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API danh sách đơn chỉ trả các cột của qr_orders; tổng hoàn tiền nằm ở pos_refunds và chỉ được tính trong màn chi tiết đơn (overview). Danh sách không có dữ liệu để phân biệt.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Danh sách đơn kèm refundedAmount bằng subquery SUM(amount) trên pos_refunds (dùng idx_refunds_order, tối đa 100 đơn). Đơn có hoàn tiền được tô đỏ, nhãn "ĐÃ HOÀN TIỀN / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">已退款</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" hoặc "HOÀN MỘT PHẦN / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">部分退款</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" và số tiền đã hoàn. Tài khoản bếp vẫn không nhận trường tiền.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-42 the order list carries the refunded total of each order", "PT-42 a refunded order is drawn in red…"; scripts/sim-browser.mjs: "Handheld: an order refunded in full/in part shows in red on the order list".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Một trạng thái chỉ có ở màn chi tiết thì danh sách có đang nói sai không? Trạng thái tiền (đã trả, đã hoàn, hoàn một phần) phải thấy được ngay ở danh sách.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1786d9f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giao diện nhân viên / Điều hướng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js render()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Điện thoại và máy SUNMI (thanh menu dưới cuộn ngang); không lộ ở trang quầy (menu dọc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giao diện / thao tác</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi lần bấm một mục, mở đơn, quay lại hay đồng bộ tự động, thanh menu dưới nhảy về mục đầu tiên; muốn bấm Hoàn tiền, Chấm công, Quản trị phải kéo sang lại mỗi lần.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">render() dựng lại toàn bộ #app (cả &lt;nav&gt;) và chỉ khôi phục nav.scrollTop, viết cho menu dọc của trang quầy. Trên điện thoại menu cuộn ngang (overflow-x), nên scrollLeft luôn về 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lưu và khôi phục cả scrollLeft lẫn scrollTop của nav trong render().</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-43 a render keeps the sideways scroll…"; scripts/sim-browser.mjs: "Handheld: the phone menu keeps its sideways scroll after a tap, opening an order and live sync" (đỏ trên code cũ: 200px → 0px).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi giữ trạng thái giao diện qua một lần vẽ lại (cuộn, ô đang gõ, focus), đã tính hết các bố cục chưa: dọc/ngang, điện thoại/quầy?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js nav()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Điện thoại và máy SUNMI, tài khoản chủ tiệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm có hai lối vào cùng một màn "Món &amp; giá": một mục riêng trên thanh menu và một ô trong Quản trị chủ tiệm, làm menu dài và rối.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mục "Món &amp; giá" thêm vào menu theo quyền CATALOG_MANAGE trước khi có màn Quản trị; khi thêm Quản trị không bỏ mục cũ cho chủ tiệm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm vào Món &amp; giá từ Quản trị, mục Quản trị sáng khi đang ở các màn con của nó. Quản lý (MANAGER, có CATALOG_MANAGE nhưng không có Quản trị) vẫn giữ mục Món &amp; giá để không mất lối vào.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-44 the owner edits dishes and prices from Quản trị; a manager keeps the menu entry"; scripts/sim-browser.mjs: "Handheld: the owner reaches dishes &amp; prices from Quản trị only…"; scripts/e2e-staff.mjs đi qua Quản trị để sửa giá.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi bỏ một lối vào, vai trò nào chỉ có lối đó? Kiểm quyền (CATALOG_MANAGE của MANAGER) trước khi gỡ.</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -3076,8 +3211,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O74" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O77"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3340,7 +3475,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O74"/>
+  <dimension ref="A1:O77"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -6791,7 +6926,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
         <v>730</v>
       </c>
@@ -6835,6 +6970,147 @@
         <v>729</v>
       </c>
       <c r="O74" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5" t="s">
+        <v>738</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>739</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="G75" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="I75" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="J75" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="K75" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="L75" s="6" t="s">
+        <v>747</v>
+      </c>
+      <c r="M75" s="6" t="s">
+        <v>748</v>
+      </c>
+      <c r="N75" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="O75" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5" t="s">
+        <v>750</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C76" s="6" t="s">
+        <v>751</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>752</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>753</v>
+      </c>
+      <c r="F76" s="6" t="s">
+        <v>754</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>756</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>757</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>758</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>759</v>
+      </c>
+      <c r="M76" s="6" t="s">
+        <v>760</v>
+      </c>
+      <c r="N76" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="O76" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="5" t="s">
+        <v>761</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C77" s="6" t="s">
+        <v>751</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>752</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>763</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>755</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="K77" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="L77" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="M77" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="N77" s="6" t="s">
+        <v>749</v>
+      </c>
+      <c r="O77" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -6871,7 +7147,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -6892,7 +7168,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>738</v>
+        <v>769</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7149,7 +7425,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>287</v>
+        <v>755</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A14,'Bug List'!$G:$G,"Cao")</f>
@@ -7161,16 +7437,16 @@
       </c>
       <c r="D14" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A14,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="12" t="n">
         <f aca="false">SUM(B14:D14)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>626</v>
+        <v>287</v>
       </c>
       <c r="B15" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A15,'Bug List'!$G:$G,"Cao")</f>
@@ -7191,15 +7467,15 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>149</v>
+        <v>626</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Trung")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Thấp")</f>
@@ -7207,41 +7483,41 @@
       </c>
       <c r="E16" s="12" t="n">
         <f aca="false">SUM(B16:D16)</f>
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="B17" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A17,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C17" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A17,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D17" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A17,'Bug List'!$G:$G,"Thấp")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E17" s="12" t="n">
         <f aca="false">SUM(B17:D17)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>83</v>
+        <v>743</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A18,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A18,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D18" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A18,'Bug List'!$G:$G,"Thấp")</f>
@@ -7254,7 +7530,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>266</v>
+        <v>309</v>
       </c>
       <c r="B19" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A19,'Bug List'!$G:$G,"Cao")</f>
@@ -7275,7 +7551,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>637</v>
+        <v>83</v>
       </c>
       <c r="B20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Cao")</f>
@@ -7283,20 +7559,20 @@
       </c>
       <c r="C20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A20,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">SUM(B20:D20)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>320</v>
+        <v>266</v>
       </c>
       <c r="B21" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A21,'Bug List'!$G:$G,"Cao")</f>
@@ -7304,11 +7580,11 @@
       </c>
       <c r="C21" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A21,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A21,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E21" s="12" t="n">
         <f aca="false">SUM(B21:D21)</f>
@@ -7317,7 +7593,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>115</v>
+        <v>637</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -7325,20 +7601,20 @@
       </c>
       <c r="C22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E22" s="12" t="n">
         <f aca="false">SUM(B22:D22)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>201</v>
+        <v>320</v>
       </c>
       <c r="B23" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A23,'Bug List'!$G:$G,"Cao")</f>
@@ -7346,7 +7622,7 @@
       </c>
       <c r="C23" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A23,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A23,'Bug List'!$G:$G,"Thấp")</f>
@@ -7354,12 +7630,12 @@
       </c>
       <c r="E23" s="12" t="n">
         <f aca="false">SUM(B23:D23)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>428</v>
+        <v>115</v>
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Cao")</f>
@@ -7380,15 +7656,15 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>361</v>
+        <v>201</v>
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Trung")</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Thấp")</f>
@@ -7396,12 +7672,12 @@
       </c>
       <c r="E25" s="12" t="n">
         <f aca="false">SUM(B25:D25)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>243</v>
+        <v>428</v>
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Cao")</f>
@@ -7422,15 +7698,15 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>30</v>
+        <v>361</v>
       </c>
       <c r="B27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Trung")</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Thấp")</f>
@@ -7438,12 +7714,12 @@
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">SUM(B27:D27)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>105</v>
+        <v>243</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Cao")</f>
@@ -7455,16 +7731,16 @@
       </c>
       <c r="D28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">SUM(B28:D28)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>562</v>
+        <v>30</v>
       </c>
       <c r="B29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Cao")</f>
@@ -7472,45 +7748,45 @@
       </c>
       <c r="C29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">SUM(B29:D29)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>222</v>
+        <v>105</v>
       </c>
       <c r="B30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">SUM(B30:D30)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>94</v>
+        <v>562</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Trung")</f>
@@ -7518,7 +7794,7 @@
       </c>
       <c r="D31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E31" s="12" t="n">
         <f aca="false">SUM(B31:D31)</f>
@@ -7527,15 +7803,15 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>160</v>
+        <v>222</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Thấp")</f>
@@ -7543,20 +7819,20 @@
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">SUM(B32:D32)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>276</v>
+        <v>94</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Thấp")</f>
@@ -7564,79 +7840,120 @@
       </c>
       <c r="E33" s="12" t="n">
         <f aca="false">SUM(B33:D33)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="B34" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Cao")</f>
+        <v>1</v>
+      </c>
+      <c r="C34" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="s">
-        <v>738</v>
-      </c>
-      <c r="B34" s="12" t="n">
-        <f aca="false">SUM(B2:B33)</f>
-        <v>24</v>
-      </c>
-      <c r="C34" s="12" t="n">
-        <f aca="false">SUM(C2:C33)</f>
-        <v>31</v>
-      </c>
-      <c r="D34" s="12" t="n">
-        <f aca="false">SUM(D2:D33)</f>
-        <v>18</v>
+      <c r="D34" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
       </c>
       <c r="E34" s="12" t="n">
-        <f aca="false">SUM(E2:E33)</f>
-        <v>73</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <f aca="false">SUM(B34:D34)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B35" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Trung")</f>
+        <v>2</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <f aca="false">SUM(B35:D35)</f>
+        <v>2</v>
+      </c>
+    </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
+        <v>769</v>
+      </c>
+      <c r="B36" s="12" t="n">
+        <f aca="false">SUM(B2:B35)</f>
+        <v>24</v>
+      </c>
+      <c r="C36" s="12" t="n">
+        <f aca="false">SUM(C2:C35)</f>
+        <v>33</v>
+      </c>
+      <c r="D36" s="12" t="n">
+        <f aca="false">SUM(D2:D35)</f>
+        <v>19</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <f aca="false">SUM(E2:E35)</f>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B36" s="12" t="s">
-        <v>739</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>740</v>
-      </c>
-      <c r="B37" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A37)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="11" t="s">
-        <v>444</v>
-      </c>
-      <c r="B38" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A38)</f>
-        <v>2</v>
+      <c r="B38" s="12" t="s">
+        <v>770</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>37</v>
+        <v>771</v>
       </c>
       <c r="B39" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A39)</f>
-        <v>71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>741</v>
+        <v>444</v>
       </c>
       <c r="B40" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A40)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A41)</f>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="11" t="s">
+        <v>772</v>
+      </c>
+      <c r="B42" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A42)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>742</v>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="13" t="s">
+        <v>773</v>
       </c>
     </row>
   </sheetData>
@@ -7664,10 +7981,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>743</v>
+        <v>774</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>744</v>
+        <v>775</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7675,7 +7992,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>745</v>
+        <v>776</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7683,15 +8000,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>746</v>
+        <v>777</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>747</v>
+        <v>778</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>748</v>
+        <v>779</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7699,95 +8016,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>749</v>
+        <v>780</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>750</v>
+        <v>781</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>751</v>
+        <v>782</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>752</v>
+        <v>783</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>753</v>
+        <v>784</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>754</v>
+        <v>785</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>755</v>
+        <v>786</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>756</v>
+        <v>787</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>757</v>
+        <v>788</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>758</v>
+        <v>789</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>759</v>
+        <v>790</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>760</v>
+        <v>791</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>761</v>
+        <v>792</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>762</v>
+        <v>793</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>763</v>
+        <v>794</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>764</v>
+        <v>795</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>765</v>
+        <v>796</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>766</v>
+        <v>797</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>767</v>
+        <v>798</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>768</v>
+        <v>799</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>769</v>
+        <v>800</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>770</v>
+        <v>801</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>771</v>
+        <v>802</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7795,31 +8112,31 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>772</v>
+        <v>803</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>773</v>
+        <v>804</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>774</v>
+        <v>805</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>775</v>
+        <v>806</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>776</v>
+        <v>807</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>777</v>
+        <v>808</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>778</v>
+        <v>809</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7827,7 +8144,7 @@
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>779</v>
+        <v>810</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: keep PT rows together ahead of SAAS rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -1569,6 +1569,141 @@
     <t xml:space="preserve">Đang làm</t>
   </si>
   <si>
+    <t xml:space="preserve">PT-42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm (ảnh chụp web nhân viên)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn hàng / Hoàn tiền</t>
+  </si>
+  <si>
+    <t xml:space="preserve">src/staff.js GET /api/staff/orders; public/staff/staff.js orderList(); public/staff/staff.css</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.../staff/ trên điện thoại, máy SUNMI, trang quầy (Lịch sử đơn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiển thị trạng thái</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn đã hoàn tiền toàn bộ vẫn hiện "POS · PAID" và "Đã thanh toán" trong danh sách đơn, giống hệt đơn bình thường; phải mở từng đơn mới thấy đã hoàn.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API danh sách đơn chỉ trả các cột của qr_orders; tổng hoàn tiền nằm ở pos_refunds và chỉ được tính trong màn chi tiết đơn (overview). Danh sách không có dữ liệu để phân biệt.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Danh sách đơn kèm refundedAmount bằng subquery SUM(amount) trên pos_refunds (dùng idx_refunds_order, tối đa 100 đơn). Đơn có hoàn tiền được tô đỏ, nhãn "ĐÃ HOÀN TIỀN / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">已退款</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" hoặc "HOÀN MỘT PHẦN / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">部分退款</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" và số tiền đã hoàn. Tài khoản bếp vẫn không nhận trường tiền.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-42 the order list carries the refunded total of each order", "PT-42 a refunded order is drawn in red…"; scripts/sim-browser.mjs: "Handheld: an order refunded in full/in part shows in red on the order list".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Một trạng thái chỉ có ở màn chi tiết thì danh sách có đang nói sai không? Trạng thái tiền (đã trả, đã hoàn, hoàn một phần) phải thấy được ngay ở danh sách.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1786d9f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giao diện nhân viên / Điều hướng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js render()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Điện thoại và máy SUNMI (thanh menu dưới cuộn ngang); không lộ ở trang quầy (menu dọc)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giao diện / thao tác</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mỗi lần bấm một mục, mở đơn, quay lại hay đồng bộ tự động, thanh menu dưới nhảy về mục đầu tiên; muốn bấm Hoàn tiền, Chấm công, Quản trị phải kéo sang lại mỗi lần.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">render() dựng lại toàn bộ #app (cả &lt;nav&gt;) và chỉ khôi phục nav.scrollTop, viết cho menu dọc của trang quầy. Trên điện thoại menu cuộn ngang (overflow-x), nên scrollLeft luôn về 0.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lưu và khôi phục cả scrollLeft lẫn scrollTop của nav trong render().</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-43 a render keeps the sideways scroll…"; scripts/sim-browser.mjs: "Handheld: the phone menu keeps its sideways scroll after a tap, opening an order and live sync" (đỏ trên code cũ: 200px → 0px).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi giữ trạng thái giao diện qua một lần vẽ lại (cuộn, ô đang gõ, focus), đã tính hết các bố cục chưa: dọc/ngang, điện thoại/quầy?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js nav()</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Điện thoại và máy SUNMI, tài khoản chủ tiệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm có hai lối vào cùng một màn "Món &amp; giá": một mục riêng trên thanh menu và một ô trong Quản trị chủ tiệm, làm menu dài và rối.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mục "Món &amp; giá" thêm vào menu theo quyền CATALOG_MANAGE trước khi có màn Quản trị; khi thêm Quản trị không bỏ mục cũ cho chủ tiệm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm vào Món &amp; giá từ Quản trị, mục Quản trị sáng khi đang ở các màn con của nó. Quản lý (MANAGER, có CATALOG_MANAGE nhưng không có Quản trị) vẫn giữ mục Món &amp; giá để không mất lối vào.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-44 the owner edits dishes and prices from Quản trị; a manager keeps the menu entry"; scripts/sim-browser.mjs: "Handheld: the owner reaches dishes &amp; prices from Quản trị only…"; scripts/e2e-staff.mjs đi qua Quản trị để sửa giá.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khi bỏ một lối vào, vai trò nào chỉ có lối đó? Kiểm quyền (CATALOG_MANAGE của MANAGER) trước khi gỡ.</t>
+  </si>
+  <si>
     <t xml:space="preserve">SAAS-01</t>
   </si>
   <si>
@@ -2605,141 +2740,6 @@
   </si>
   <si>
     <t xml:space="preserve">Chữ trên giấy in là cam kết với khách và thuế: đặt ở một nơi (payload), các máy in chỉ trình bày.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PT-42</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ tiệm (ảnh chụp web nhân viên)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đơn hàng / Hoàn tiền</t>
-  </si>
-  <si>
-    <t xml:space="preserve">src/staff.js GET /api/staff/orders; public/staff/staff.js orderList(); public/staff/staff.css</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.../staff/ trên điện thoại, máy SUNMI, trang quầy (Lịch sử đơn)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hiển thị trạng thái</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Đơn đã hoàn tiền toàn bộ vẫn hiện "POS · PAID" và "Đã thanh toán" trong danh sách đơn, giống hệt đơn bình thường; phải mở từng đơn mới thấy đã hoàn.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">API danh sách đơn chỉ trả các cột của qr_orders; tổng hoàn tiền nằm ở pos_refunds và chỉ được tính trong màn chi tiết đơn (overview). Danh sách không có dữ liệu để phân biệt.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Danh sách đơn kèm refundedAmount bằng subquery SUM(amount) trên pos_refunds (dùng idx_refunds_order, tối đa 100 đơn). Đơn có hoàn tiền được tô đỏ, nhãn "ĐÃ HOÀN TIỀN / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">已退款</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">" hoặc "HOÀN MỘT PHẦN / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Noto Sans CJK SC"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">部分退款</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">" và số tiền đã hoàn. Tài khoản bếp vẫn không nhận trường tiền.</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-42 the order list carries the refunded total of each order", "PT-42 a refunded order is drawn in red…"; scripts/sim-browser.mjs: "Handheld: an order refunded in full/in part shows in red on the order list".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Một trạng thái chỉ có ở màn chi tiết thì danh sách có đang nói sai không? Trạng thái tiền (đã trả, đã hoàn, hoàn một phần) phải thấy được ngay ở danh sách.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1786d9f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PT-43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ tiệm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giao diện nhân viên / Điều hướng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">public/staff/staff.js render()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Điện thoại và máy SUNMI (thanh menu dưới cuộn ngang); không lộ ở trang quầy (menu dọc)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Giao diện / thao tác</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mỗi lần bấm một mục, mở đơn, quay lại hay đồng bộ tự động, thanh menu dưới nhảy về mục đầu tiên; muốn bấm Hoàn tiền, Chấm công, Quản trị phải kéo sang lại mỗi lần.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">render() dựng lại toàn bộ #app (cả &lt;nav&gt;) và chỉ khôi phục nav.scrollTop, viết cho menu dọc của trang quầy. Trên điện thoại menu cuộn ngang (overflow-x), nên scrollLeft luôn về 0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lưu và khôi phục cả scrollLeft lẫn scrollTop của nav trong render().</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-43 a render keeps the sideways scroll…"; scripts/sim-browser.mjs: "Handheld: the phone menu keeps its sideways scroll after a tap, opening an order and live sync" (đỏ trên code cũ: 200px → 0px).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khi giữ trạng thái giao diện qua một lần vẽ lại (cuộn, ô đang gõ, focus), đã tính hết các bố cục chưa: dọc/ngang, điện thoại/quầy?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PT-44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">public/staff/staff.js nav()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Điện thoại và máy SUNMI, tài khoản chủ tiệm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ tiệm có hai lối vào cùng một màn "Món &amp; giá": một mục riêng trên thanh menu và một ô trong Quản trị chủ tiệm, làm menu dài và rối.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mục "Món &amp; giá" thêm vào menu theo quyền CATALOG_MANAGE trước khi có màn Quản trị; khi thêm Quản trị không bỏ mục cũ cho chủ tiệm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ tiệm vào Món &amp; giá từ Quản trị, mục Quản trị sáng khi đang ở các màn con của nó. Quản lý (MANAGER, có CATALOG_MANAGE nhưng không có Quản trị) vẫn giữ mục Món &amp; giá để không mất lối vào.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/phattai-v182-owner-ux.test.mjs: "PT-44 the owner edits dishes and prices from Quản trị; a manager keeps the menu entry"; scripts/sim-browser.mjs: "Handheld: the owner reaches dishes &amp; prices from Quản trị only…"; scripts/e2e-staff.mjs đi qua Quản trị để sửa giá.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khi bỏ một lối vào, vai trò nào chỉ có lối đó? Kiểm quyền (CATALOG_MANAGE của MANAGER) trước khi gỡ.</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -3028,7 +3028,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3073,19 +3073,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5469,77 +5465,77 @@
         <v>444</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
         <v>445</v>
       </c>
       <c r="B43" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C43" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="D43" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="E43" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="F43" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="F43" s="6" t="s">
+      <c r="G43" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H43" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="G43" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H43" s="6" t="s">
+      <c r="I43" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="J43" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="J43" s="6" t="s">
+      <c r="K43" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="K43" s="6" t="s">
+      <c r="L43" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="L43" s="6" t="s">
+      <c r="M43" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="M43" s="6" t="s">
+      <c r="N43" s="6" t="s">
         <v>456</v>
-      </c>
-      <c r="N43" s="6" t="s">
-        <v>457</v>
       </c>
       <c r="O43" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C44" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="B44" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C44" s="6" t="s">
+      <c r="D44" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="E44" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="E44" s="6" t="s">
+      <c r="F44" s="6" t="s">
         <v>461</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>462</v>
       </c>
       <c r="G44" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>451</v>
+        <v>462</v>
       </c>
       <c r="I44" s="6" t="s">
         <v>463</v>
@@ -5557,101 +5553,101 @@
         <v>467</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
         <v>468</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>446</v>
+        <v>251</v>
       </c>
       <c r="C45" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>459</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="E45" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="E45" s="6" t="s">
+      <c r="F45" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="F45" s="6" t="s">
+      <c r="G45" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H45" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="I45" s="6" t="s">
         <v>471</v>
       </c>
-      <c r="G45" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H45" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="I45" s="6" t="s">
+      <c r="J45" s="6" t="s">
         <v>472</v>
       </c>
-      <c r="J45" s="6" t="s">
+      <c r="K45" s="6" t="s">
         <v>473</v>
       </c>
-      <c r="K45" s="6" t="s">
+      <c r="L45" s="6" t="s">
         <v>474</v>
       </c>
-      <c r="L45" s="6" t="s">
+      <c r="M45" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="M45" s="6" t="s">
-        <v>476</v>
-      </c>
       <c r="N45" s="6" t="s">
-        <v>477</v>
+        <v>456</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>459</v>
-      </c>
       <c r="D46" s="6" t="s">
-        <v>146</v>
+        <v>479</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G46" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="L46" s="6" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="M46" s="6" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
@@ -5659,140 +5655,140 @@
     </row>
     <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
+        <v>489</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>491</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>493</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>482</v>
+      </c>
+      <c r="I47" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="M47" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="N47" s="6" t="s">
         <v>488</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>490</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>480</v>
-      </c>
-      <c r="G47" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H47" s="6" t="s">
-        <v>481</v>
-      </c>
-      <c r="I47" s="6" t="s">
-        <v>491</v>
-      </c>
-      <c r="J47" s="6" t="s">
-        <v>492</v>
-      </c>
-      <c r="K47" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="L47" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="M47" s="6" t="s">
-        <v>495</v>
-      </c>
-      <c r="N47" s="6" t="s">
-        <v>487</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="G48" s="7" t="s">
-        <v>29</v>
+        <v>502</v>
+      </c>
+      <c r="G48" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="J48" s="6" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="K48" s="6" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="L48" s="6" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="M48" s="6" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>487</v>
+        <v>508</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>80</v>
+        <v>146</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>480</v>
+        <v>511</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>481</v>
+        <v>512</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>507</v>
+        <v>513</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>508</v>
+        <v>514</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>509</v>
+        <v>515</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>487</v>
+        <v>518</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
@@ -5800,592 +5796,592 @@
     </row>
     <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
+        <v>519</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="G50" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H50" s="6" t="s">
         <v>512</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>513</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>515</v>
-      </c>
-      <c r="G50" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>372</v>
-      </c>
       <c r="I50" s="6" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="K50" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="M50" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="N50" s="6" t="s">
         <v>518</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>519</v>
-      </c>
-      <c r="M50" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="N50" s="6" t="s">
-        <v>521</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>522</v>
+        <v>527</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>523</v>
+        <v>528</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>524</v>
+        <v>529</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>525</v>
-      </c>
-      <c r="G51" s="9" t="s">
-        <v>73</v>
+        <v>530</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>526</v>
+        <v>512</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>533</v>
+        <v>80</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>535</v>
-      </c>
-      <c r="G52" s="9" t="s">
-        <v>73</v>
+        <v>511</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>53</v>
+        <v>512</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>541</v>
+        <v>518</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>533</v>
+        <v>544</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G53" s="7" t="s">
-        <v>29</v>
+        <v>546</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>30</v>
+        <v>372</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="M53" s="6" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>541</v>
+        <v>552</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>451</v>
+        <v>557</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>553</v>
+        <v>558</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>554</v>
+        <v>559</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>556</v>
+        <v>561</v>
       </c>
       <c r="M54" s="6" t="s">
-        <v>557</v>
+        <v>562</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>521</v>
+        <v>552</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>559</v>
+        <v>564</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>560</v>
+        <v>565</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>561</v>
+        <v>566</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>562</v>
+        <v>53</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>338</v>
+        <v>564</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G56" s="8" t="s">
-        <v>52</v>
+        <v>28</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>149</v>
+        <v>30</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="J56" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="K56" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="L56" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="M56" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="N56" s="6" t="s">
         <v>572</v>
-      </c>
-      <c r="K56" s="6" t="s">
-        <v>573</v>
-      </c>
-      <c r="L56" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="M56" s="6" t="s">
-        <v>575</v>
-      </c>
-      <c r="N56" s="6" t="s">
-        <v>576</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>447</v>
+        <v>490</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>146</v>
+        <v>581</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="G57" s="8" t="s">
-        <v>52</v>
+        <v>583</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>149</v>
+        <v>482</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>539</v>
+        <v>587</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>583</v>
+        <v>588</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>584</v>
+        <v>552</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>306</v>
+        <v>590</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>307</v>
+        <v>591</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>586</v>
+        <v>592</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>309</v>
+        <v>593</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>592</v>
+        <v>599</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>593</v>
+        <v>600</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>435</v>
+        <v>338</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>594</v>
+        <v>601</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>595</v>
+        <v>211</v>
       </c>
       <c r="G59" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>361</v>
+        <v>149</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>596</v>
+        <v>602</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>597</v>
+        <v>603</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>598</v>
+        <v>604</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>599</v>
+        <v>605</v>
       </c>
       <c r="M59" s="6" t="s">
-        <v>600</v>
+        <v>606</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>602</v>
+        <v>608</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>459</v>
+        <v>478</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>603</v>
+        <v>146</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>604</v>
+        <v>609</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>605</v>
+        <v>610</v>
       </c>
       <c r="G60" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>481</v>
+        <v>149</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>606</v>
+        <v>611</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>607</v>
+        <v>612</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>608</v>
+        <v>613</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>609</v>
+        <v>570</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>601</v>
+        <v>615</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>611</v>
+        <v>616</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>612</v>
+        <v>306</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>613</v>
+        <v>307</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>614</v>
-      </c>
-      <c r="G61" s="7" t="s">
-        <v>29</v>
+        <v>617</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>615</v>
+        <v>309</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="K61" s="6" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>623</v>
+        <v>435</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="G62" s="7" t="s">
-        <v>29</v>
+        <v>626</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>626</v>
+        <v>361</v>
       </c>
       <c r="I62" s="6" t="s">
         <v>627</v>
@@ -6409,15 +6405,15 @@
         <v>37</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
         <v>633</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D63" s="6" t="s">
         <v>634</v>
@@ -6432,495 +6428,495 @@
         <v>52</v>
       </c>
       <c r="H63" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="I63" s="6" t="s">
         <v>637</v>
       </c>
-      <c r="I63" s="6" t="s">
+      <c r="J63" s="6" t="s">
         <v>638</v>
       </c>
-      <c r="J63" s="6" t="s">
+      <c r="K63" s="6" t="s">
         <v>639</v>
       </c>
-      <c r="K63" s="6" t="s">
+      <c r="L63" s="6" t="s">
         <v>640</v>
       </c>
-      <c r="L63" s="6" t="s">
+      <c r="M63" s="6" t="s">
         <v>641</v>
       </c>
-      <c r="M63" s="6" t="s">
-        <v>642</v>
-      </c>
       <c r="N63" s="6" t="s">
-        <v>643</v>
+        <v>632</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
+        <v>642</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="E64" s="6" t="s">
         <v>644</v>
       </c>
-      <c r="B64" s="6" t="s">
-        <v>446</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>459</v>
-      </c>
-      <c r="D64" s="6" t="s">
+      <c r="F64" s="6" t="s">
         <v>645</v>
       </c>
-      <c r="E64" s="6" t="s">
+      <c r="G64" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H64" s="6" t="s">
         <v>646</v>
       </c>
-      <c r="F64" s="6" t="s">
+      <c r="I64" s="6" t="s">
         <v>647</v>
       </c>
-      <c r="G64" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>637</v>
-      </c>
-      <c r="I64" s="6" t="s">
+      <c r="J64" s="6" t="s">
         <v>648</v>
       </c>
-      <c r="J64" s="6" t="s">
+      <c r="K64" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="K64" s="6" t="s">
+      <c r="L64" s="6" t="s">
         <v>650</v>
       </c>
-      <c r="L64" s="6" t="s">
+      <c r="M64" s="6" t="s">
         <v>651</v>
       </c>
-      <c r="M64" s="6" t="s">
+      <c r="N64" s="6" t="s">
         <v>652</v>
-      </c>
-      <c r="N64" s="6" t="s">
-        <v>632</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
         <v>653</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>295</v>
+        <v>654</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>296</v>
+        <v>655</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>297</v>
+        <v>656</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>298</v>
+        <v>657</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>299</v>
+        <v>658</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>300</v>
+        <v>659</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>656</v>
+        <v>662</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>632</v>
+        <v>663</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>657</v>
+        <v>664</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>658</v>
+        <v>665</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>659</v>
+        <v>666</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>660</v>
-      </c>
-      <c r="G66" s="7" t="s">
-        <v>29</v>
+        <v>667</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>637</v>
+        <v>668</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>661</v>
+        <v>669</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>662</v>
+        <v>670</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>663</v>
+        <v>671</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>664</v>
+        <v>672</v>
       </c>
       <c r="M66" s="6" t="s">
-        <v>665</v>
+        <v>673</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>666</v>
+        <v>674</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>667</v>
+        <v>675</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>435</v>
+        <v>676</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>594</v>
+        <v>677</v>
       </c>
       <c r="F67" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H67" s="6" t="s">
         <v>668</v>
       </c>
-      <c r="G67" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H67" s="6" t="s">
-        <v>361</v>
-      </c>
       <c r="I67" s="6" t="s">
-        <v>669</v>
+        <v>679</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>670</v>
+        <v>680</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>671</v>
+        <v>681</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>672</v>
+        <v>682</v>
       </c>
       <c r="M67" s="6" t="s">
-        <v>673</v>
+        <v>683</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>674</v>
+        <v>663</v>
       </c>
       <c r="O67" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>675</v>
+        <v>684</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>658</v>
+        <v>295</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>676</v>
+        <v>296</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>677</v>
+        <v>297</v>
       </c>
       <c r="G68" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>637</v>
+        <v>298</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>678</v>
+        <v>299</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>679</v>
+        <v>300</v>
       </c>
       <c r="K68" s="6" t="s">
-        <v>680</v>
+        <v>685</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>681</v>
+        <v>686</v>
       </c>
       <c r="M68" s="6" t="s">
-        <v>682</v>
+        <v>687</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>683</v>
+        <v>663</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>687</v>
-      </c>
-      <c r="G69" s="8" t="s">
-        <v>52</v>
+        <v>691</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>688</v>
+        <v>668</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="K69" s="6" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>25</v>
+        <v>490</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>696</v>
+        <v>435</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>697</v>
+        <v>625</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>698</v>
-      </c>
-      <c r="G70" s="8" t="s">
-        <v>52</v>
+        <v>699</v>
+      </c>
+      <c r="G70" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>255</v>
+        <v>361</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="K70" s="6" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="M70" s="6" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>694</v>
+        <v>705</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>25</v>
+        <v>490</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>705</v>
+        <v>689</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>707</v>
-      </c>
-      <c r="G71" s="9" t="s">
-        <v>73</v>
+        <v>708</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>266</v>
+        <v>668</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>268</v>
+        <v>710</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>271</v>
+        <v>713</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>694</v>
+        <v>714</v>
       </c>
       <c r="O71" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>459</v>
+        <v>490</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>714</v>
-      </c>
-      <c r="G72" s="7" t="s">
-        <v>29</v>
+        <v>718</v>
+      </c>
+      <c r="G72" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>276</v>
+        <v>719</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="K72" s="6" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>694</v>
+        <v>725</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C73" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>330</v>
+        <v>255</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="J73" s="6" t="s">
+        <v>731</v>
+      </c>
+      <c r="K73" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="L73" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="M73" s="6" t="s">
+        <v>734</v>
+      </c>
+      <c r="N73" s="6" t="s">
         <v>725</v>
-      </c>
-      <c r="K73" s="6" t="s">
-        <v>726</v>
-      </c>
-      <c r="L73" s="6" t="s">
-        <v>727</v>
-      </c>
-      <c r="M73" s="6" t="s">
-        <v>728</v>
-      </c>
-      <c r="N73" s="6" t="s">
-        <v>729</v>
       </c>
       <c r="O73" s="6" t="s">
         <v>37</v>
@@ -6928,107 +6924,107 @@
     </row>
     <row r="74" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>730</v>
+        <v>735</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>446</v>
+        <v>477</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>317</v>
+        <v>736</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>732</v>
-      </c>
-      <c r="G74" s="7" t="s">
-        <v>29</v>
+        <v>738</v>
+      </c>
+      <c r="G74" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>320</v>
+        <v>266</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>734</v>
+        <v>268</v>
       </c>
       <c r="K74" s="6" t="s">
-        <v>735</v>
+        <v>740</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="M74" s="6" t="s">
-        <v>737</v>
+        <v>271</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>729</v>
+        <v>725</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>251</v>
+        <v>477</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>739</v>
+        <v>490</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="G75" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>743</v>
+        <v>276</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="K75" s="6" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="M75" s="6" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>749</v>
+        <v>725</v>
       </c>
       <c r="O75" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>251</v>
+        <v>477</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>751</v>
+        <v>25</v>
       </c>
       <c r="D76" s="6" t="s">
         <v>752</v>
@@ -7039,46 +7035,46 @@
       <c r="F76" s="6" t="s">
         <v>754</v>
       </c>
-      <c r="G76" s="7" t="s">
-        <v>29</v>
+      <c r="G76" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H76" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I76" s="6" t="s">
         <v>755</v>
       </c>
-      <c r="I76" s="6" t="s">
+      <c r="J76" s="6" t="s">
         <v>756</v>
       </c>
-      <c r="J76" s="6" t="s">
+      <c r="K76" s="6" t="s">
         <v>757</v>
       </c>
-      <c r="K76" s="6" t="s">
+      <c r="L76" s="6" t="s">
         <v>758</v>
       </c>
-      <c r="L76" s="6" t="s">
+      <c r="M76" s="6" t="s">
         <v>759</v>
       </c>
-      <c r="M76" s="6" t="s">
+      <c r="N76" s="6" t="s">
         <v>760</v>
-      </c>
-      <c r="N76" s="6" t="s">
-        <v>749</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
         <v>761</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>251</v>
+        <v>477</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>751</v>
+        <v>25</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>752</v>
+        <v>317</v>
       </c>
       <c r="E77" s="6" t="s">
         <v>762</v>
@@ -7086,11 +7082,11 @@
       <c r="F77" s="6" t="s">
         <v>763</v>
       </c>
-      <c r="G77" s="9" t="s">
-        <v>73</v>
+      <c r="G77" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>755</v>
+        <v>320</v>
       </c>
       <c r="I77" s="6" t="s">
         <v>764</v>
@@ -7108,7 +7104,7 @@
         <v>768</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="O77" s="6" t="s">
         <v>37</v>
@@ -7215,7 +7211,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>481</v>
+        <v>512</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -7236,7 +7232,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>526</v>
+        <v>557</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -7257,7 +7253,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>615</v>
+        <v>646</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -7341,7 +7337,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>451</v>
+        <v>482</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7404,7 +7400,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>688</v>
+        <v>719</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7425,7 +7421,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>755</v>
+        <v>462</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A14,'Bug List'!$G:$G,"Cao")</f>
@@ -7467,7 +7463,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>626</v>
+        <v>657</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
@@ -7509,7 +7505,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>743</v>
+        <v>450</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A18,'Bug List'!$G:$G,"Cao")</f>
@@ -7593,7 +7589,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>637</v>
+        <v>668</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -7782,7 +7778,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>562</v>
+        <v>593</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Cao")</f>
@@ -7951,7 +7947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="13" t="s">
         <v>773</v>
       </c>
@@ -7988,7 +7984,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -7996,7 +7992,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -8004,7 +8000,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>778</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -8012,7 +8008,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="12" t="s">
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -8020,7 +8016,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="12" t="s">
         <v>781</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -8028,7 +8024,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="12" t="s">
         <v>783</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -8036,7 +8032,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="12" t="s">
         <v>785</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -8044,7 +8040,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="12" t="s">
         <v>787</v>
       </c>
       <c r="B9" s="3" t="s">
@@ -8052,7 +8048,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="12" t="s">
         <v>789</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -8060,7 +8056,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="12" t="s">
         <v>791</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -8068,7 +8064,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="12" t="s">
         <v>793</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -8076,7 +8072,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="12" t="s">
         <v>795</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -8084,7 +8080,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
+      <c r="A14" s="12" t="s">
         <v>797</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -8092,7 +8088,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="12" t="s">
         <v>799</v>
       </c>
       <c r="B15" s="3" t="s">
@@ -8100,7 +8096,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
+      <c r="A16" s="12" t="s">
         <v>801</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -8108,7 +8104,7 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
@@ -8116,7 +8112,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="12" t="s">
         <v>804</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -8124,7 +8120,7 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+      <c r="A19" s="12" t="s">
         <v>806</v>
       </c>
       <c r="B19" s="3" t="s">
@@ -8132,7 +8128,7 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
+      <c r="A20" s="12" t="s">
         <v>808</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -8140,7 +8136,7 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="12" t="s">
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">

</xml_diff>

<commit_message>
Bug list: PT-45 cash-short simulation case read a fading notice too late on CI
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1252" uniqueCount="811">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="823">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1702,6 +1702,42 @@
   </si>
   <si>
     <t xml:space="preserve">Khi bỏ một lối vào, vai trò nào chỉ có lối đó? Kiểm quyền (CATALOG_MANAGE của MANAGER) trước khi gỡ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI (run 37322764520, main 0b3e27c)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kiểm thử / Mô phỏng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs case "Handheld: cash short of the total is refused and the order stays unpaid"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GitHub Actions ubuntu-24.04, Chromium bóp CPU 4 lần</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test chập chờn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI đỏ với "no message" ở case tiền mặt thiếu, trong khi cùng commit xanh trên nhánh online-v1.7 và chạy ở máy; app vẫn từ chối và đơn vẫn UNPAID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case đọc màn hình sau khi click xong để tìm "chưa đủ", nhưng thông báo tự tắt sau 7 giây. Trên runner tải nặng, click cùng hộp nhập số tiền có thể kéo dài quá thời gian đó nên test thấy màn hình đã sạch. Lỗi ở cách đo, không ở app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case gắn MutationObserver ghi mọi .notice ngay khi hiện, kiểm cả màn hình lẫn danh sách đã ghi; khi hỏng in mã đơn, tổng, các hộp thoại và thông báo đã thấy. Đã kiểm: bỏ thông báo khỏi app thì case vẫn đỏ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs: "Handheld: cash short of the total is refused and the order stays unpaid" (chạy trong job e2e của CI).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test kiểm một thứ tự biến mất (toast, thông báo có hẹn giờ) có đang đọc nó sau một thao tác dài không? Ghi lại lúc nó xuất hiện, đừng đọc sau.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">93f63ab</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-01</t>
@@ -3028,7 +3064,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3073,15 +3109,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3207,8 +3247,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O77" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O77"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O78"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3471,7 +3511,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:O78"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -5606,59 +5646,59 @@
         <v>37</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>476</v>
       </c>
       <c r="B46" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C46" s="6" t="s">
         <v>477</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="D46" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="E46" s="6" t="s">
         <v>479</v>
       </c>
-      <c r="E46" s="6" t="s">
+      <c r="F46" s="6" t="s">
         <v>480</v>
       </c>
-      <c r="F46" s="6" t="s">
+      <c r="G46" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H46" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="G46" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H46" s="6" t="s">
+      <c r="I46" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="I46" s="6" t="s">
+      <c r="J46" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="J46" s="6" t="s">
+      <c r="K46" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="K46" s="6" t="s">
+      <c r="L46" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="L46" s="6" t="s">
+      <c r="M46" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="M46" s="6" t="s">
+      <c r="N46" s="6" t="s">
         <v>487</v>
-      </c>
-      <c r="N46" s="6" t="s">
-        <v>488</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>489</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>477</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>490</v>
@@ -5672,76 +5712,76 @@
       <c r="F47" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="G47" s="7" t="s">
-        <v>29</v>
+      <c r="G47" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="L47" s="6" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="M47" s="6" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="N47" s="6" t="s">
-        <v>488</v>
+        <v>500</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D48" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="F48" s="6" t="s">
+        <v>505</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H48" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="M48" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="N48" s="6" t="s">
         <v>500</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>501</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="G48" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>482</v>
-      </c>
-      <c r="I48" s="6" t="s">
-        <v>503</v>
-      </c>
-      <c r="J48" s="6" t="s">
-        <v>504</v>
-      </c>
-      <c r="K48" s="6" t="s">
-        <v>505</v>
-      </c>
-      <c r="L48" s="6" t="s">
-        <v>506</v>
-      </c>
-      <c r="M48" s="6" t="s">
-        <v>507</v>
-      </c>
-      <c r="N48" s="6" t="s">
-        <v>508</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
@@ -5749,140 +5789,140 @@
     </row>
     <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>146</v>
+        <v>512</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="G49" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>512</v>
+        <v>494</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>520</v>
+        <v>146</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>511</v>
+        <v>523</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H50" s="6" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="J50" s="6" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="K50" s="6" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="L50" s="6" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="M50" s="6" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="F51" s="6" t="s">
+        <v>523</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="I51" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="J51" s="6" t="s">
+        <v>535</v>
+      </c>
+      <c r="K51" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="L51" s="6" t="s">
+        <v>537</v>
+      </c>
+      <c r="M51" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="N51" s="6" t="s">
         <v>530</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>512</v>
-      </c>
-      <c r="I51" s="6" t="s">
-        <v>531</v>
-      </c>
-      <c r="J51" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="K51" s="6" t="s">
-        <v>533</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>534</v>
-      </c>
-      <c r="M51" s="6" t="s">
-        <v>535</v>
-      </c>
-      <c r="N51" s="6" t="s">
-        <v>518</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
@@ -5890,398 +5930,398 @@
     </row>
     <row r="52" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>80</v>
+        <v>540</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>52</v>
+        <v>542</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>538</v>
+        <v>543</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>539</v>
+        <v>544</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>540</v>
+        <v>545</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>542</v>
+        <v>547</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>518</v>
+        <v>530</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>543</v>
+        <v>548</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>544</v>
+        <v>80</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="G53" s="9" t="s">
-        <v>73</v>
+        <v>523</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>372</v>
+        <v>524</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="M53" s="6" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>552</v>
+        <v>530</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>557</v>
+        <v>372</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="M54" s="6" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>53</v>
+        <v>569</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>572</v>
+        <v>564</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>564</v>
+        <v>576</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>29</v>
+        <v>578</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>572</v>
+        <v>584</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>580</v>
+        <v>585</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>581</v>
+        <v>576</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>583</v>
-      </c>
-      <c r="G57" s="9" t="s">
-        <v>73</v>
+        <v>28</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>482</v>
+        <v>30</v>
       </c>
       <c r="I57" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="J57" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="L57" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="M57" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="N57" s="6" t="s">
         <v>584</v>
-      </c>
-      <c r="J57" s="6" t="s">
-        <v>585</v>
-      </c>
-      <c r="K57" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="L57" s="6" t="s">
-        <v>587</v>
-      </c>
-      <c r="M57" s="6" t="s">
-        <v>588</v>
-      </c>
-      <c r="N57" s="6" t="s">
-        <v>552</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>593</v>
+        <v>494</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>599</v>
+        <v>564</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>338</v>
+        <v>602</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G59" s="8" t="s">
-        <v>52</v>
+        <v>604</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>149</v>
+        <v>605</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="M59" s="6" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>478</v>
+        <v>502</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>610</v>
+        <v>211</v>
       </c>
       <c r="G60" s="8" t="s">
         <v>52</v>
@@ -6290,69 +6330,69 @@
         <v>149</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>570</v>
+        <v>617</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>490</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>307</v>
+        <v>621</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>617</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>73</v>
+        <v>622</v>
+      </c>
+      <c r="G61" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>618</v>
+        <v>623</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>619</v>
+        <v>624</v>
       </c>
       <c r="K61" s="6" t="s">
-        <v>620</v>
+        <v>625</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>621</v>
+        <v>582</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
@@ -6360,328 +6400,328 @@
     </row>
     <row r="62" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>435</v>
+        <v>306</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>625</v>
+        <v>307</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>626</v>
-      </c>
-      <c r="G62" s="8" t="s">
-        <v>52</v>
+        <v>629</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>361</v>
+        <v>309</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="K62" s="6" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>634</v>
+        <v>435</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="G63" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>512</v>
+        <v>361</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="K63" s="6" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="M63" s="6" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>632</v>
+        <v>644</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="E64" s="6" t="s">
+        <v>647</v>
+      </c>
+      <c r="F64" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="I64" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="J64" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="K64" s="6" t="s">
+        <v>651</v>
+      </c>
+      <c r="L64" s="6" t="s">
+        <v>652</v>
+      </c>
+      <c r="M64" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="N64" s="6" t="s">
         <v>644</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>645</v>
-      </c>
-      <c r="G64" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>646</v>
-      </c>
-      <c r="I64" s="6" t="s">
-        <v>647</v>
-      </c>
-      <c r="J64" s="6" t="s">
-        <v>648</v>
-      </c>
-      <c r="K64" s="6" t="s">
-        <v>649</v>
-      </c>
-      <c r="L64" s="6" t="s">
-        <v>650</v>
-      </c>
-      <c r="M64" s="6" t="s">
-        <v>651</v>
-      </c>
-      <c r="N64" s="6" t="s">
-        <v>652</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="G65" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>667</v>
-      </c>
-      <c r="G66" s="8" t="s">
-        <v>52</v>
+        <v>668</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="M66" s="6" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>678</v>
-      </c>
-      <c r="G67" s="9" t="s">
-        <v>73</v>
+        <v>679</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>668</v>
+        <v>680</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="M67" s="6" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>663</v>
+        <v>686</v>
       </c>
       <c r="O67" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>295</v>
+        <v>688</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>296</v>
+        <v>689</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G68" s="7" t="s">
-        <v>29</v>
+        <v>690</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>298</v>
+        <v>680</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>299</v>
+        <v>691</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>300</v>
+        <v>692</v>
       </c>
       <c r="K68" s="6" t="s">
-        <v>685</v>
+        <v>693</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>686</v>
+        <v>694</v>
       </c>
       <c r="M68" s="6" t="s">
-        <v>687</v>
+        <v>695</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>663</v>
+        <v>675</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
@@ -6689,375 +6729,375 @@
     </row>
     <row r="69" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>688</v>
+        <v>696</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>689</v>
+        <v>295</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>690</v>
+        <v>296</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>691</v>
+        <v>297</v>
       </c>
       <c r="G69" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>668</v>
+        <v>298</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>692</v>
+        <v>299</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>693</v>
+        <v>300</v>
       </c>
       <c r="K69" s="6" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>697</v>
+        <v>675</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>435</v>
+        <v>701</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>625</v>
+        <v>702</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="G70" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>361</v>
+        <v>680</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="K70" s="6" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="M70" s="6" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>689</v>
+        <v>435</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>707</v>
+        <v>637</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>668</v>
+        <v>361</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="O71" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>490</v>
+        <v>502</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>716</v>
+        <v>701</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>718</v>
-      </c>
-      <c r="G72" s="8" t="s">
-        <v>52</v>
+        <v>720</v>
+      </c>
+      <c r="G72" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>719</v>
+        <v>680</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="K72" s="6" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>25</v>
+        <v>502</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>255</v>
+        <v>731</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="K73" s="6" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="M73" s="6" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>725</v>
+        <v>737</v>
       </c>
       <c r="O73" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C74" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="E74" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="G74" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H74" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I74" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="J74" s="6" t="s">
+        <v>743</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>744</v>
+      </c>
+      <c r="L74" s="6" t="s">
+        <v>745</v>
+      </c>
+      <c r="M74" s="6" t="s">
+        <v>746</v>
+      </c>
+      <c r="N74" s="6" t="s">
         <v>737</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>738</v>
-      </c>
-      <c r="G74" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="I74" s="6" t="s">
-        <v>739</v>
-      </c>
-      <c r="J74" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="K74" s="6" t="s">
-        <v>740</v>
-      </c>
-      <c r="L74" s="6" t="s">
-        <v>741</v>
-      </c>
-      <c r="M74" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="N74" s="6" t="s">
-        <v>725</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>742</v>
+        <v>747</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>490</v>
+        <v>25</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>743</v>
+        <v>748</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>744</v>
+        <v>749</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>745</v>
-      </c>
-      <c r="G75" s="7" t="s">
-        <v>29</v>
+        <v>750</v>
+      </c>
+      <c r="G75" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>746</v>
+        <v>751</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>747</v>
+        <v>268</v>
       </c>
       <c r="K75" s="6" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="M75" s="6" t="s">
-        <v>750</v>
+        <v>271</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>725</v>
+        <v>737</v>
       </c>
       <c r="O75" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>25</v>
+        <v>502</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>754</v>
-      </c>
-      <c r="G76" s="8" t="s">
-        <v>52</v>
+        <v>757</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="K76" s="6" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="M76" s="6" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>760</v>
+        <v>737</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>37</v>
@@ -7065,48 +7105,95 @@
     </row>
     <row r="77" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>477</v>
+        <v>489</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D77" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="J77" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="K77" s="6" t="s">
+        <v>769</v>
+      </c>
+      <c r="L77" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="M77" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="N77" s="6" t="s">
+        <v>772</v>
+      </c>
+      <c r="O77" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="5" t="s">
+        <v>773</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E77" s="6" t="s">
-        <v>762</v>
-      </c>
-      <c r="F77" s="6" t="s">
-        <v>763</v>
-      </c>
-      <c r="G77" s="7" t="s">
+      <c r="E78" s="6" t="s">
+        <v>774</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>775</v>
+      </c>
+      <c r="G78" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H77" s="6" t="s">
+      <c r="H78" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I77" s="6" t="s">
-        <v>764</v>
-      </c>
-      <c r="J77" s="6" t="s">
-        <v>765</v>
-      </c>
-      <c r="K77" s="6" t="s">
-        <v>766</v>
-      </c>
-      <c r="L77" s="6" t="s">
-        <v>767</v>
-      </c>
-      <c r="M77" s="6" t="s">
-        <v>768</v>
-      </c>
-      <c r="N77" s="6" t="s">
-        <v>760</v>
-      </c>
-      <c r="O77" s="6" t="s">
+      <c r="I78" s="6" t="s">
+        <v>776</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>777</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="L78" s="6" t="s">
+        <v>779</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>780</v>
+      </c>
+      <c r="N78" s="6" t="s">
+        <v>772</v>
+      </c>
+      <c r="O78" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7143,7 +7230,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -7164,7 +7251,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>769</v>
+        <v>781</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7211,7 +7298,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>512</v>
+        <v>524</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -7232,7 +7319,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>557</v>
+        <v>569</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -7253,7 +7340,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>646</v>
+        <v>658</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -7337,7 +7424,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>482</v>
+        <v>494</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7400,7 +7487,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>719</v>
+        <v>731</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7463,7 +7550,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>657</v>
+        <v>669</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
@@ -7589,7 +7676,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>668</v>
+        <v>680</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -7778,7 +7865,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>593</v>
+        <v>605</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Cao")</f>
@@ -7799,7 +7886,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>222</v>
+        <v>481</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
@@ -7807,11 +7894,11 @@
       </c>
       <c r="C32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">SUM(B32:D32)</f>
@@ -7820,15 +7907,15 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Thấp")</f>
@@ -7841,7 +7928,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Cao")</f>
@@ -7849,7 +7936,7 @@
       </c>
       <c r="C34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Thấp")</f>
@@ -7857,16 +7944,16 @@
       </c>
       <c r="E34" s="12" t="n">
         <f aca="false">SUM(B34:D34)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>276</v>
+        <v>160</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Trung")</f>
@@ -7878,78 +7965,100 @@
       </c>
       <c r="E35" s="12" t="n">
         <f aca="false">SUM(B35:D35)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B36" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="s">
-        <v>769</v>
-      </c>
-      <c r="B36" s="12" t="n">
-        <f aca="false">SUM(B2:B35)</f>
+      <c r="D36" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <f aca="false">SUM(B36:D36)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
+        <v>781</v>
+      </c>
+      <c r="B37" s="12" t="n">
+        <f aca="false">SUM(B2:B36)</f>
         <v>24</v>
       </c>
-      <c r="C36" s="12" t="n">
-        <f aca="false">SUM(C2:C35)</f>
+      <c r="C37" s="12" t="n">
+        <f aca="false">SUM(C2:C36)</f>
         <v>33</v>
       </c>
-      <c r="D36" s="12" t="n">
-        <f aca="false">SUM(D2:D35)</f>
-        <v>19</v>
-      </c>
-      <c r="E36" s="12" t="n">
-        <f aca="false">SUM(E2:E35)</f>
-        <v>76</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
+      <c r="D37" s="12" t="n">
+        <f aca="false">SUM(D2:D36)</f>
+        <v>20</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <f aca="false">SUM(E2:E36)</f>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="12" t="s">
-        <v>770</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
-        <v>771</v>
-      </c>
-      <c r="B39" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A39)</f>
-        <v>0</v>
+      <c r="B39" s="12" t="s">
+        <v>782</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>444</v>
+        <v>783</v>
       </c>
       <c r="B40" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A40)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
       <c r="B41" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A41)</f>
-        <v>74</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>772</v>
+        <v>37</v>
       </c>
       <c r="B42" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A42)</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="11" t="s">
+        <v>784</v>
+      </c>
+      <c r="B43" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="s">
-        <v>773</v>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="13" t="s">
+        <v>785</v>
       </c>
     </row>
   </sheetData>
@@ -7977,170 +8086,170 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>774</v>
+        <v>786</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>775</v>
+        <v>787</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>776</v>
+        <v>788</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>777</v>
+        <v>789</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>778</v>
+      <c r="A4" s="14" t="s">
+        <v>790</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>779</v>
+        <v>791</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>780</v>
+        <v>792</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>781</v>
+      <c r="A6" s="14" t="s">
+        <v>793</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>782</v>
+        <v>794</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>783</v>
+      <c r="A7" s="14" t="s">
+        <v>795</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>784</v>
+        <v>796</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>785</v>
+      <c r="A8" s="14" t="s">
+        <v>797</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>786</v>
+        <v>798</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>787</v>
+      <c r="A9" s="14" t="s">
+        <v>799</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>788</v>
+        <v>800</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>789</v>
+      <c r="A10" s="14" t="s">
+        <v>801</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>790</v>
+        <v>802</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>791</v>
+      <c r="A11" s="14" t="s">
+        <v>803</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>792</v>
+        <v>804</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>793</v>
+      <c r="A12" s="14" t="s">
+        <v>805</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>794</v>
+        <v>806</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>795</v>
+      <c r="A13" s="14" t="s">
+        <v>807</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>796</v>
+        <v>808</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>797</v>
+      <c r="A14" s="14" t="s">
+        <v>809</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>798</v>
+        <v>810</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>799</v>
+      <c r="A15" s="14" t="s">
+        <v>811</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>800</v>
+        <v>812</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>801</v>
+      <c r="A16" s="14" t="s">
+        <v>813</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>802</v>
+        <v>814</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>803</v>
+        <v>815</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>804</v>
+      <c r="A18" s="14" t="s">
+        <v>816</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>805</v>
+        <v>817</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>806</v>
+      <c r="A19" s="14" t="s">
+        <v>818</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>807</v>
+        <v>819</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
-        <v>808</v>
+      <c r="A20" s="14" t="s">
+        <v>820</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>809</v>
+        <v>821</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="14" t="s">
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>810</v>
+        <v>822</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-46 cash-payment simulation case read the print queue before the receipt was sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1268" uniqueCount="823">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="832">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1738,6 +1738,33 @@
   </si>
   <si>
     <t xml:space="preserve">93f63ab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI (run 37324875053, main 8627bf7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs case "Handheld: pay cash with change; the receipt goes to the SUNMI printer…"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI đỏ với "no receipt printed" sau khi thu tiền mặt, trong khi cùng commit xanh trên nhánh; app vẫn in biên lai.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case coi mã đơn "-TM" hiện trên màn hình là dấu hiệu đã in xong, rồi đọc ngay hàng đợi in. Nhưng đồng bộ trực tiếp có thể vẽ mã đã trả trước khi callback thanh toán gửi biên lai sang máy in (printReceipt chạy sau). Lỗi ở cách đo, không ở app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Case ghi số lệnh in trước khi bấm thanh toán, rồi chờ có lệnh in mới (tối đa 15 s) trước khi đọc. Đã kiểm: bỏ lệnh in khỏi app thì case đỏ. Toàn bộ 105 case xanh khi bóp CPU 6 lần.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs: "Handheld: pay cash with change; the receipt goes to the SUNMI printer as \"BIÊN LAI THU TIỀN\" naming the cashier".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dấu hiệu test đang chờ có thật sự đến sau việc cần kiểm không, hay một đường khác (đồng bộ, realtime) cũng tạo ra nó? Chờ chính kết quả cần kiểm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09b0980</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-01</t>
@@ -3247,8 +3274,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O78"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O79"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3511,7 +3538,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O78"/>
+  <dimension ref="A1:O79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -5646,7 +5673,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>476</v>
       </c>
@@ -5693,109 +5720,109 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
         <v>488</v>
       </c>
       <c r="B47" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="D47" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="E47" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="F47" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H47" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="I47" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="J47" s="6" t="s">
         <v>492</v>
       </c>
-      <c r="F47" s="6" t="s">
+      <c r="K47" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="G47" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H47" s="6" t="s">
+      <c r="L47" s="6" t="s">
         <v>494</v>
       </c>
-      <c r="I47" s="6" t="s">
+      <c r="M47" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="J47" s="6" t="s">
+      <c r="N47" s="6" t="s">
         <v>496</v>
-      </c>
-      <c r="K47" s="6" t="s">
-        <v>497</v>
-      </c>
-      <c r="L47" s="6" t="s">
-        <v>498</v>
-      </c>
-      <c r="M47" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="N47" s="6" t="s">
-        <v>500</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C48" s="6" t="s">
+      <c r="F48" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="G48" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="E48" s="6" t="s">
+      <c r="I48" s="6" t="s">
         <v>504</v>
       </c>
-      <c r="F48" s="6" t="s">
+      <c r="J48" s="6" t="s">
         <v>505</v>
       </c>
-      <c r="G48" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="I48" s="6" t="s">
+      <c r="K48" s="6" t="s">
         <v>506</v>
       </c>
-      <c r="J48" s="6" t="s">
+      <c r="L48" s="6" t="s">
         <v>507</v>
       </c>
-      <c r="K48" s="6" t="s">
+      <c r="M48" s="6" t="s">
         <v>508</v>
       </c>
-      <c r="L48" s="6" t="s">
+      <c r="N48" s="6" t="s">
         <v>509</v>
-      </c>
-      <c r="M48" s="6" t="s">
-        <v>510</v>
-      </c>
-      <c r="N48" s="6" t="s">
-        <v>500</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C49" s="6" t="s">
         <v>511</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>502</v>
       </c>
       <c r="D49" s="6" t="s">
         <v>512</v>
@@ -5806,11 +5833,11 @@
       <c r="F49" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="G49" s="8" t="s">
-        <v>52</v>
+      <c r="G49" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="I49" s="6" t="s">
         <v>515</v>
@@ -5828,7 +5855,7 @@
         <v>519</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
@@ -5836,16 +5863,16 @@
     </row>
     <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D50" s="6" t="s">
         <v>521</v>
-      </c>
-      <c r="B50" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>522</v>
@@ -5857,54 +5884,54 @@
         <v>52</v>
       </c>
       <c r="H50" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="I50" s="6" t="s">
         <v>524</v>
       </c>
-      <c r="I50" s="6" t="s">
+      <c r="J50" s="6" t="s">
         <v>525</v>
       </c>
-      <c r="J50" s="6" t="s">
+      <c r="K50" s="6" t="s">
         <v>526</v>
       </c>
-      <c r="K50" s="6" t="s">
+      <c r="L50" s="6" t="s">
         <v>527</v>
       </c>
-      <c r="L50" s="6" t="s">
+      <c r="M50" s="6" t="s">
         <v>528</v>
       </c>
-      <c r="M50" s="6" t="s">
+      <c r="N50" s="6" t="s">
         <v>529</v>
-      </c>
-      <c r="N50" s="6" t="s">
-        <v>530</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
+        <v>530</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E51" s="6" t="s">
         <v>531</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D51" s="6" t="s">
+      <c r="F51" s="6" t="s">
         <v>532</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>533</v>
-      </c>
-      <c r="F51" s="6" t="s">
-        <v>523</v>
       </c>
       <c r="G51" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="I51" s="6" t="s">
         <v>534</v>
@@ -5922,36 +5949,36 @@
         <v>538</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>542</v>
-      </c>
-      <c r="G52" s="7" t="s">
-        <v>29</v>
+        <v>532</v>
+      </c>
+      <c r="G52" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="I52" s="6" t="s">
         <v>543</v>
@@ -5969,7 +5996,7 @@
         <v>547</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
@@ -5980,72 +6007,72 @@
         <v>548</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>80</v>
+        <v>549</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>523</v>
-      </c>
-      <c r="G53" s="8" t="s">
-        <v>52</v>
+        <v>551</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="M53" s="6" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>530</v>
+        <v>539</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>556</v>
+        <v>80</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>558</v>
-      </c>
-      <c r="G54" s="9" t="s">
-        <v>73</v>
+        <v>532</v>
+      </c>
+      <c r="G54" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>372</v>
+        <v>533</v>
       </c>
       <c r="I54" s="6" t="s">
         <v>559</v>
@@ -6063,83 +6090,83 @@
         <v>563</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>564</v>
+        <v>539</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
+        <v>564</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D55" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D55" s="6" t="s">
+      <c r="E55" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="E55" s="6" t="s">
+      <c r="F55" s="6" t="s">
         <v>567</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>568</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H55" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="J55" s="6" t="s">
         <v>569</v>
       </c>
-      <c r="I55" s="6" t="s">
+      <c r="K55" s="6" t="s">
         <v>570</v>
       </c>
-      <c r="J55" s="6" t="s">
+      <c r="L55" s="6" t="s">
         <v>571</v>
       </c>
-      <c r="K55" s="6" t="s">
+      <c r="M55" s="6" t="s">
         <v>572</v>
       </c>
-      <c r="L55" s="6" t="s">
+      <c r="N55" s="6" t="s">
         <v>573</v>
-      </c>
-      <c r="M55" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="N55" s="6" t="s">
-        <v>564</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
+        <v>574</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D56" s="6" t="s">
         <v>575</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D56" s="6" t="s">
+      <c r="E56" s="6" t="s">
         <v>576</v>
       </c>
-      <c r="E56" s="6" t="s">
+      <c r="F56" s="6" t="s">
         <v>577</v>
-      </c>
-      <c r="F56" s="6" t="s">
-        <v>578</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>53</v>
+        <v>578</v>
       </c>
       <c r="I56" s="6" t="s">
         <v>579</v>
@@ -6157,83 +6184,83 @@
         <v>583</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>584</v>
+        <v>573</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
+        <v>584</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D57" s="6" t="s">
         <v>585</v>
-      </c>
-      <c r="B57" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>576</v>
       </c>
       <c r="E57" s="6" t="s">
         <v>586</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G57" s="7" t="s">
-        <v>29</v>
+        <v>587</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>584</v>
+        <v>593</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>593</v>
+        <v>585</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="G58" s="9" t="s">
-        <v>73</v>
+        <v>28</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>494</v>
+        <v>30</v>
       </c>
       <c r="I58" s="6" t="s">
         <v>596</v>
@@ -6251,21 +6278,21 @@
         <v>600</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>564</v>
+        <v>593</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
         <v>601</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D59" s="6" t="s">
         <v>602</v>
@@ -6280,95 +6307,95 @@
         <v>73</v>
       </c>
       <c r="H59" s="6" t="s">
+        <v>503</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>605</v>
       </c>
-      <c r="I59" s="6" t="s">
+      <c r="J59" s="6" t="s">
         <v>606</v>
       </c>
-      <c r="J59" s="6" t="s">
+      <c r="K59" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="K59" s="6" t="s">
+      <c r="L59" s="6" t="s">
         <v>608</v>
       </c>
-      <c r="L59" s="6" t="s">
+      <c r="M59" s="6" t="s">
         <v>609</v>
       </c>
-      <c r="M59" s="6" t="s">
-        <v>610</v>
-      </c>
       <c r="N59" s="6" t="s">
-        <v>611</v>
+        <v>573</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>612</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D60" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="E60" s="6" t="s">
+      <c r="F60" s="6" t="s">
         <v>613</v>
       </c>
-      <c r="F60" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G60" s="8" t="s">
-        <v>52</v>
+      <c r="G60" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>149</v>
+        <v>614</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>490</v>
+        <v>511</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>622</v>
+        <v>211</v>
       </c>
       <c r="G61" s="8" t="s">
         <v>52</v>
@@ -6386,60 +6413,60 @@
         <v>625</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>582</v>
+        <v>626</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>502</v>
+        <v>499</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>307</v>
+        <v>630</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>629</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>73</v>
+        <v>631</v>
+      </c>
+      <c r="G62" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="K62" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>633</v>
+        <v>591</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
@@ -6447,28 +6474,28 @@
     </row>
     <row r="63" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>435</v>
+        <v>306</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>637</v>
+        <v>307</v>
       </c>
       <c r="F63" s="6" t="s">
         <v>638</v>
       </c>
-      <c r="G63" s="8" t="s">
-        <v>52</v>
+      <c r="G63" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>361</v>
+        <v>309</v>
       </c>
       <c r="I63" s="6" t="s">
         <v>639</v>
@@ -6492,62 +6519,62 @@
         <v>37</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
         <v>645</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D64" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E64" s="6" t="s">
         <v>646</v>
       </c>
-      <c r="E64" s="6" t="s">
+      <c r="F64" s="6" t="s">
         <v>647</v>
-      </c>
-      <c r="F64" s="6" t="s">
-        <v>648</v>
       </c>
       <c r="G64" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>524</v>
+        <v>361</v>
       </c>
       <c r="I64" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="J64" s="6" t="s">
         <v>649</v>
       </c>
-      <c r="J64" s="6" t="s">
+      <c r="K64" s="6" t="s">
         <v>650</v>
       </c>
-      <c r="K64" s="6" t="s">
+      <c r="L64" s="6" t="s">
         <v>651</v>
       </c>
-      <c r="L64" s="6" t="s">
+      <c r="M64" s="6" t="s">
         <v>652</v>
       </c>
-      <c r="M64" s="6" t="s">
+      <c r="N64" s="6" t="s">
         <v>653</v>
-      </c>
-      <c r="N64" s="6" t="s">
-        <v>644</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
         <v>654</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>655</v>
@@ -6558,217 +6585,217 @@
       <c r="F65" s="6" t="s">
         <v>657</v>
       </c>
-      <c r="G65" s="7" t="s">
-        <v>29</v>
+      <c r="G65" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H65" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="I65" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="I65" s="6" t="s">
+      <c r="J65" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="J65" s="6" t="s">
+      <c r="K65" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="K65" s="6" t="s">
+      <c r="L65" s="6" t="s">
         <v>661</v>
       </c>
-      <c r="L65" s="6" t="s">
+      <c r="M65" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="M65" s="6" t="s">
-        <v>663</v>
-      </c>
       <c r="N65" s="6" t="s">
-        <v>664</v>
+        <v>653</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
+        <v>663</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>664</v>
+      </c>
+      <c r="E66" s="6" t="s">
         <v>665</v>
       </c>
-      <c r="B66" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D66" s="6" t="s">
+      <c r="F66" s="6" t="s">
         <v>666</v>
-      </c>
-      <c r="E66" s="6" t="s">
-        <v>667</v>
-      </c>
-      <c r="F66" s="6" t="s">
-        <v>668</v>
       </c>
       <c r="G66" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H66" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="J66" s="6" t="s">
         <v>669</v>
       </c>
-      <c r="I66" s="6" t="s">
+      <c r="K66" s="6" t="s">
         <v>670</v>
       </c>
-      <c r="J66" s="6" t="s">
+      <c r="L66" s="6" t="s">
         <v>671</v>
       </c>
-      <c r="K66" s="6" t="s">
+      <c r="M66" s="6" t="s">
         <v>672</v>
       </c>
-      <c r="L66" s="6" t="s">
+      <c r="N66" s="6" t="s">
         <v>673</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>674</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>675</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
+        <v>674</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="E67" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D67" s="6" t="s">
+      <c r="F67" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="E67" s="6" t="s">
+      <c r="G67" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H67" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="F67" s="6" t="s">
+      <c r="I67" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="G67" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H67" s="6" t="s">
+      <c r="J67" s="6" t="s">
         <v>680</v>
       </c>
-      <c r="I67" s="6" t="s">
+      <c r="K67" s="6" t="s">
         <v>681</v>
       </c>
-      <c r="J67" s="6" t="s">
+      <c r="L67" s="6" t="s">
         <v>682</v>
       </c>
-      <c r="K67" s="6" t="s">
+      <c r="M67" s="6" t="s">
         <v>683</v>
       </c>
-      <c r="L67" s="6" t="s">
+      <c r="N67" s="6" t="s">
         <v>684</v>
-      </c>
-      <c r="M67" s="6" t="s">
-        <v>685</v>
-      </c>
-      <c r="N67" s="6" t="s">
-        <v>686</v>
       </c>
       <c r="O67" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
+        <v>685</v>
+      </c>
+      <c r="B68" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="E68" s="6" t="s">
         <v>687</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D68" s="6" t="s">
+      <c r="F68" s="6" t="s">
         <v>688</v>
       </c>
-      <c r="E68" s="6" t="s">
+      <c r="G68" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H68" s="6" t="s">
         <v>689</v>
       </c>
-      <c r="F68" s="6" t="s">
+      <c r="I68" s="6" t="s">
         <v>690</v>
       </c>
-      <c r="G68" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>680</v>
-      </c>
-      <c r="I68" s="6" t="s">
+      <c r="J68" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="J68" s="6" t="s">
+      <c r="K68" s="6" t="s">
         <v>692</v>
       </c>
-      <c r="K68" s="6" t="s">
+      <c r="L68" s="6" t="s">
         <v>693</v>
       </c>
-      <c r="L68" s="6" t="s">
+      <c r="M68" s="6" t="s">
         <v>694</v>
       </c>
-      <c r="M68" s="6" t="s">
+      <c r="N68" s="6" t="s">
         <v>695</v>
-      </c>
-      <c r="N68" s="6" t="s">
-        <v>675</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
         <v>696</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>295</v>
+        <v>697</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>296</v>
+        <v>698</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G69" s="7" t="s">
-        <v>29</v>
+        <v>699</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>298</v>
+        <v>689</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>299</v>
+        <v>700</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>300</v>
+        <v>701</v>
       </c>
       <c r="K69" s="6" t="s">
-        <v>697</v>
+        <v>702</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>698</v>
+        <v>703</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>699</v>
+        <v>704</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>675</v>
+        <v>684</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
@@ -6776,34 +6803,34 @@
     </row>
     <row r="70" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>701</v>
+        <v>295</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>702</v>
+        <v>296</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>703</v>
+        <v>297</v>
       </c>
       <c r="G70" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>680</v>
+        <v>298</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>704</v>
+        <v>299</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>705</v>
+        <v>300</v>
       </c>
       <c r="K70" s="6" t="s">
         <v>706</v>
@@ -6815,74 +6842,74 @@
         <v>708</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>709</v>
+        <v>684</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D71" s="6" t="s">
         <v>710</v>
       </c>
-      <c r="B71" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>502</v>
-      </c>
-      <c r="D71" s="6" t="s">
-        <v>435</v>
-      </c>
       <c r="E71" s="6" t="s">
-        <v>637</v>
+        <v>711</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>361</v>
+        <v>689</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="O71" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>701</v>
+        <v>435</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>719</v>
+        <v>646</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>720</v>
@@ -6891,7 +6918,7 @@
         <v>29</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>680</v>
+        <v>361</v>
       </c>
       <c r="I72" s="6" t="s">
         <v>721</v>
@@ -6912,109 +6939,109 @@
         <v>726</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
         <v>727</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>502</v>
+        <v>511</v>
       </c>
       <c r="D73" s="6" t="s">
+        <v>710</v>
+      </c>
+      <c r="E73" s="6" t="s">
         <v>728</v>
       </c>
-      <c r="E73" s="6" t="s">
+      <c r="F73" s="6" t="s">
         <v>729</v>
       </c>
-      <c r="F73" s="6" t="s">
+      <c r="G73" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H73" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="I73" s="6" t="s">
         <v>730</v>
       </c>
-      <c r="G73" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H73" s="6" t="s">
+      <c r="J73" s="6" t="s">
         <v>731</v>
       </c>
-      <c r="I73" s="6" t="s">
+      <c r="K73" s="6" t="s">
         <v>732</v>
       </c>
-      <c r="J73" s="6" t="s">
+      <c r="L73" s="6" t="s">
         <v>733</v>
       </c>
-      <c r="K73" s="6" t="s">
+      <c r="M73" s="6" t="s">
         <v>734</v>
       </c>
-      <c r="L73" s="6" t="s">
+      <c r="N73" s="6" t="s">
         <v>735</v>
-      </c>
-      <c r="M73" s="6" t="s">
-        <v>736</v>
-      </c>
-      <c r="N73" s="6" t="s">
-        <v>737</v>
       </c>
       <c r="O73" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
+        <v>736</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>737</v>
+      </c>
+      <c r="E74" s="6" t="s">
         <v>738</v>
       </c>
-      <c r="B74" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D74" s="6" t="s">
+      <c r="F74" s="6" t="s">
         <v>739</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>740</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>741</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>255</v>
+        <v>740</v>
       </c>
       <c r="I74" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="J74" s="6" t="s">
         <v>742</v>
       </c>
-      <c r="J74" s="6" t="s">
+      <c r="K74" s="6" t="s">
         <v>743</v>
       </c>
-      <c r="K74" s="6" t="s">
+      <c r="L74" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="L74" s="6" t="s">
+      <c r="M74" s="6" t="s">
         <v>745</v>
       </c>
-      <c r="M74" s="6" t="s">
+      <c r="N74" s="6" t="s">
         <v>746</v>
-      </c>
-      <c r="N74" s="6" t="s">
-        <v>737</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
         <v>747</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C75" s="6" t="s">
         <v>25</v>
@@ -7028,90 +7055,90 @@
       <c r="F75" s="6" t="s">
         <v>750</v>
       </c>
-      <c r="G75" s="9" t="s">
-        <v>73</v>
+      <c r="G75" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="I75" s="6" t="s">
         <v>751</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>268</v>
+        <v>752</v>
       </c>
       <c r="K75" s="6" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="M75" s="6" t="s">
-        <v>271</v>
+        <v>755</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>737</v>
+        <v>746</v>
       </c>
       <c r="O75" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>502</v>
+        <v>25</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>757</v>
-      </c>
-      <c r="G76" s="7" t="s">
-        <v>29</v>
+        <v>759</v>
+      </c>
+      <c r="G76" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I76" s="6" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="J76" s="6" t="s">
-        <v>759</v>
+        <v>268</v>
       </c>
       <c r="K76" s="6" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="L76" s="6" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
       <c r="M76" s="6" t="s">
-        <v>762</v>
+        <v>271</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>737</v>
+        <v>746</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
         <v>763</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>25</v>
+        <v>511</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>764</v>
@@ -7122,11 +7149,11 @@
       <c r="F77" s="6" t="s">
         <v>766</v>
       </c>
-      <c r="G77" s="8" t="s">
-        <v>52</v>
+      <c r="G77" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="I77" s="6" t="s">
         <v>767</v>
@@ -7144,7 +7171,7 @@
         <v>771</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>772</v>
+        <v>746</v>
       </c>
       <c r="O77" s="6" t="s">
         <v>37</v>
@@ -7152,16 +7179,16 @@
     </row>
     <row r="78" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>489</v>
+        <v>498</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>317</v>
+        <v>773</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>774</v>
@@ -7169,11 +7196,11 @@
       <c r="F78" s="6" t="s">
         <v>775</v>
       </c>
-      <c r="G78" s="7" t="s">
-        <v>29</v>
+      <c r="G78" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>320</v>
+        <v>330</v>
       </c>
       <c r="I78" s="6" t="s">
         <v>776</v>
@@ -7191,9 +7218,56 @@
         <v>780</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>772</v>
+        <v>781</v>
       </c>
       <c r="O78" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A79" s="5" t="s">
+        <v>782</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>783</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>784</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>785</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>787</v>
+      </c>
+      <c r="L79" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="M79" s="6" t="s">
+        <v>789</v>
+      </c>
+      <c r="N79" s="6" t="s">
+        <v>781</v>
+      </c>
+      <c r="O79" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7251,7 +7325,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>781</v>
+        <v>790</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7298,7 +7372,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>524</v>
+        <v>533</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -7319,7 +7393,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -7340,7 +7414,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>658</v>
+        <v>667</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -7424,7 +7498,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>494</v>
+        <v>503</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7487,7 +7561,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>731</v>
+        <v>740</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7550,7 +7624,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>669</v>
+        <v>678</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
@@ -7676,7 +7750,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>680</v>
+        <v>689</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -7865,7 +7939,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>605</v>
+        <v>614</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Cao")</f>
@@ -7898,11 +7972,11 @@
       </c>
       <c r="D32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">SUM(B32:D32)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7991,7 +8065,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>781</v>
+        <v>790</v>
       </c>
       <c r="B37" s="12" t="n">
         <f aca="false">SUM(B2:B36)</f>
@@ -8003,11 +8077,11 @@
       </c>
       <c r="D37" s="12" t="n">
         <f aca="false">SUM(D2:D36)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E37" s="12" t="n">
         <f aca="false">SUM(E2:E36)</f>
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -8016,12 +8090,12 @@
         <v>22</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>782</v>
+        <v>791</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>783</v>
+        <v>792</v>
       </c>
       <c r="B40" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A40)</f>
@@ -8043,12 +8117,12 @@
       </c>
       <c r="B42" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A42)</f>
-        <v>75</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>784</v>
+        <v>793</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
@@ -8056,9 +8130,9 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="13" t="s">
-        <v>785</v>
+        <v>794</v>
       </c>
     </row>
   </sheetData>
@@ -8086,10 +8160,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>786</v>
+        <v>795</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>787</v>
+        <v>796</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8097,7 +8171,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>788</v>
+        <v>797</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8105,15 +8179,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>789</v>
+        <v>798</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>790</v>
+        <v>799</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>791</v>
+        <v>800</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8121,95 +8195,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>792</v>
+        <v>801</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>793</v>
+        <v>802</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>794</v>
+        <v>803</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>795</v>
+        <v>804</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>796</v>
+        <v>805</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>797</v>
+        <v>806</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>798</v>
+        <v>807</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>799</v>
+        <v>808</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>800</v>
+        <v>809</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>801</v>
+        <v>810</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>802</v>
+        <v>811</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>803</v>
+        <v>812</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>804</v>
+        <v>813</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>805</v>
+        <v>814</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>806</v>
+        <v>815</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>807</v>
+        <v>816</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>808</v>
+        <v>817</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>809</v>
+        <v>818</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>810</v>
+        <v>819</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>811</v>
+        <v>820</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>812</v>
+        <v>821</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>813</v>
+        <v>822</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>814</v>
+        <v>823</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8217,31 +8291,31 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>815</v>
+        <v>824</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>816</v>
+        <v>825</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>817</v>
+        <v>826</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>818</v>
+        <v>827</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>819</v>
+        <v>828</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>820</v>
+        <v>829</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>821</v>
+        <v>830</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8249,7 +8323,7 @@
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>822</v>
+        <v>831</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-47 shift refused on the SUNMI with a message that did not say why
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="832">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="845">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1765,6 +1765,171 @@
   </si>
   <si>
     <t xml:space="preserve">09b0980</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chủ tiệm (ảnh máy SUNMI, APK 1.7.79)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phân ca / Chấm công</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js form xếp ca (input type=time); src/management.js POST /api/staff/schedules/bulk</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SUNMI V2s, WebView Chromium 83, ngôn ngữ tiếng Trung (ô giờ hiện </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上午</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">下午</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Nhập liệu / thông báo lỗi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tạo ca "CA SANG" cho 3 nhân viên trên máy SUNMI báo "Dữ liệu nhập không hợp lệ", không nói sai ô nào; chủ tiệm không tạo được ca.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Server gộp mọi lỗi lịch (giờ ra không sau giờ vào, tên trống, ngày sai, nhân viên bị khóa) vào một mã INVALID_SCHEDULE với câu chung. Cùng thao tác (3 nhân viên, 10:00–14:00) lưu được trên Chromium, nên request từ máy mang một giá trị bị từ chối. Khả năng cao nhất: ô giờ của WebView hiển thị 12 giờ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上午</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">下午</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, chọn "2:00" thành 02:00, trước giờ vào 10:00. Không đọc được request thật trên production để khẳng định.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Giờ vào/ra chọn từ danh sách 24 giờ (05:00–23:30, mỗi 30 phút, kèm "2h chiều"), app kiểm giờ ra sau giờ vào trước khi gửi. Server trả câu nói rõ ô sai: giờ (kèm giá trị), tên ca, ngày, nhân viên bị khóa. Cùng đợt: ca cố định lặp hằng ngày từ ngày bắt đầu (migration 0022).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v183-fixed-shifts.test.mjs: "PT-47 a refused schedule says which field is wrong", "the shift form picks hours from a 24-hour list…"; scripts/sim-browser.mjs: "Handheld: a refused end time before the start is explained, not \"Dữ liệu nhập không hợp lệ\"".</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Ô giờ/ngày gốc của trình duyệt có hiển thị theo ngôn ngữ máy (12h, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">上午</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">下午</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) không, và người dùng có thể chọn nhầm không? Mỗi lỗi nhập trả về có nói đúng ô nào sai không?</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">a7f7a8f</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-01</t>
@@ -3274,8 +3439,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O79"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O80"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3538,7 +3703,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O79"/>
+  <dimension ref="A1:O80"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -5720,7 +5885,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
         <v>488</v>
       </c>
@@ -5767,7 +5932,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
         <v>497</v>
       </c>
@@ -5786,8 +5951,8 @@
       <c r="F48" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="G48" s="8" t="s">
-        <v>52</v>
+      <c r="G48" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H48" s="6" t="s">
         <v>503</v>
@@ -5814,95 +5979,95 @@
         <v>37</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
         <v>510</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="G49" s="7" t="s">
-        <v>29</v>
+        <v>515</v>
+      </c>
+      <c r="G49" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H49" s="6" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="L49" s="6" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="M49" s="6" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="N49" s="6" t="s">
-        <v>509</v>
+        <v>522</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="E50" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>527</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>516</v>
+      </c>
+      <c r="I50" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="K50" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="L50" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="M50" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="N50" s="6" t="s">
         <v>522</v>
-      </c>
-      <c r="F50" s="6" t="s">
-        <v>523</v>
-      </c>
-      <c r="G50" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>503</v>
-      </c>
-      <c r="I50" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>525</v>
-      </c>
-      <c r="K50" s="6" t="s">
-        <v>526</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>527</v>
-      </c>
-      <c r="M50" s="6" t="s">
-        <v>528</v>
-      </c>
-      <c r="N50" s="6" t="s">
-        <v>529</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
@@ -5910,140 +6075,140 @@
     </row>
     <row r="51" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>146</v>
+        <v>534</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="G51" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H51" s="6" t="s">
-        <v>533</v>
+        <v>516</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="J51" s="6" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="K51" s="6" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="L51" s="6" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="M51" s="6" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>541</v>
+        <v>146</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>532</v>
+        <v>545</v>
       </c>
       <c r="G52" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>533</v>
+        <v>546</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="J52" s="6" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="K52" s="6" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="L52" s="6" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="M52" s="6" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>539</v>
+        <v>552</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>549</v>
+        <v>554</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>550</v>
+        <v>555</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>551</v>
-      </c>
-      <c r="G53" s="7" t="s">
-        <v>29</v>
+        <v>545</v>
+      </c>
+      <c r="G53" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>533</v>
+        <v>546</v>
       </c>
       <c r="I53" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>557</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="L53" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="M53" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="N53" s="6" t="s">
         <v>552</v>
-      </c>
-      <c r="J53" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="K53" s="6" t="s">
-        <v>554</v>
-      </c>
-      <c r="L53" s="6" t="s">
-        <v>555</v>
-      </c>
-      <c r="M53" s="6" t="s">
-        <v>556</v>
-      </c>
-      <c r="N53" s="6" t="s">
-        <v>539</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
@@ -6051,398 +6216,398 @@
     </row>
     <row r="54" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>80</v>
+        <v>562</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>558</v>
+        <v>563</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="G54" s="8" t="s">
-        <v>52</v>
+        <v>564</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>533</v>
+        <v>546</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>560</v>
+        <v>566</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>561</v>
+        <v>567</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="M54" s="6" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>539</v>
+        <v>552</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>564</v>
+        <v>570</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>565</v>
+        <v>80</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>567</v>
-      </c>
-      <c r="G55" s="9" t="s">
-        <v>73</v>
+        <v>545</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H55" s="6" t="s">
-        <v>372</v>
+        <v>546</v>
       </c>
       <c r="I55" s="6" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="J55" s="6" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="K55" s="6" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="L55" s="6" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="M55" s="6" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="N55" s="6" t="s">
-        <v>573</v>
+        <v>552</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>578</v>
+        <v>372</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>573</v>
+        <v>586</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>53</v>
+        <v>591</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>593</v>
+        <v>586</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>585</v>
+        <v>598</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G58" s="7" t="s">
-        <v>29</v>
+        <v>600</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>596</v>
+        <v>601</v>
       </c>
       <c r="J58" s="6" t="s">
-        <v>597</v>
+        <v>602</v>
       </c>
       <c r="K58" s="6" t="s">
-        <v>598</v>
+        <v>603</v>
       </c>
       <c r="L58" s="6" t="s">
-        <v>599</v>
+        <v>604</v>
       </c>
       <c r="M58" s="6" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>593</v>
+        <v>606</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>601</v>
+        <v>607</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>603</v>
+        <v>608</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>73</v>
+        <v>28</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>503</v>
+        <v>30</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="J59" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="K59" s="6" t="s">
+        <v>611</v>
+      </c>
+      <c r="L59" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="M59" s="6" t="s">
+        <v>613</v>
+      </c>
+      <c r="N59" s="6" t="s">
         <v>606</v>
-      </c>
-      <c r="K59" s="6" t="s">
-        <v>607</v>
-      </c>
-      <c r="L59" s="6" t="s">
-        <v>608</v>
-      </c>
-      <c r="M59" s="6" t="s">
-        <v>609</v>
-      </c>
-      <c r="N59" s="6" t="s">
-        <v>573</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="G60" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>614</v>
+        <v>516</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>620</v>
+        <v>586</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>338</v>
+        <v>624</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G61" s="8" t="s">
-        <v>52</v>
+        <v>626</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H61" s="6" t="s">
-        <v>149</v>
+        <v>627</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>623</v>
+        <v>628</v>
       </c>
       <c r="J61" s="6" t="s">
-        <v>624</v>
+        <v>629</v>
       </c>
       <c r="K61" s="6" t="s">
-        <v>625</v>
+        <v>630</v>
       </c>
       <c r="L61" s="6" t="s">
-        <v>626</v>
+        <v>631</v>
       </c>
       <c r="M61" s="6" t="s">
-        <v>627</v>
+        <v>632</v>
       </c>
       <c r="N61" s="6" t="s">
-        <v>628</v>
+        <v>633</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>499</v>
+        <v>524</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>630</v>
+        <v>635</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>631</v>
+        <v>211</v>
       </c>
       <c r="G62" s="8" t="s">
         <v>52</v>
@@ -6451,69 +6616,69 @@
         <v>149</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="K62" s="6" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>591</v>
+        <v>639</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>307</v>
+        <v>643</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>638</v>
-      </c>
-      <c r="G63" s="9" t="s">
-        <v>73</v>
+        <v>644</v>
+      </c>
+      <c r="G63" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>639</v>
+        <v>645</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="K63" s="6" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>642</v>
+        <v>604</v>
       </c>
       <c r="M63" s="6" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
@@ -6521,328 +6686,328 @@
     </row>
     <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>435</v>
+        <v>306</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>646</v>
+        <v>307</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>647</v>
-      </c>
-      <c r="G64" s="8" t="s">
-        <v>52</v>
+        <v>651</v>
+      </c>
+      <c r="G64" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>361</v>
+        <v>309</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="M64" s="6" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>655</v>
+        <v>435</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="G65" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>533</v>
+        <v>361</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>653</v>
+        <v>666</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="F66" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H66" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="I66" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>672</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>673</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="M66" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="N66" s="6" t="s">
         <v>666</v>
-      </c>
-      <c r="G66" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H66" s="6" t="s">
-        <v>667</v>
-      </c>
-      <c r="I66" s="6" t="s">
-        <v>668</v>
-      </c>
-      <c r="J66" s="6" t="s">
-        <v>669</v>
-      </c>
-      <c r="K66" s="6" t="s">
-        <v>670</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>671</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>672</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>673</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="G67" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="M67" s="6" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="O67" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>688</v>
-      </c>
-      <c r="G68" s="8" t="s">
-        <v>52</v>
+        <v>690</v>
+      </c>
+      <c r="G68" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="J68" s="6" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="K68" s="6" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="L68" s="6" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="M68" s="6" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="N68" s="6" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>699</v>
-      </c>
-      <c r="G69" s="9" t="s">
-        <v>73</v>
+        <v>701</v>
+      </c>
+      <c r="G69" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H69" s="6" t="s">
-        <v>689</v>
+        <v>702</v>
       </c>
       <c r="I69" s="6" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="J69" s="6" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="K69" s="6" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="L69" s="6" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="M69" s="6" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="N69" s="6" t="s">
-        <v>684</v>
+        <v>708</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>295</v>
+        <v>710</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>296</v>
+        <v>711</v>
       </c>
       <c r="F70" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G70" s="7" t="s">
-        <v>29</v>
+        <v>712</v>
+      </c>
+      <c r="G70" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>298</v>
+        <v>702</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>299</v>
+        <v>713</v>
       </c>
       <c r="J70" s="6" t="s">
-        <v>300</v>
+        <v>714</v>
       </c>
       <c r="K70" s="6" t="s">
-        <v>706</v>
+        <v>715</v>
       </c>
       <c r="L70" s="6" t="s">
-        <v>707</v>
+        <v>716</v>
       </c>
       <c r="M70" s="6" t="s">
-        <v>708</v>
+        <v>717</v>
       </c>
       <c r="N70" s="6" t="s">
-        <v>684</v>
+        <v>697</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>37</v>
@@ -6850,375 +7015,375 @@
     </row>
     <row r="71" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
-        <v>709</v>
+        <v>718</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>710</v>
+        <v>295</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>711</v>
+        <v>296</v>
       </c>
       <c r="F71" s="6" t="s">
-        <v>712</v>
+        <v>297</v>
       </c>
       <c r="G71" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>689</v>
+        <v>298</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>713</v>
+        <v>299</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>714</v>
+        <v>300</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>718</v>
+        <v>697</v>
       </c>
       <c r="O71" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>435</v>
+        <v>723</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>646</v>
+        <v>724</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="G72" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>361</v>
+        <v>702</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="K72" s="6" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>710</v>
+        <v>435</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>728</v>
+        <v>659</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="G73" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>689</v>
+        <v>361</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="K73" s="6" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="M73" s="6" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="O73" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>737</v>
+        <v>723</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>739</v>
-      </c>
-      <c r="G74" s="8" t="s">
-        <v>52</v>
+        <v>742</v>
+      </c>
+      <c r="G74" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>740</v>
+        <v>702</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="K74" s="6" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="M74" s="6" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="O74" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>25</v>
+        <v>524</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="G75" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>255</v>
+        <v>753</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="K75" s="6" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="M75" s="6" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>746</v>
+        <v>759</v>
       </c>
       <c r="O75" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C76" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>757</v>
+        <v>761</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="F76" s="6" t="s">
+        <v>763</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H76" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="M76" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="N76" s="6" t="s">
         <v>759</v>
-      </c>
-      <c r="G76" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="I76" s="6" t="s">
-        <v>760</v>
-      </c>
-      <c r="J76" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="K76" s="6" t="s">
-        <v>761</v>
-      </c>
-      <c r="L76" s="6" t="s">
-        <v>762</v>
-      </c>
-      <c r="M76" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="N76" s="6" t="s">
-        <v>746</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>511</v>
+        <v>25</v>
       </c>
       <c r="D77" s="6" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>766</v>
-      </c>
-      <c r="G77" s="7" t="s">
-        <v>29</v>
+        <v>772</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="J77" s="6" t="s">
-        <v>768</v>
+        <v>268</v>
       </c>
       <c r="K77" s="6" t="s">
-        <v>769</v>
+        <v>774</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>770</v>
+        <v>775</v>
       </c>
       <c r="M77" s="6" t="s">
-        <v>771</v>
+        <v>271</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>746</v>
+        <v>759</v>
       </c>
       <c r="O77" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>772</v>
+        <v>776</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C78" s="6" t="s">
-        <v>25</v>
+        <v>524</v>
       </c>
       <c r="D78" s="6" t="s">
-        <v>773</v>
+        <v>777</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>774</v>
+        <v>778</v>
       </c>
       <c r="F78" s="6" t="s">
-        <v>775</v>
-      </c>
-      <c r="G78" s="8" t="s">
-        <v>52</v>
+        <v>779</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="I78" s="6" t="s">
-        <v>776</v>
+        <v>780</v>
       </c>
       <c r="J78" s="6" t="s">
-        <v>777</v>
+        <v>781</v>
       </c>
       <c r="K78" s="6" t="s">
-        <v>778</v>
+        <v>782</v>
       </c>
       <c r="L78" s="6" t="s">
-        <v>779</v>
+        <v>783</v>
       </c>
       <c r="M78" s="6" t="s">
-        <v>780</v>
+        <v>784</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>781</v>
+        <v>759</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>37</v>
@@ -7226,48 +7391,95 @@
     </row>
     <row r="79" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>498</v>
+        <v>511</v>
       </c>
       <c r="C79" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D79" s="6" t="s">
+        <v>786</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>787</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>788</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>789</v>
+      </c>
+      <c r="J79" s="6" t="s">
+        <v>790</v>
+      </c>
+      <c r="K79" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="L79" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="M79" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="N79" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="O79" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A80" s="5" t="s">
+        <v>795</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>511</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D80" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E79" s="6" t="s">
-        <v>783</v>
-      </c>
-      <c r="F79" s="6" t="s">
-        <v>784</v>
-      </c>
-      <c r="G79" s="7" t="s">
+      <c r="E80" s="6" t="s">
+        <v>796</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>797</v>
+      </c>
+      <c r="G80" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H79" s="6" t="s">
+      <c r="H80" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I79" s="6" t="s">
-        <v>785</v>
-      </c>
-      <c r="J79" s="6" t="s">
-        <v>786</v>
-      </c>
-      <c r="K79" s="6" t="s">
-        <v>787</v>
-      </c>
-      <c r="L79" s="6" t="s">
-        <v>788</v>
-      </c>
-      <c r="M79" s="6" t="s">
-        <v>789</v>
-      </c>
-      <c r="N79" s="6" t="s">
-        <v>781</v>
-      </c>
-      <c r="O79" s="6" t="s">
+      <c r="I80" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="L80" s="6" t="s">
+        <v>801</v>
+      </c>
+      <c r="M80" s="6" t="s">
+        <v>802</v>
+      </c>
+      <c r="N80" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="O80" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7304,7 +7516,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -7325,7 +7537,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>790</v>
+        <v>803</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7372,7 +7584,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>533</v>
+        <v>546</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -7393,7 +7605,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>578</v>
+        <v>591</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -7414,7 +7626,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>667</v>
+        <v>680</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -7498,7 +7710,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7561,7 +7773,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>740</v>
+        <v>753</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7624,7 +7836,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>678</v>
+        <v>691</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
@@ -7750,7 +7962,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>689</v>
+        <v>702</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -7792,15 +8004,15 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>115</v>
+        <v>503</v>
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Thấp")</f>
@@ -7813,15 +8025,15 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>201</v>
+        <v>115</v>
       </c>
       <c r="B25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A25,'Bug List'!$G:$G,"Thấp")</f>
@@ -7834,15 +8046,15 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>428</v>
+        <v>201</v>
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A26,'Bug List'!$G:$G,"Thấp")</f>
@@ -7855,7 +8067,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>361</v>
+        <v>428</v>
       </c>
       <c r="B27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Cao")</f>
@@ -7863,7 +8075,7 @@
       </c>
       <c r="C27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Trung")</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D27" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A27,'Bug List'!$G:$G,"Thấp")</f>
@@ -7871,12 +8083,12 @@
       </c>
       <c r="E27" s="12" t="n">
         <f aca="false">SUM(B27:D27)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="s">
-        <v>243</v>
+        <v>361</v>
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Cao")</f>
@@ -7884,7 +8096,7 @@
       </c>
       <c r="C28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D28" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A28,'Bug List'!$G:$G,"Thấp")</f>
@@ -7892,20 +8104,20 @@
       </c>
       <c r="E28" s="12" t="n">
         <f aca="false">SUM(B28:D28)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>30</v>
+        <v>243</v>
       </c>
       <c r="B29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Trung")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="D29" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A29,'Bug List'!$G:$G,"Thấp")</f>
@@ -7913,37 +8125,37 @@
       </c>
       <c r="E29" s="12" t="n">
         <f aca="false">SUM(B29:D29)</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="s">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="B30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="D30" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A30,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">SUM(B30:D30)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>614</v>
+        <v>105</v>
       </c>
       <c r="B31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C31" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A31,'Bug List'!$G:$G,"Trung")</f>
@@ -7955,12 +8167,12 @@
       </c>
       <c r="E31" s="12" t="n">
         <f aca="false">SUM(B31:D31)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>481</v>
+        <v>627</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
@@ -7972,16 +8184,16 @@
       </c>
       <c r="D32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Thấp")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">SUM(B32:D32)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>222</v>
+        <v>481</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Cao")</f>
@@ -7989,28 +8201,28 @@
       </c>
       <c r="C33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E33" s="12" t="n">
         <f aca="false">SUM(B33:D33)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Thấp")</f>
@@ -8023,7 +8235,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Cao")</f>
@@ -8031,7 +8243,7 @@
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Thấp")</f>
@@ -8039,16 +8251,16 @@
       </c>
       <c r="E35" s="12" t="n">
         <f aca="false">SUM(B35:D35)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>276</v>
+        <v>160</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Trung")</f>
@@ -8060,79 +8272,100 @@
       </c>
       <c r="E36" s="12" t="n">
         <f aca="false">SUM(B36:D36)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B37" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
-        <v>790</v>
-      </c>
-      <c r="B37" s="12" t="n">
-        <f aca="false">SUM(B2:B36)</f>
+      <c r="D37" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <f aca="false">SUM(B37:D37)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="12" t="s">
+        <v>803</v>
+      </c>
+      <c r="B38" s="12" t="n">
+        <f aca="false">SUM(B2:B37)</f>
         <v>24</v>
       </c>
-      <c r="C37" s="12" t="n">
-        <f aca="false">SUM(C2:C36)</f>
-        <v>33</v>
-      </c>
-      <c r="D37" s="12" t="n">
-        <f aca="false">SUM(D2:D36)</f>
+      <c r="C38" s="12" t="n">
+        <f aca="false">SUM(C2:C37)</f>
+        <v>34</v>
+      </c>
+      <c r="D38" s="12" t="n">
+        <f aca="false">SUM(D2:D37)</f>
         <v>21</v>
       </c>
-      <c r="E37" s="12" t="n">
-        <f aca="false">SUM(E2:E36)</f>
-        <v>78</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
+      <c r="E38" s="12" t="n">
+        <f aca="false">SUM(E2:E37)</f>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="12" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
-        <v>792</v>
-      </c>
-      <c r="B40" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A40)</f>
-        <v>0</v>
+      <c r="B40" s="12" t="s">
+        <v>804</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>444</v>
+        <v>805</v>
       </c>
       <c r="B41" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A41)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
       <c r="B42" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A42)</f>
-        <v>76</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>793</v>
+        <v>37</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="11" t="s">
+        <v>806</v>
+      </c>
+      <c r="B44" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A44)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="13" t="s">
-        <v>794</v>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>807</v>
       </c>
     </row>
   </sheetData>
@@ -8160,10 +8393,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>795</v>
+        <v>808</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>796</v>
+        <v>809</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8171,7 +8404,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>797</v>
+        <v>810</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8179,15 +8412,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>798</v>
+        <v>811</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>799</v>
+        <v>812</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>800</v>
+        <v>813</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8195,95 +8428,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>801</v>
+        <v>814</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>802</v>
+        <v>815</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>803</v>
+        <v>816</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>804</v>
+        <v>817</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>805</v>
+        <v>818</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>806</v>
+        <v>819</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>807</v>
+        <v>820</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>808</v>
+        <v>821</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>809</v>
+        <v>822</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>810</v>
+        <v>823</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>811</v>
+        <v>824</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>812</v>
+        <v>825</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>813</v>
+        <v>826</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>814</v>
+        <v>827</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>815</v>
+        <v>828</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>816</v>
+        <v>829</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>817</v>
+        <v>830</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>818</v>
+        <v>831</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>819</v>
+        <v>832</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>820</v>
+        <v>833</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>821</v>
+        <v>834</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>822</v>
+        <v>835</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>823</v>
+        <v>836</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8291,31 +8524,31 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>824</v>
+        <v>837</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>825</v>
+        <v>838</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>826</v>
+        <v>839</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>827</v>
+        <v>840</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>828</v>
+        <v>841</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>829</v>
+        <v>842</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>830</v>
+        <v>843</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8323,7 +8556,7 @@
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>831</v>
+        <v>844</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-48 new-order speaker module; Nguồn and Trạng thái back to the sheet's drop-down values
PT-41..PT-48 had free text in Nguồn (kept in Triệu chứng) and PT-48 an "Đã làm" status the summary does
not count. scripts/add-bug.py now refuses values outside the sheet's drop-down lists.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1299" uniqueCount="845">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="851">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1572,9 +1572,6 @@
     <t xml:space="preserve">PT-42</t>
   </si>
   <si>
-    <t xml:space="preserve">Chủ tiệm (ảnh chụp web nhân viên)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Đơn hàng / Hoàn tiền</t>
   </si>
   <si>
@@ -1587,7 +1584,7 @@
     <t xml:space="preserve">Hiển thị trạng thái</t>
   </si>
   <si>
-    <t xml:space="preserve">Đơn đã hoàn tiền toàn bộ vẫn hiện "POS · PAID" và "Đã thanh toán" trong danh sách đơn, giống hệt đơn bình thường; phải mở từng đơn mới thấy đã hoàn.</t>
+    <t xml:space="preserve">Chủ tiệm gửi ảnh web nhân viên: Đơn đã hoàn tiền toàn bộ vẫn hiện "POS · PAID" và "Đã thanh toán" trong danh sách đơn, giống hệt đơn bình thường; phải mở từng đơn mới thấy đã hoàn.</t>
   </si>
   <si>
     <t xml:space="preserve">API danh sách đơn chỉ trả các cột của qr_orders; tổng hoàn tiền nằm ở pos_refunds và chỉ được tính trong màn chi tiết đơn (overview). Danh sách không có dữ liệu để phân biệt.</t>
@@ -1650,9 +1647,6 @@
     <t xml:space="preserve">PT-43</t>
   </si>
   <si>
-    <t xml:space="preserve">Chủ tiệm</t>
-  </si>
-  <si>
     <t xml:space="preserve">Giao diện nhân viên / Điều hướng</t>
   </si>
   <si>
@@ -1665,7 +1659,7 @@
     <t xml:space="preserve">Giao diện / thao tác</t>
   </si>
   <si>
-    <t xml:space="preserve">Mỗi lần bấm một mục, mở đơn, quay lại hay đồng bộ tự động, thanh menu dưới nhảy về mục đầu tiên; muốn bấm Hoàn tiền, Chấm công, Quản trị phải kéo sang lại mỗi lần.</t>
+    <t xml:space="preserve">Chủ tiệm báo: Mỗi lần bấm một mục, mở đơn, quay lại hay đồng bộ tự động, thanh menu dưới nhảy về mục đầu tiên; muốn bấm Hoàn tiền, Chấm công, Quản trị phải kéo sang lại mỗi lần.</t>
   </si>
   <si>
     <t xml:space="preserve">render() dựng lại toàn bộ #app (cả &lt;nav&gt;) và chỉ khôi phục nav.scrollTop, viết cho menu dọc của trang quầy. Trên điện thoại menu cuộn ngang (overflow-x), nên scrollLeft luôn về 0.</t>
@@ -1689,7 +1683,7 @@
     <t xml:space="preserve">Điện thoại và máy SUNMI, tài khoản chủ tiệm</t>
   </si>
   <si>
-    <t xml:space="preserve">Chủ tiệm có hai lối vào cùng một màn "Món &amp; giá": một mục riêng trên thanh menu và một ô trong Quản trị chủ tiệm, làm menu dài và rối.</t>
+    <t xml:space="preserve">Chủ tiệm yêu cầu: Chủ tiệm có hai lối vào cùng một màn "Món &amp; giá": một mục riêng trên thanh menu và một ô trong Quản trị chủ tiệm, làm menu dài và rối.</t>
   </si>
   <si>
     <t xml:space="preserve">Mục "Món &amp; giá" thêm vào menu theo quyền CATALOG_MANAGE trước khi có màn Quản trị; khi thêm Quản trị không bỏ mục cũ cho chủ tiệm.</t>
@@ -1707,9 +1701,6 @@
     <t xml:space="preserve">PT-45</t>
   </si>
   <si>
-    <t xml:space="preserve">CI (run 37322764520, main 0b3e27c)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Kiểm thử / Mô phỏng</t>
   </si>
   <si>
@@ -1722,7 +1713,7 @@
     <t xml:space="preserve">Test chập chờn</t>
   </si>
   <si>
-    <t xml:space="preserve">CI đỏ với "no message" ở case tiền mặt thiếu, trong khi cùng commit xanh trên nhánh online-v1.7 và chạy ở máy; app vẫn từ chối và đơn vẫn UNPAID.</t>
+    <t xml:space="preserve">CI run 37322764520 (main 0b3e27c): CI đỏ với "no message" ở case tiền mặt thiếu, trong khi cùng commit xanh trên nhánh online-v1.7 và chạy ở máy; app vẫn từ chối và đơn vẫn UNPAID.</t>
   </si>
   <si>
     <t xml:space="preserve">Case đọc màn hình sau khi click xong để tìm "chưa đủ", nhưng thông báo tự tắt sau 7 giây. Trên runner tải nặng, click cùng hộp nhập số tiền có thể kéo dài quá thời gian đó nên test thấy màn hình đã sạch. Lỗi ở cách đo, không ở app.</t>
@@ -1743,13 +1734,10 @@
     <t xml:space="preserve">PT-46</t>
   </si>
   <si>
-    <t xml:space="preserve">CI (run 37324875053, main 8627bf7)</t>
-  </si>
-  <si>
     <t xml:space="preserve">scripts/sim-browser.mjs case "Handheld: pay cash with change; the receipt goes to the SUNMI printer…"</t>
   </si>
   <si>
-    <t xml:space="preserve">CI đỏ với "no receipt printed" sau khi thu tiền mặt, trong khi cùng commit xanh trên nhánh; app vẫn in biên lai.</t>
+    <t xml:space="preserve">CI run 37324875053 (main 8627bf7): CI đỏ với "no receipt printed" sau khi thu tiền mặt, trong khi cùng commit xanh trên nhánh; app vẫn in biên lai.</t>
   </si>
   <si>
     <t xml:space="preserve">Case coi mã đơn "-TM" hiện trên màn hình là dấu hiệu đã in xong, rồi đọc ngay hàng đợi in. Nhưng đồng bộ trực tiếp có thể vẽ mã đã trả trước khi callback thanh toán gửi biên lai sang máy in (printReceipt chạy sau). Lỗi ở cách đo, không ở app.</t>
@@ -1771,9 +1759,6 @@
   </si>
   <si>
     <t xml:space="preserve">2026-10-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chủ tiệm (ảnh máy SUNMI, APK 1.7.79)</t>
   </si>
   <si>
     <t xml:space="preserve">Phân ca / Chấm công</t>
@@ -1830,7 +1815,7 @@
     <t xml:space="preserve">Nhập liệu / thông báo lỗi</t>
   </si>
   <si>
-    <t xml:space="preserve">Tạo ca "CA SANG" cho 3 nhân viên trên máy SUNMI báo "Dữ liệu nhập không hợp lệ", không nói sai ô nào; chủ tiệm không tạo được ca.</t>
+    <t xml:space="preserve">Chủ tiệm gửi ảnh máy SUNMI, APK 1.7.79: Tạo ca "CA SANG" cho 3 nhân viên trên máy SUNMI báo "Dữ liệu nhập không hợp lệ", không nói sai ô nào; chủ tiệm không tạo được ca.</t>
   </si>
   <si>
     <r>
@@ -1930,6 +1915,81 @@
   </si>
   <si>
     <t xml:space="preserve">a7f7a8f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đơn hàng / Thông báo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js (announce*, watchOrders, announceCard); android MainActivity.java (speak, chime, keepScreenOn); AndroidManifest.xml (TTS_SERVICE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máy SUNMI ghép loa Bluetooth, app mở liên tục; Phát Tài không có máy quầy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiếu chức năng / vận hành</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yêu cầu của khách hàng qua chủ tiệm: Khách đặt đơn QR nhưng không có âm thanh báo, nhân viên phải nhìn màn hình mới biết; khách hàng yêu cầu phát loa mỗi khi có đơn. Loa của máy SUNMI rè, không dùng được; quán không có máy quầy; cần đọc bằng tiếng Trung.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hệ thống chỉ đẩy đơn mới lên màn hình (realtime + đồng bộ), không có khâu phát âm thanh. Đồng bộ đơn chỉ chạy ở một số màn hình, và khi màn hình tắt thì WebView dừng, nên không thể đọc đơn nếu máy không mở.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Module loa: máy có đơn QR mới phát chuông rồi đọc "5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">号桌，有新订单</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">" (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Sans CJK SC"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">外带 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">với đơn mang về) bằng giọng tiếng Trung của Android (APK) hoặc của trình duyệt, kèm bảng thông báo; tài khoản bếp nghe mọi đơn mới. Bật/tắt riêng từng máy trong Cài đặt, mặc định tắt; khi bật, APK giữ màn hình luôn sáng. Bộ theo dõi đơn nhẹ chạy ở mọi màn hình; lúc bật loa lấy đơn hiện có làm mốc để không đọc muộn đơn đặt khi đang tắt. Cách dùng: ghép loa Bluetooth với một máy SUNMI, mở app, cắm sạc, bật loa trong Cài đặt.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v184-announce.test.mjs: "PT-48 what was there when the device opened is not read out…", "PT-48 the kitchen account hears every new order…", "PT-48 off by default, turned on per device…"; scripts/sim-browser.mjs: "Handheld: the speaker is off by default; turned on, the screen stays awake and a customer QR order is read out…", "Handheld: an order the staff enter themselves is not read out", "Handheld: still read out on the order list…", "Handheld: the test button speaks…", "Browser: with no Chinese voice a turned-on page still chimes…".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thông báo cần chạy khi người dùng đang ở màn hình nào, và khi màn hình/app tắt thì sao? Bật lại sau khi tắt có đọc lại việc cũ không? Máy thật có giọng đọc của ngôn ngữ cần không (Android 11+ phải khai báo TTS_SERVICE)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9faa2bf</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-01</t>
@@ -3256,7 +3316,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3301,19 +3361,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3439,8 +3495,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O80" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O80"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O81"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3703,7 +3759,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O80"/>
+  <dimension ref="A1:O81"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -5705,40 +5761,40 @@
         <v>251</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="E43" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="E43" s="6" t="s">
+      <c r="F43" s="6" t="s">
         <v>448</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>449</v>
       </c>
       <c r="G43" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H43" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="I43" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="I43" s="6" t="s">
+      <c r="J43" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="J43" s="6" t="s">
+      <c r="K43" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="K43" s="6" t="s">
+      <c r="L43" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="L43" s="6" t="s">
+      <c r="M43" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="M43" s="6" t="s">
+      <c r="N43" s="6" t="s">
         <v>455</v>
-      </c>
-      <c r="N43" s="6" t="s">
-        <v>456</v>
       </c>
       <c r="O43" s="6" t="s">
         <v>37</v>
@@ -5746,46 +5802,46 @@
     </row>
     <row r="44" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B44" s="6" t="s">
         <v>251</v>
       </c>
       <c r="C44" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="E44" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="F44" s="6" t="s">
         <v>459</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>460</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>461</v>
       </c>
       <c r="G44" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H44" s="6" t="s">
+        <v>460</v>
+      </c>
+      <c r="I44" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="J44" s="6" t="s">
         <v>462</v>
       </c>
-      <c r="I44" s="6" t="s">
+      <c r="K44" s="6" t="s">
         <v>463</v>
       </c>
-      <c r="J44" s="6" t="s">
+      <c r="L44" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="K44" s="6" t="s">
+      <c r="M44" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="L44" s="6" t="s">
-        <v>466</v>
-      </c>
-      <c r="M44" s="6" t="s">
-        <v>467</v>
-      </c>
       <c r="N44" s="6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="O44" s="6" t="s">
         <v>37</v>
@@ -5793,46 +5849,46 @@
     </row>
     <row r="45" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B45" s="6" t="s">
         <v>251</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>458</v>
+        <v>25</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="F45" s="6" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H45" s="6" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="I45" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="J45" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="K45" s="6" t="s">
         <v>471</v>
       </c>
-      <c r="J45" s="6" t="s">
+      <c r="L45" s="6" t="s">
         <v>472</v>
       </c>
-      <c r="K45" s="6" t="s">
+      <c r="M45" s="6" t="s">
         <v>473</v>
       </c>
-      <c r="L45" s="6" t="s">
-        <v>474</v>
-      </c>
-      <c r="M45" s="6" t="s">
-        <v>475</v>
-      </c>
       <c r="N45" s="6" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="O45" s="6" t="s">
         <v>37</v>
@@ -5840,46 +5896,46 @@
     </row>
     <row r="46" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="B46" s="6" t="s">
         <v>251</v>
       </c>
       <c r="C46" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="F46" s="6" t="s">
         <v>477</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>478</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>479</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>480</v>
       </c>
       <c r="G46" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H46" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="I46" s="6" t="s">
+        <v>479</v>
+      </c>
+      <c r="J46" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="K46" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="I46" s="6" t="s">
+      <c r="L46" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="J46" s="6" t="s">
+      <c r="M46" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="K46" s="6" t="s">
+      <c r="N46" s="6" t="s">
         <v>484</v>
-      </c>
-      <c r="L46" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="M46" s="6" t="s">
-        <v>486</v>
-      </c>
-      <c r="N46" s="6" t="s">
-        <v>487</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>37</v>
@@ -5887,234 +5943,234 @@
     </row>
     <row r="47" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
       <c r="B47" s="6" t="s">
         <v>251</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>489</v>
+        <v>25</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="F47" s="6" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H47" s="6" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="I47" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="K47" s="6" t="s">
+        <v>489</v>
+      </c>
+      <c r="L47" s="6" t="s">
+        <v>490</v>
+      </c>
+      <c r="M47" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="J47" s="6" t="s">
+      <c r="N47" s="6" t="s">
         <v>492</v>
-      </c>
-      <c r="K47" s="6" t="s">
-        <v>493</v>
-      </c>
-      <c r="L47" s="6" t="s">
-        <v>494</v>
-      </c>
-      <c r="M47" s="6" t="s">
-        <v>495</v>
-      </c>
-      <c r="N47" s="6" t="s">
-        <v>496</v>
       </c>
       <c r="O47" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
+        <v>493</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="F48" s="6" t="s">
         <v>497</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>498</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>499</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>500</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>501</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>502</v>
       </c>
       <c r="G48" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H48" s="6" t="s">
+        <v>498</v>
+      </c>
+      <c r="I48" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="J48" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="K48" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="L48" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="M48" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="I48" s="6" t="s">
+      <c r="N48" s="6" t="s">
         <v>504</v>
-      </c>
-      <c r="J48" s="6" t="s">
-        <v>505</v>
-      </c>
-      <c r="K48" s="6" t="s">
-        <v>506</v>
-      </c>
-      <c r="L48" s="6" t="s">
-        <v>507</v>
-      </c>
-      <c r="M48" s="6" t="s">
-        <v>508</v>
-      </c>
-      <c r="N48" s="6" t="s">
-        <v>509</v>
       </c>
       <c r="O48" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="168.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
+        <v>505</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>494</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>508</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H49" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="I49" s="6" t="s">
         <v>510</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="J49" s="6" t="s">
         <v>511</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="K49" s="6" t="s">
         <v>512</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="L49" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="M49" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="F49" s="6" t="s">
+      <c r="N49" s="6" t="s">
         <v>515</v>
-      </c>
-      <c r="G49" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H49" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="I49" s="6" t="s">
-        <v>517</v>
-      </c>
-      <c r="J49" s="6" t="s">
-        <v>518</v>
-      </c>
-      <c r="K49" s="6" t="s">
-        <v>519</v>
-      </c>
-      <c r="L49" s="6" t="s">
-        <v>520</v>
-      </c>
-      <c r="M49" s="6" t="s">
-        <v>521</v>
-      </c>
-      <c r="N49" s="6" t="s">
-        <v>522</v>
       </c>
       <c r="O49" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
+        <v>516</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>519</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="F50" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="G50" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="I50" s="6" t="s">
         <v>523</v>
       </c>
-      <c r="B50" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C50" s="6" t="s">
+      <c r="J50" s="6" t="s">
         <v>524</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="K50" s="6" t="s">
         <v>525</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="L50" s="6" t="s">
         <v>526</v>
       </c>
-      <c r="F50" s="6" t="s">
+      <c r="M50" s="6" t="s">
         <v>527</v>
       </c>
-      <c r="G50" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="I50" s="6" t="s">
+      <c r="N50" s="6" t="s">
         <v>528</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>529</v>
-      </c>
-      <c r="K50" s="6" t="s">
-        <v>530</v>
-      </c>
-      <c r="L50" s="6" t="s">
-        <v>531</v>
-      </c>
-      <c r="M50" s="6" t="s">
-        <v>532</v>
-      </c>
-      <c r="N50" s="6" t="s">
-        <v>522</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>532</v>
+      </c>
+      <c r="F51" s="6" t="s">
         <v>533</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D51" s="6" t="s">
+      <c r="G51" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="I51" s="6" t="s">
         <v>534</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="J51" s="6" t="s">
         <v>535</v>
       </c>
-      <c r="F51" s="6" t="s">
+      <c r="K51" s="6" t="s">
         <v>536</v>
       </c>
-      <c r="G51" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="I51" s="6" t="s">
+      <c r="L51" s="6" t="s">
         <v>537</v>
       </c>
-      <c r="J51" s="6" t="s">
+      <c r="M51" s="6" t="s">
         <v>538</v>
       </c>
-      <c r="K51" s="6" t="s">
-        <v>539</v>
-      </c>
-      <c r="L51" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="M51" s="6" t="s">
-        <v>541</v>
-      </c>
       <c r="N51" s="6" t="s">
-        <v>542</v>
+        <v>528</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
@@ -6122,140 +6178,140 @@
     </row>
     <row r="52" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>543</v>
+        <v>539</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>146</v>
+        <v>540</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="F52" s="6" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="G52" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H52" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="L52" s="6" t="s">
         <v>546</v>
       </c>
-      <c r="I52" s="6" t="s">
+      <c r="M52" s="6" t="s">
         <v>547</v>
       </c>
-      <c r="J52" s="6" t="s">
+      <c r="N52" s="6" t="s">
         <v>548</v>
-      </c>
-      <c r="K52" s="6" t="s">
-        <v>549</v>
-      </c>
-      <c r="L52" s="6" t="s">
-        <v>550</v>
-      </c>
-      <c r="M52" s="6" t="s">
-        <v>551</v>
-      </c>
-      <c r="N52" s="6" t="s">
-        <v>552</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>554</v>
+        <v>146</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>555</v>
+        <v>550</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>545</v>
+        <v>551</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="I53" s="6" t="s">
+        <v>553</v>
+      </c>
+      <c r="J53" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="K53" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="L53" s="6" t="s">
         <v>556</v>
       </c>
-      <c r="J53" s="6" t="s">
+      <c r="M53" s="6" t="s">
         <v>557</v>
       </c>
-      <c r="K53" s="6" t="s">
+      <c r="N53" s="6" t="s">
         <v>558</v>
-      </c>
-      <c r="L53" s="6" t="s">
-        <v>559</v>
-      </c>
-      <c r="M53" s="6" t="s">
-        <v>560</v>
-      </c>
-      <c r="N53" s="6" t="s">
-        <v>552</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="E54" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D54" s="6" t="s">
+      <c r="F54" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="G54" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="I54" s="6" t="s">
         <v>562</v>
       </c>
-      <c r="E54" s="6" t="s">
+      <c r="J54" s="6" t="s">
         <v>563</v>
       </c>
-      <c r="F54" s="6" t="s">
+      <c r="K54" s="6" t="s">
         <v>564</v>
       </c>
-      <c r="G54" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="I54" s="6" t="s">
+      <c r="L54" s="6" t="s">
         <v>565</v>
       </c>
-      <c r="J54" s="6" t="s">
+      <c r="M54" s="6" t="s">
         <v>566</v>
       </c>
-      <c r="K54" s="6" t="s">
-        <v>567</v>
-      </c>
-      <c r="L54" s="6" t="s">
-        <v>568</v>
-      </c>
-      <c r="M54" s="6" t="s">
-        <v>569</v>
-      </c>
       <c r="N54" s="6" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
@@ -6263,398 +6319,398 @@
     </row>
     <row r="55" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
+        <v>567</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="F55" s="6" t="s">
         <v>570</v>
       </c>
-      <c r="B55" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="E55" s="6" t="s">
+      <c r="G55" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="I55" s="6" t="s">
         <v>571</v>
       </c>
-      <c r="F55" s="6" t="s">
-        <v>545</v>
-      </c>
-      <c r="G55" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="I55" s="6" t="s">
+      <c r="J55" s="6" t="s">
         <v>572</v>
       </c>
-      <c r="J55" s="6" t="s">
+      <c r="K55" s="6" t="s">
         <v>573</v>
       </c>
-      <c r="K55" s="6" t="s">
+      <c r="L55" s="6" t="s">
         <v>574</v>
       </c>
-      <c r="L55" s="6" t="s">
+      <c r="M55" s="6" t="s">
         <v>575</v>
       </c>
-      <c r="M55" s="6" t="s">
-        <v>576</v>
-      </c>
       <c r="N55" s="6" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
+        <v>576</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E56" s="6" t="s">
         <v>577</v>
       </c>
-      <c r="B56" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D56" s="6" t="s">
+      <c r="F56" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="G56" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="I56" s="6" t="s">
         <v>578</v>
       </c>
-      <c r="E56" s="6" t="s">
+      <c r="J56" s="6" t="s">
         <v>579</v>
       </c>
-      <c r="F56" s="6" t="s">
+      <c r="K56" s="6" t="s">
         <v>580</v>
       </c>
-      <c r="G56" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>372</v>
-      </c>
-      <c r="I56" s="6" t="s">
+      <c r="L56" s="6" t="s">
         <v>581</v>
       </c>
-      <c r="J56" s="6" t="s">
+      <c r="M56" s="6" t="s">
         <v>582</v>
       </c>
-      <c r="K56" s="6" t="s">
-        <v>583</v>
-      </c>
-      <c r="L56" s="6" t="s">
-        <v>584</v>
-      </c>
-      <c r="M56" s="6" t="s">
-        <v>585</v>
-      </c>
       <c r="N56" s="6" t="s">
-        <v>586</v>
+        <v>558</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H57" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="J57" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="K57" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="L57" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="M57" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="I57" s="6" t="s">
+      <c r="N57" s="6" t="s">
         <v>592</v>
-      </c>
-      <c r="J57" s="6" t="s">
-        <v>593</v>
-      </c>
-      <c r="K57" s="6" t="s">
-        <v>594</v>
-      </c>
-      <c r="L57" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="M57" s="6" t="s">
-        <v>596</v>
-      </c>
-      <c r="N57" s="6" t="s">
-        <v>586</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>53</v>
+        <v>597</v>
       </c>
       <c r="I58" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="J58" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="K58" s="6" t="s">
+        <v>600</v>
+      </c>
+      <c r="L58" s="6" t="s">
         <v>601</v>
       </c>
-      <c r="J58" s="6" t="s">
+      <c r="M58" s="6" t="s">
         <v>602</v>
       </c>
-      <c r="K58" s="6" t="s">
-        <v>603</v>
-      </c>
-      <c r="L58" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="M58" s="6" t="s">
-        <v>605</v>
-      </c>
       <c r="N58" s="6" t="s">
-        <v>606</v>
+        <v>592</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>605</v>
+      </c>
+      <c r="F59" s="6" t="s">
+        <v>606</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>607</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>598</v>
-      </c>
-      <c r="E59" s="6" t="s">
+      <c r="J59" s="6" t="s">
         <v>608</v>
       </c>
-      <c r="F59" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G59" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H59" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I59" s="6" t="s">
+      <c r="K59" s="6" t="s">
         <v>609</v>
       </c>
-      <c r="J59" s="6" t="s">
+      <c r="L59" s="6" t="s">
         <v>610</v>
       </c>
-      <c r="K59" s="6" t="s">
+      <c r="M59" s="6" t="s">
         <v>611</v>
       </c>
-      <c r="L59" s="6" t="s">
+      <c r="N59" s="6" t="s">
         <v>612</v>
-      </c>
-      <c r="M59" s="6" t="s">
-        <v>613</v>
-      </c>
-      <c r="N59" s="6" t="s">
-        <v>606</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>604</v>
+      </c>
+      <c r="E60" s="6" t="s">
         <v>614</v>
       </c>
-      <c r="B60" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D60" s="6" t="s">
+      <c r="F60" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G60" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I60" s="6" t="s">
         <v>615</v>
       </c>
-      <c r="E60" s="6" t="s">
+      <c r="J60" s="6" t="s">
         <v>616</v>
       </c>
-      <c r="F60" s="6" t="s">
+      <c r="K60" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="G60" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="I60" s="6" t="s">
+      <c r="L60" s="6" t="s">
         <v>618</v>
       </c>
-      <c r="J60" s="6" t="s">
+      <c r="M60" s="6" t="s">
         <v>619</v>
       </c>
-      <c r="K60" s="6" t="s">
-        <v>620</v>
-      </c>
-      <c r="L60" s="6" t="s">
-        <v>621</v>
-      </c>
-      <c r="M60" s="6" t="s">
-        <v>622</v>
-      </c>
       <c r="N60" s="6" t="s">
-        <v>586</v>
+        <v>612</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>621</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>622</v>
+      </c>
+      <c r="F61" s="6" t="s">
         <v>623</v>
-      </c>
-      <c r="B61" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>624</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="F61" s="6" t="s">
-        <v>626</v>
       </c>
       <c r="G61" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H61" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="J61" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="L61" s="6" t="s">
         <v>627</v>
       </c>
-      <c r="I61" s="6" t="s">
+      <c r="M61" s="6" t="s">
         <v>628</v>
       </c>
-      <c r="J61" s="6" t="s">
-        <v>629</v>
-      </c>
-      <c r="K61" s="6" t="s">
-        <v>630</v>
-      </c>
-      <c r="L61" s="6" t="s">
-        <v>631</v>
-      </c>
-      <c r="M61" s="6" t="s">
-        <v>632</v>
-      </c>
       <c r="N61" s="6" t="s">
-        <v>633</v>
+        <v>592</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>631</v>
+      </c>
+      <c r="F62" s="6" t="s">
+        <v>632</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H62" s="6" t="s">
+        <v>633</v>
+      </c>
+      <c r="I62" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="B62" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D62" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="E62" s="6" t="s">
+      <c r="J62" s="6" t="s">
         <v>635</v>
       </c>
-      <c r="F62" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G62" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H62" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="I62" s="6" t="s">
+      <c r="K62" s="6" t="s">
         <v>636</v>
       </c>
-      <c r="J62" s="6" t="s">
+      <c r="L62" s="6" t="s">
         <v>637</v>
       </c>
-      <c r="K62" s="6" t="s">
+      <c r="M62" s="6" t="s">
         <v>638</v>
       </c>
-      <c r="L62" s="6" t="s">
+      <c r="N62" s="6" t="s">
         <v>639</v>
-      </c>
-      <c r="M62" s="6" t="s">
-        <v>640</v>
-      </c>
-      <c r="N62" s="6" t="s">
-        <v>641</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>642</v>
+        <v>640</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>512</v>
+        <v>530</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>644</v>
+        <v>211</v>
       </c>
       <c r="G63" s="8" t="s">
         <v>52</v>
@@ -6663,69 +6719,69 @@
         <v>149</v>
       </c>
       <c r="I63" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="J63" s="6" t="s">
+        <v>643</v>
+      </c>
+      <c r="K63" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="L63" s="6" t="s">
         <v>645</v>
       </c>
-      <c r="J63" s="6" t="s">
+      <c r="M63" s="6" t="s">
         <v>646</v>
       </c>
-      <c r="K63" s="6" t="s">
+      <c r="N63" s="6" t="s">
         <v>647</v>
-      </c>
-      <c r="L63" s="6" t="s">
-        <v>604</v>
-      </c>
-      <c r="M63" s="6" t="s">
-        <v>648</v>
-      </c>
-      <c r="N63" s="6" t="s">
-        <v>649</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
+        <v>648</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>649</v>
+      </c>
+      <c r="F64" s="6" t="s">
         <v>650</v>
       </c>
-      <c r="B64" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D64" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>307</v>
-      </c>
-      <c r="F64" s="6" t="s">
+      <c r="G64" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H64" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="I64" s="6" t="s">
         <v>651</v>
       </c>
-      <c r="G64" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H64" s="6" t="s">
-        <v>309</v>
-      </c>
-      <c r="I64" s="6" t="s">
+      <c r="J64" s="6" t="s">
         <v>652</v>
       </c>
-      <c r="J64" s="6" t="s">
+      <c r="K64" s="6" t="s">
         <v>653</v>
       </c>
-      <c r="K64" s="6" t="s">
+      <c r="L64" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="M64" s="6" t="s">
         <v>654</v>
       </c>
-      <c r="L64" s="6" t="s">
+      <c r="N64" s="6" t="s">
         <v>655</v>
-      </c>
-      <c r="M64" s="6" t="s">
-        <v>656</v>
-      </c>
-      <c r="N64" s="6" t="s">
-        <v>657</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
@@ -6733,328 +6789,328 @@
     </row>
     <row r="65" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
+        <v>656</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F65" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="G65" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H65" s="6" t="s">
+        <v>309</v>
+      </c>
+      <c r="I65" s="6" t="s">
         <v>658</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>435</v>
-      </c>
-      <c r="E65" s="6" t="s">
+      <c r="J65" s="6" t="s">
         <v>659</v>
       </c>
-      <c r="F65" s="6" t="s">
+      <c r="K65" s="6" t="s">
         <v>660</v>
       </c>
-      <c r="G65" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H65" s="6" t="s">
-        <v>361</v>
-      </c>
-      <c r="I65" s="6" t="s">
+      <c r="L65" s="6" t="s">
         <v>661</v>
       </c>
-      <c r="J65" s="6" t="s">
+      <c r="M65" s="6" t="s">
         <v>662</v>
       </c>
-      <c r="K65" s="6" t="s">
+      <c r="N65" s="6" t="s">
         <v>663</v>
-      </c>
-      <c r="L65" s="6" t="s">
-        <v>664</v>
-      </c>
-      <c r="M65" s="6" t="s">
-        <v>665</v>
-      </c>
-      <c r="N65" s="6" t="s">
-        <v>666</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>667</v>
+        <v>664</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>668</v>
+        <v>435</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>669</v>
+        <v>665</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>670</v>
+        <v>666</v>
       </c>
       <c r="G66" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>546</v>
+        <v>361</v>
       </c>
       <c r="I66" s="6" t="s">
+        <v>667</v>
+      </c>
+      <c r="J66" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="K66" s="6" t="s">
+        <v>669</v>
+      </c>
+      <c r="L66" s="6" t="s">
+        <v>670</v>
+      </c>
+      <c r="M66" s="6" t="s">
         <v>671</v>
       </c>
-      <c r="J66" s="6" t="s">
+      <c r="N66" s="6" t="s">
         <v>672</v>
-      </c>
-      <c r="K66" s="6" t="s">
-        <v>673</v>
-      </c>
-      <c r="L66" s="6" t="s">
-        <v>674</v>
-      </c>
-      <c r="M66" s="6" t="s">
-        <v>675</v>
-      </c>
-      <c r="N66" s="6" t="s">
-        <v>666</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
+        <v>673</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>674</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="F67" s="6" t="s">
         <v>676</v>
       </c>
-      <c r="B67" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D67" s="6" t="s">
+      <c r="G67" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H67" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="I67" s="6" t="s">
         <v>677</v>
       </c>
-      <c r="E67" s="6" t="s">
+      <c r="J67" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="F67" s="6" t="s">
+      <c r="K67" s="6" t="s">
         <v>679</v>
       </c>
-      <c r="G67" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H67" s="6" t="s">
+      <c r="L67" s="6" t="s">
         <v>680</v>
       </c>
-      <c r="I67" s="6" t="s">
+      <c r="M67" s="6" t="s">
         <v>681</v>
       </c>
-      <c r="J67" s="6" t="s">
-        <v>682</v>
-      </c>
-      <c r="K67" s="6" t="s">
-        <v>683</v>
-      </c>
-      <c r="L67" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="M67" s="6" t="s">
-        <v>685</v>
-      </c>
       <c r="N67" s="6" t="s">
-        <v>686</v>
+        <v>672</v>
       </c>
       <c r="O67" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>687</v>
+        <v>682</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>688</v>
+        <v>683</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>689</v>
+        <v>684</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>690</v>
+        <v>685</v>
       </c>
       <c r="G68" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H68" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="J68" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="M68" s="6" t="s">
         <v>691</v>
       </c>
-      <c r="I68" s="6" t="s">
+      <c r="N68" s="6" t="s">
         <v>692</v>
-      </c>
-      <c r="J68" s="6" t="s">
-        <v>693</v>
-      </c>
-      <c r="K68" s="6" t="s">
-        <v>694</v>
-      </c>
-      <c r="L68" s="6" t="s">
-        <v>695</v>
-      </c>
-      <c r="M68" s="6" t="s">
-        <v>696</v>
-      </c>
-      <c r="N68" s="6" t="s">
-        <v>697</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
+        <v>693</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>694</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>695</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>697</v>
+      </c>
+      <c r="I69" s="6" t="s">
         <v>698</v>
       </c>
-      <c r="B69" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D69" s="6" t="s">
+      <c r="J69" s="6" t="s">
         <v>699</v>
       </c>
-      <c r="E69" s="6" t="s">
+      <c r="K69" s="6" t="s">
         <v>700</v>
       </c>
-      <c r="F69" s="6" t="s">
+      <c r="L69" s="6" t="s">
         <v>701</v>
       </c>
-      <c r="G69" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H69" s="6" t="s">
+      <c r="M69" s="6" t="s">
         <v>702</v>
       </c>
-      <c r="I69" s="6" t="s">
+      <c r="N69" s="6" t="s">
         <v>703</v>
-      </c>
-      <c r="J69" s="6" t="s">
-        <v>704</v>
-      </c>
-      <c r="K69" s="6" t="s">
-        <v>705</v>
-      </c>
-      <c r="L69" s="6" t="s">
-        <v>706</v>
-      </c>
-      <c r="M69" s="6" t="s">
-        <v>707</v>
-      </c>
-      <c r="N69" s="6" t="s">
-        <v>708</v>
       </c>
       <c r="O69" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D70" s="6" t="s">
+        <v>705</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>706</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>707</v>
+      </c>
+      <c r="G70" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H70" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="I70" s="6" t="s">
         <v>709</v>
       </c>
-      <c r="B70" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D70" s="6" t="s">
+      <c r="J70" s="6" t="s">
         <v>710</v>
       </c>
-      <c r="E70" s="6" t="s">
+      <c r="K70" s="6" t="s">
         <v>711</v>
       </c>
-      <c r="F70" s="6" t="s">
+      <c r="L70" s="6" t="s">
         <v>712</v>
       </c>
-      <c r="G70" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H70" s="6" t="s">
-        <v>702</v>
-      </c>
-      <c r="I70" s="6" t="s">
+      <c r="M70" s="6" t="s">
         <v>713</v>
       </c>
-      <c r="J70" s="6" t="s">
+      <c r="N70" s="6" t="s">
         <v>714</v>
-      </c>
-      <c r="K70" s="6" t="s">
-        <v>715</v>
-      </c>
-      <c r="L70" s="6" t="s">
-        <v>716</v>
-      </c>
-      <c r="M70" s="6" t="s">
-        <v>717</v>
-      </c>
-      <c r="N70" s="6" t="s">
-        <v>697</v>
       </c>
       <c r="O70" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
+        <v>715</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D71" s="6" t="s">
+        <v>716</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>717</v>
+      </c>
+      <c r="F71" s="6" t="s">
         <v>718</v>
       </c>
-      <c r="B71" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D71" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>296</v>
-      </c>
-      <c r="F71" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G71" s="7" t="s">
-        <v>29</v>
+      <c r="G71" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>298</v>
+        <v>708</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>299</v>
+        <v>719</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>300</v>
+        <v>720</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="O71" s="6" t="s">
         <v>37</v>
@@ -7062,375 +7118,375 @@
     </row>
     <row r="72" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>723</v>
+        <v>295</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>724</v>
+        <v>296</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>725</v>
+        <v>297</v>
       </c>
       <c r="G72" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>702</v>
+        <v>298</v>
       </c>
       <c r="I72" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="J72" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="K72" s="6" t="s">
+        <v>725</v>
+      </c>
+      <c r="L72" s="6" t="s">
         <v>726</v>
       </c>
-      <c r="J72" s="6" t="s">
+      <c r="M72" s="6" t="s">
         <v>727</v>
       </c>
-      <c r="K72" s="6" t="s">
-        <v>728</v>
-      </c>
-      <c r="L72" s="6" t="s">
-        <v>729</v>
-      </c>
-      <c r="M72" s="6" t="s">
-        <v>730</v>
-      </c>
       <c r="N72" s="6" t="s">
-        <v>731</v>
+        <v>703</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>732</v>
+        <v>728</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>524</v>
+        <v>530</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>435</v>
+        <v>729</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>659</v>
+        <v>730</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>733</v>
+        <v>731</v>
       </c>
       <c r="G73" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>361</v>
+        <v>708</v>
       </c>
       <c r="I73" s="6" t="s">
+        <v>732</v>
+      </c>
+      <c r="J73" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="K73" s="6" t="s">
         <v>734</v>
       </c>
-      <c r="J73" s="6" t="s">
+      <c r="L73" s="6" t="s">
         <v>735</v>
       </c>
-      <c r="K73" s="6" t="s">
+      <c r="M73" s="6" t="s">
         <v>736</v>
       </c>
-      <c r="L73" s="6" t="s">
+      <c r="N73" s="6" t="s">
         <v>737</v>
       </c>
-      <c r="M73" s="6" t="s">
+      <c r="O73" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="5" t="s">
         <v>738</v>
       </c>
-      <c r="N73" s="6" t="s">
+      <c r="B74" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="F74" s="6" t="s">
         <v>739</v>
-      </c>
-      <c r="O73" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
-        <v>740</v>
-      </c>
-      <c r="B74" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>723</v>
-      </c>
-      <c r="E74" s="6" t="s">
-        <v>741</v>
-      </c>
-      <c r="F74" s="6" t="s">
-        <v>742</v>
       </c>
       <c r="G74" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>702</v>
+        <v>361</v>
       </c>
       <c r="I74" s="6" t="s">
+        <v>740</v>
+      </c>
+      <c r="J74" s="6" t="s">
+        <v>741</v>
+      </c>
+      <c r="K74" s="6" t="s">
+        <v>742</v>
+      </c>
+      <c r="L74" s="6" t="s">
         <v>743</v>
       </c>
-      <c r="J74" s="6" t="s">
+      <c r="M74" s="6" t="s">
         <v>744</v>
       </c>
-      <c r="K74" s="6" t="s">
+      <c r="N74" s="6" t="s">
         <v>745</v>
       </c>
-      <c r="L74" s="6" t="s">
+      <c r="O74" s="6" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="5" t="s">
         <v>746</v>
       </c>
-      <c r="M74" s="6" t="s">
+      <c r="B75" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C75" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>729</v>
+      </c>
+      <c r="E75" s="6" t="s">
         <v>747</v>
       </c>
-      <c r="N74" s="6" t="s">
+      <c r="F75" s="6" t="s">
         <v>748</v>
       </c>
-      <c r="O74" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A75" s="5" t="s">
+      <c r="G75" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H75" s="6" t="s">
+        <v>708</v>
+      </c>
+      <c r="I75" s="6" t="s">
         <v>749</v>
       </c>
-      <c r="B75" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C75" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D75" s="6" t="s">
+      <c r="J75" s="6" t="s">
         <v>750</v>
       </c>
-      <c r="E75" s="6" t="s">
+      <c r="K75" s="6" t="s">
         <v>751</v>
       </c>
-      <c r="F75" s="6" t="s">
+      <c r="L75" s="6" t="s">
         <v>752</v>
       </c>
-      <c r="G75" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H75" s="6" t="s">
+      <c r="M75" s="6" t="s">
         <v>753</v>
       </c>
-      <c r="I75" s="6" t="s">
+      <c r="N75" s="6" t="s">
         <v>754</v>
-      </c>
-      <c r="J75" s="6" t="s">
-        <v>755</v>
-      </c>
-      <c r="K75" s="6" t="s">
-        <v>756</v>
-      </c>
-      <c r="L75" s="6" t="s">
-        <v>757</v>
-      </c>
-      <c r="M75" s="6" t="s">
-        <v>758</v>
-      </c>
-      <c r="N75" s="6" t="s">
-        <v>759</v>
       </c>
       <c r="O75" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>25</v>
+        <v>530</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>762</v>
+        <v>757</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>763</v>
+        <v>758</v>
       </c>
       <c r="G76" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>255</v>
+        <v>759</v>
       </c>
       <c r="I76" s="6" t="s">
+        <v>760</v>
+      </c>
+      <c r="J76" s="6" t="s">
+        <v>761</v>
+      </c>
+      <c r="K76" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="L76" s="6" t="s">
+        <v>763</v>
+      </c>
+      <c r="M76" s="6" t="s">
         <v>764</v>
       </c>
-      <c r="J76" s="6" t="s">
+      <c r="N76" s="6" t="s">
         <v>765</v>
-      </c>
-      <c r="K76" s="6" t="s">
-        <v>766</v>
-      </c>
-      <c r="L76" s="6" t="s">
-        <v>767</v>
-      </c>
-      <c r="M76" s="6" t="s">
-        <v>768</v>
-      </c>
-      <c r="N76" s="6" t="s">
-        <v>759</v>
       </c>
       <c r="O76" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C77" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D77" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>769</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H77" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I77" s="6" t="s">
         <v>770</v>
       </c>
-      <c r="E77" s="6" t="s">
+      <c r="J77" s="6" t="s">
         <v>771</v>
       </c>
-      <c r="F77" s="6" t="s">
+      <c r="K77" s="6" t="s">
         <v>772</v>
       </c>
-      <c r="G77" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H77" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="I77" s="6" t="s">
+      <c r="L77" s="6" t="s">
         <v>773</v>
       </c>
-      <c r="J77" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="K77" s="6" t="s">
+      <c r="M77" s="6" t="s">
         <v>774</v>
       </c>
-      <c r="L77" s="6" t="s">
-        <v>775</v>
-      </c>
-      <c r="M77" s="6" t="s">
-        <v>271</v>
-      </c>
       <c r="N77" s="6" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="O77" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
+        <v>775</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" s="6" t="s">
         <v>776</v>
       </c>
-      <c r="B78" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C78" s="6" t="s">
-        <v>524</v>
-      </c>
-      <c r="D78" s="6" t="s">
+      <c r="E78" s="6" t="s">
         <v>777</v>
       </c>
-      <c r="E78" s="6" t="s">
+      <c r="F78" s="6" t="s">
         <v>778</v>
       </c>
-      <c r="F78" s="6" t="s">
+      <c r="G78" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="I78" s="6" t="s">
         <v>779</v>
       </c>
-      <c r="G78" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="I78" s="6" t="s">
+      <c r="J78" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="K78" s="6" t="s">
         <v>780</v>
       </c>
-      <c r="J78" s="6" t="s">
+      <c r="L78" s="6" t="s">
         <v>781</v>
       </c>
-      <c r="K78" s="6" t="s">
-        <v>782</v>
-      </c>
-      <c r="L78" s="6" t="s">
-        <v>783</v>
-      </c>
       <c r="M78" s="6" t="s">
-        <v>784</v>
+        <v>271</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>759</v>
+        <v>765</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
+        <v>782</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C79" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>783</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>784</v>
+      </c>
+      <c r="F79" s="6" t="s">
         <v>785</v>
       </c>
-      <c r="B79" s="6" t="s">
-        <v>511</v>
-      </c>
-      <c r="C79" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D79" s="6" t="s">
+      <c r="G79" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H79" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="I79" s="6" t="s">
         <v>786</v>
       </c>
-      <c r="E79" s="6" t="s">
+      <c r="J79" s="6" t="s">
         <v>787</v>
       </c>
-      <c r="F79" s="6" t="s">
+      <c r="K79" s="6" t="s">
         <v>788</v>
       </c>
-      <c r="G79" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H79" s="6" t="s">
-        <v>330</v>
-      </c>
-      <c r="I79" s="6" t="s">
+      <c r="L79" s="6" t="s">
         <v>789</v>
       </c>
-      <c r="J79" s="6" t="s">
+      <c r="M79" s="6" t="s">
         <v>790</v>
       </c>
-      <c r="K79" s="6" t="s">
-        <v>791</v>
-      </c>
-      <c r="L79" s="6" t="s">
-        <v>792</v>
-      </c>
-      <c r="M79" s="6" t="s">
-        <v>793</v>
-      </c>
       <c r="N79" s="6" t="s">
-        <v>794</v>
+        <v>765</v>
       </c>
       <c r="O79" s="6" t="s">
         <v>37</v>
@@ -7438,48 +7494,95 @@
     </row>
     <row r="80" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
-        <v>795</v>
+        <v>791</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="C80" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D80" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="E80" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="F80" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="G80" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H80" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>795</v>
+      </c>
+      <c r="J80" s="6" t="s">
+        <v>796</v>
+      </c>
+      <c r="K80" s="6" t="s">
+        <v>797</v>
+      </c>
+      <c r="L80" s="6" t="s">
+        <v>798</v>
+      </c>
+      <c r="M80" s="6" t="s">
+        <v>799</v>
+      </c>
+      <c r="N80" s="6" t="s">
+        <v>800</v>
+      </c>
+      <c r="O80" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A81" s="5" t="s">
+        <v>801</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D81" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E80" s="6" t="s">
-        <v>796</v>
-      </c>
-      <c r="F80" s="6" t="s">
-        <v>797</v>
-      </c>
-      <c r="G80" s="7" t="s">
+      <c r="E81" s="6" t="s">
+        <v>802</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>803</v>
+      </c>
+      <c r="G81" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H80" s="6" t="s">
+      <c r="H81" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I80" s="6" t="s">
-        <v>798</v>
-      </c>
-      <c r="J80" s="6" t="s">
-        <v>799</v>
-      </c>
-      <c r="K80" s="6" t="s">
+      <c r="I81" s="6" t="s">
+        <v>804</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="K81" s="6" t="s">
+        <v>806</v>
+      </c>
+      <c r="L81" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="M81" s="6" t="s">
+        <v>808</v>
+      </c>
+      <c r="N81" s="6" t="s">
         <v>800</v>
       </c>
-      <c r="L80" s="6" t="s">
-        <v>801</v>
-      </c>
-      <c r="M80" s="6" t="s">
-        <v>802</v>
-      </c>
-      <c r="N80" s="6" t="s">
-        <v>794</v>
-      </c>
-      <c r="O80" s="6" t="s">
+      <c r="O81" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7516,7 +7619,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -7537,7 +7640,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>803</v>
+        <v>809</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7584,7 +7687,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>546</v>
+        <v>552</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -7605,7 +7708,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>591</v>
+        <v>597</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -7626,7 +7729,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -7710,7 +7813,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>516</v>
+        <v>522</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7773,7 +7876,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>753</v>
+        <v>759</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7794,7 +7897,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
       <c r="B14" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A14,'Bug List'!$G:$G,"Cao")</f>
@@ -7836,7 +7939,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
@@ -7878,7 +7981,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B18" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A18,'Bug List'!$G:$G,"Cao")</f>
@@ -7962,7 +8065,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -8004,7 +8107,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="B24" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A24,'Bug List'!$G:$G,"Cao")</f>
@@ -8172,7 +8275,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>627</v>
+        <v>633</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
@@ -8193,7 +8296,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Cao")</f>
@@ -8214,7 +8317,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>222</v>
+        <v>509</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Cao")</f>
@@ -8235,15 +8338,15 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Thấp")</f>
@@ -8256,7 +8359,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Cao")</f>
@@ -8264,7 +8367,7 @@
       </c>
       <c r="C36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Thấp")</f>
@@ -8272,16 +8375,16 @@
       </c>
       <c r="E36" s="12" t="n">
         <f aca="false">SUM(B36:D36)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>276</v>
+        <v>160</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Trung")</f>
@@ -8293,79 +8396,100 @@
       </c>
       <c r="E37" s="12" t="n">
         <f aca="false">SUM(B37:D37)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B38" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
-        <v>803</v>
-      </c>
-      <c r="B38" s="12" t="n">
-        <f aca="false">SUM(B2:B37)</f>
+      <c r="D38" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="12" t="n">
+        <f aca="false">SUM(B38:D38)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="12" t="s">
+        <v>809</v>
+      </c>
+      <c r="B39" s="12" t="n">
+        <f aca="false">SUM(B2:B38)</f>
         <v>24</v>
       </c>
-      <c r="C38" s="12" t="n">
-        <f aca="false">SUM(C2:C37)</f>
-        <v>34</v>
-      </c>
-      <c r="D38" s="12" t="n">
-        <f aca="false">SUM(D2:D37)</f>
+      <c r="C39" s="12" t="n">
+        <f aca="false">SUM(C2:C38)</f>
+        <v>35</v>
+      </c>
+      <c r="D39" s="12" t="n">
+        <f aca="false">SUM(D2:D38)</f>
         <v>21</v>
       </c>
-      <c r="E38" s="12" t="n">
-        <f aca="false">SUM(E2:E37)</f>
-        <v>79</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="s">
+      <c r="E39" s="12" t="n">
+        <f aca="false">SUM(E2:E38)</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B40" s="12" t="s">
-        <v>804</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11" t="s">
-        <v>805</v>
-      </c>
-      <c r="B41" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A41)</f>
-        <v>0</v>
+      <c r="B41" s="12" t="s">
+        <v>810</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="11" t="s">
-        <v>444</v>
+        <v>811</v>
       </c>
       <c r="B42" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A42)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
-        <v>77</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
-        <v>806</v>
+        <v>37</v>
       </c>
       <c r="B44" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A44)</f>
+        <v>78</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11" t="s">
+        <v>812</v>
+      </c>
+      <c r="B45" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A45)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="13" t="s">
-        <v>807</v>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="13" t="s">
+        <v>813</v>
       </c>
     </row>
   </sheetData>
@@ -8393,170 +8517,170 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>808</v>
+        <v>814</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>809</v>
+        <v>815</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>810</v>
+        <v>816</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>811</v>
+        <v>817</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="14" t="s">
-        <v>812</v>
+      <c r="A4" s="12" t="s">
+        <v>818</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>813</v>
+        <v>819</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="12" t="s">
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>814</v>
+        <v>820</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="14" t="s">
-        <v>815</v>
+      <c r="A6" s="12" t="s">
+        <v>821</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>816</v>
+        <v>822</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="14" t="s">
-        <v>817</v>
+      <c r="A7" s="12" t="s">
+        <v>823</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>818</v>
+        <v>824</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="14" t="s">
-        <v>819</v>
+      <c r="A8" s="12" t="s">
+        <v>825</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>820</v>
+        <v>826</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>821</v>
+      <c r="A9" s="12" t="s">
+        <v>827</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>822</v>
+        <v>828</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="14" t="s">
-        <v>823</v>
+      <c r="A10" s="12" t="s">
+        <v>829</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>824</v>
+        <v>830</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>825</v>
+      <c r="A11" s="12" t="s">
+        <v>831</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>826</v>
+        <v>832</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>827</v>
+      <c r="A12" s="12" t="s">
+        <v>833</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>828</v>
+        <v>834</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="14" t="s">
-        <v>829</v>
+      <c r="A13" s="12" t="s">
+        <v>835</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>830</v>
+        <v>836</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
-        <v>831</v>
+      <c r="A14" s="12" t="s">
+        <v>837</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>832</v>
+        <v>838</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="14" t="s">
-        <v>833</v>
+      <c r="A15" s="12" t="s">
+        <v>839</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>834</v>
+        <v>840</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
-        <v>835</v>
+      <c r="A16" s="12" t="s">
+        <v>841</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>836</v>
+        <v>842</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
+      <c r="A17" s="12" t="s">
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>837</v>
+        <v>843</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>838</v>
+      <c r="A18" s="12" t="s">
+        <v>844</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>839</v>
+        <v>845</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>840</v>
+      <c r="A19" s="12" t="s">
+        <v>846</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>841</v>
+        <v>847</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="14" t="s">
-        <v>842</v>
+      <c r="A20" s="12" t="s">
+        <v>848</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>843</v>
+        <v>849</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="A21" s="12" t="s">
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>844</v>
+        <v>850</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update channel back to 1.7.85: speaker module off main; CI reuses any earlier release with the same app
Owner's decision (06/10/2026): the shop stays on 1.7.85 until the speaker module is tested. With 9faa2bf reverted
the app inputs are 072bd6da26eec7eb again, the ones of android-v1085; the release step now looks through the recent
releases for those inputs instead of only the newest, so the signed 1.7.85 APK goes back on the update channel
rather than a rebuild under a new version. Bug list: PT-48 back to Đang làm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -1989,7 +1989,7 @@
     <t xml:space="preserve">Thông báo cần chạy khi người dùng đang ở màn hình nào, và khi màn hình/app tắt thì sao? Bật lại sau khi tắt có đọc lại việc cũ không? Máy thật có giọng đọc của ngôn ngữ cần không (Android 11+ phải khai báo TTS_SERVICE)?</t>
   </si>
   <si>
-    <t xml:space="preserve">9faa2bf</t>
+    <t xml:space="preserve">9faa2bf (đã lên 1.7.90 rồi gỡ khỏi main bằng 026853f theo yêu cầu chủ tiệm 06/10; máy khách giữ 1.7.85; làm tiếp trên nhánh online-v1.7)</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-01</t>
@@ -6079,7 +6079,7 @@
         <v>515</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8474,7 +8474,7 @@
       </c>
       <c r="B44" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A44)</f>
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Bug list: PT-49 issues the speaker cross-check found; PT-48 done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1315" uniqueCount="851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="862">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -1989,7 +1989,40 @@
     <t xml:space="preserve">Thông báo cần chạy khi người dùng đang ở màn hình nào, và khi màn hình/app tắt thì sao? Bật lại sau khi tắt có đọc lại việc cũ không? Máy thật có giọng đọc của ngôn ngữ cần không (Android 11+ phải khai báo TTS_SERVICE)?</t>
   </si>
   <si>
-    <t xml:space="preserve">9faa2bf (đã lên 1.7.90 rồi gỡ khỏi main bằng 026853f theo yêu cầu chủ tiệm 06/10; máy khách giữ 1.7.85; làm tiếp trên nhánh online-v1.7)</t>
+    <t xml:space="preserve">9faa2bf, f093645 (gỡ khỏi main ngày 06/10 bằng 026853f; đưa lại production 14/10 theo yêu cầu chủ tiệm sau 69 case kiểm chéo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js (say, speakerOut, pollService, scheduler/realtime); android MainActivity.java (audioOutput); scripts/sim-announce.mjs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Máy SUNMI ghép loa Bluetooth và trình duyệt (thử trước khi giao quán)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thông báo / đồng bộ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bộ kiểm chéo 69 case của module loa (PT-48) tìm ra: (1) chỉ đọc yêu cầu gọi nhân viên đầu tiên trong danh sách, yêu cầu mới bị bỏ qua nếu có yêu cầu cũ còn treo; (2) có mạng lại hoặc server hết lỗi thì đơn mới vẫn bị báo trễ 1–2 phút; (3) máy chưa nối loa vẫn phát bằng loa máy (rè); (4) tab trình duyệt bị ẩn thì không báo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1) pollService chỉ xét requests[0]; (2) lịch chạy giữ thời gian chờ lùi của các lần lỗi trước và realtime nối lại theo backoff, cả khi mạng/server đã ổn; (3) không có cách biết máy đang có loa ngoài; (4) tab ẩn đóng realtime và tắt mọi tác vụ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1) Đọc mọi yêu cầu chưa đọc (serviceSeen). (2) Sự kiện online xóa backoff và nối realtime ngay; tin realtime xóa backoff của bộ theo dõi đơn. (3) APK báo audioOutput (Bluetooth/có dây/USB); không có loa ngoài thì chỉ hiện chữ "chưa kết nối loa", Cài đặt hiện trạng thái loa. (4) Khi loa bật, tab ẩn vẫn giữ realtime và bộ theo dõi; tắt thì đóng như cũ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-announce.mjs (npm run test:announce, job CI speaker): 69 case A1–I1, gồm B16 gọi nhân viên, C1–C6 loa ngắt/nối lại, F1–F3 mạng/server, G3–G4 tab ẩn; tests/phattai-v184-announce.test.mjs: "PT-49 plays only through a connected speaker; every service call; no stale backoff…".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thông báo có xét hết danh sách hay chỉ phần tử đầu? Sau lỗi mạng/server, thời gian chờ lùi có làm trễ việc khẩn không? Âm thanh có phát ra đúng thiết bị người dùng muốn không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f093645</t>
   </si>
   <si>
     <t xml:space="preserve">SAAS-01</t>
@@ -3316,7 +3349,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3361,15 +3394,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3495,8 +3532,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O81" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O81"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O82"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3759,7 +3796,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O81"/>
+  <dimension ref="A1:O82"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -6079,10 +6116,10 @@
         <v>515</v>
       </c>
       <c r="O49" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>516</v>
       </c>
@@ -6090,69 +6127,69 @@
         <v>517</v>
       </c>
       <c r="C50" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="E50" s="6" t="s">
         <v>518</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="F50" s="6" t="s">
         <v>519</v>
       </c>
-      <c r="E50" s="6" t="s">
+      <c r="G50" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H50" s="6" t="s">
         <v>520</v>
       </c>
-      <c r="F50" s="6" t="s">
+      <c r="I50" s="6" t="s">
         <v>521</v>
       </c>
-      <c r="G50" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H50" s="6" t="s">
+      <c r="J50" s="6" t="s">
         <v>522</v>
       </c>
-      <c r="I50" s="6" t="s">
+      <c r="K50" s="6" t="s">
         <v>523</v>
       </c>
-      <c r="J50" s="6" t="s">
+      <c r="L50" s="6" t="s">
         <v>524</v>
       </c>
-      <c r="K50" s="6" t="s">
+      <c r="M50" s="6" t="s">
         <v>525</v>
       </c>
-      <c r="L50" s="6" t="s">
+      <c r="N50" s="6" t="s">
         <v>526</v>
-      </c>
-      <c r="M50" s="6" t="s">
-        <v>527</v>
-      </c>
-      <c r="N50" s="6" t="s">
-        <v>528</v>
       </c>
       <c r="O50" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
+        <v>527</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="B51" s="6" t="s">
-        <v>517</v>
-      </c>
-      <c r="C51" s="6" t="s">
+      <c r="D51" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>531</v>
       </c>
-      <c r="E51" s="6" t="s">
+      <c r="F51" s="6" t="s">
         <v>532</v>
       </c>
-      <c r="F51" s="6" t="s">
+      <c r="G51" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H51" s="6" t="s">
         <v>533</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H51" s="6" t="s">
-        <v>522</v>
       </c>
       <c r="I51" s="6" t="s">
         <v>534</v>
@@ -6170,54 +6207,54 @@
         <v>538</v>
       </c>
       <c r="N51" s="6" t="s">
-        <v>528</v>
+        <v>539</v>
       </c>
       <c r="O51" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
+        <v>540</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>544</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="J52" s="6" t="s">
+        <v>546</v>
+      </c>
+      <c r="K52" s="6" t="s">
+        <v>547</v>
+      </c>
+      <c r="L52" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="M52" s="6" t="s">
+        <v>549</v>
+      </c>
+      <c r="N52" s="6" t="s">
         <v>539</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>517</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>530</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>541</v>
-      </c>
-      <c r="F52" s="6" t="s">
-        <v>542</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>522</v>
-      </c>
-      <c r="I52" s="6" t="s">
-        <v>543</v>
-      </c>
-      <c r="J52" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="K52" s="6" t="s">
-        <v>545</v>
-      </c>
-      <c r="L52" s="6" t="s">
-        <v>546</v>
-      </c>
-      <c r="M52" s="6" t="s">
-        <v>547</v>
-      </c>
-      <c r="N52" s="6" t="s">
-        <v>548</v>
       </c>
       <c r="O52" s="6" t="s">
         <v>37</v>
@@ -6225,140 +6262,140 @@
     </row>
     <row r="53" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="5" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>146</v>
+        <v>551</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="G53" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H53" s="6" t="s">
-        <v>552</v>
+        <v>533</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="J53" s="6" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="K53" s="6" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="L53" s="6" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="M53" s="6" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="N53" s="6" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="O53" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>560</v>
+        <v>146</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>561</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>551</v>
+        <v>562</v>
       </c>
       <c r="G54" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="I54" s="6" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="J54" s="6" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="K54" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="L54" s="6" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="M54" s="6" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="O54" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="E55" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="F55" s="6" t="s">
+        <v>562</v>
+      </c>
+      <c r="G55" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>573</v>
+      </c>
+      <c r="J55" s="6" t="s">
+        <v>574</v>
+      </c>
+      <c r="K55" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="L55" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="M55" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="N55" s="6" t="s">
         <v>569</v>
-      </c>
-      <c r="F55" s="6" t="s">
-        <v>570</v>
-      </c>
-      <c r="G55" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H55" s="6" t="s">
-        <v>552</v>
-      </c>
-      <c r="I55" s="6" t="s">
-        <v>571</v>
-      </c>
-      <c r="J55" s="6" t="s">
-        <v>572</v>
-      </c>
-      <c r="K55" s="6" t="s">
-        <v>573</v>
-      </c>
-      <c r="L55" s="6" t="s">
-        <v>574</v>
-      </c>
-      <c r="M55" s="6" t="s">
-        <v>575</v>
-      </c>
-      <c r="N55" s="6" t="s">
-        <v>558</v>
       </c>
       <c r="O55" s="6" t="s">
         <v>37</v>
@@ -6366,122 +6403,122 @@
     </row>
     <row r="56" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>80</v>
+        <v>579</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="F56" s="6" t="s">
-        <v>551</v>
-      </c>
-      <c r="G56" s="8" t="s">
-        <v>52</v>
+        <v>581</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="I56" s="6" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="J56" s="6" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="K56" s="6" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="L56" s="6" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="M56" s="6" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>558</v>
+        <v>569</v>
       </c>
       <c r="O56" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>584</v>
+        <v>80</v>
       </c>
       <c r="E57" s="6" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="F57" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="G57" s="9" t="s">
-        <v>73</v>
+        <v>562</v>
+      </c>
+      <c r="G57" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H57" s="6" t="s">
-        <v>372</v>
+        <v>563</v>
       </c>
       <c r="I57" s="6" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="J57" s="6" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="K57" s="6" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="L57" s="6" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="M57" s="6" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="N57" s="6" t="s">
-        <v>592</v>
+        <v>569</v>
       </c>
       <c r="O57" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>597</v>
+        <v>372</v>
       </c>
       <c r="I58" s="6" t="s">
         <v>598</v>
@@ -6499,265 +6536,265 @@
         <v>602</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>592</v>
+        <v>603</v>
       </c>
       <c r="O58" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="5" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="F59" s="6" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="G59" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H59" s="6" t="s">
-        <v>53</v>
+        <v>608</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="J59" s="6" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="K59" s="6" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="L59" s="6" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="M59" s="6" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="N59" s="6" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
       <c r="O59" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>604</v>
+        <v>615</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G60" s="7" t="s">
-        <v>29</v>
+        <v>617</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="J60" s="6" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="K60" s="6" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="L60" s="6" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="M60" s="6" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>612</v>
+        <v>623</v>
       </c>
       <c r="O60" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>621</v>
+        <v>615</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="F61" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H61" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="I61" s="6" t="s">
+        <v>626</v>
+      </c>
+      <c r="J61" s="6" t="s">
+        <v>627</v>
+      </c>
+      <c r="K61" s="6" t="s">
+        <v>628</v>
+      </c>
+      <c r="L61" s="6" t="s">
+        <v>629</v>
+      </c>
+      <c r="M61" s="6" t="s">
+        <v>630</v>
+      </c>
+      <c r="N61" s="6" t="s">
         <v>623</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H61" s="6" t="s">
-        <v>522</v>
-      </c>
-      <c r="I61" s="6" t="s">
-        <v>624</v>
-      </c>
-      <c r="J61" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="K61" s="6" t="s">
-        <v>626</v>
-      </c>
-      <c r="L61" s="6" t="s">
-        <v>627</v>
-      </c>
-      <c r="M61" s="6" t="s">
-        <v>628</v>
-      </c>
-      <c r="N61" s="6" t="s">
-        <v>592</v>
       </c>
       <c r="O61" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="G62" s="9" t="s">
         <v>73</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>633</v>
+        <v>533</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="J62" s="6" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="K62" s="6" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="L62" s="6" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="M62" s="6" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>639</v>
+        <v>603</v>
       </c>
       <c r="O62" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
         <v>640</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>338</v>
+        <v>641</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="G63" s="8" t="s">
-        <v>52</v>
+        <v>643</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H63" s="6" t="s">
-        <v>149</v>
+        <v>644</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="J63" s="6" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="K63" s="6" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="L63" s="6" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="M63" s="6" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="N63" s="6" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="O63" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>518</v>
+        <v>541</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>146</v>
+        <v>338</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>650</v>
+        <v>211</v>
       </c>
       <c r="G64" s="8" t="s">
         <v>52</v>
@@ -6766,69 +6803,69 @@
         <v>149</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="J64" s="6" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="K64" s="6" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="L64" s="6" t="s">
-        <v>610</v>
+        <v>656</v>
       </c>
       <c r="M64" s="6" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="N64" s="6" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="O64" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>306</v>
+        <v>146</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>307</v>
+        <v>660</v>
       </c>
       <c r="F65" s="6" t="s">
-        <v>657</v>
-      </c>
-      <c r="G65" s="9" t="s">
-        <v>73</v>
+        <v>661</v>
+      </c>
+      <c r="G65" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H65" s="6" t="s">
-        <v>309</v>
+        <v>149</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="J65" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="K65" s="6" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="L65" s="6" t="s">
-        <v>661</v>
+        <v>621</v>
       </c>
       <c r="M65" s="6" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="N65" s="6" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="O65" s="6" t="s">
         <v>37</v>
@@ -6836,154 +6873,154 @@
     </row>
     <row r="66" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>435</v>
+        <v>306</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>665</v>
+        <v>307</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>666</v>
-      </c>
-      <c r="G66" s="8" t="s">
-        <v>52</v>
+        <v>668</v>
+      </c>
+      <c r="G66" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>361</v>
+        <v>309</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="J66" s="6" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="K66" s="6" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="L66" s="6" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="M66" s="6" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="N66" s="6" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="O66" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>674</v>
+        <v>435</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="G67" s="8" t="s">
         <v>52</v>
       </c>
       <c r="H67" s="6" t="s">
-        <v>552</v>
+        <v>361</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="J67" s="6" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="K67" s="6" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="L67" s="6" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="M67" s="6" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="N67" s="6" t="s">
-        <v>672</v>
+        <v>683</v>
       </c>
       <c r="O67" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D68" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="F68" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H68" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="I68" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="J68" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="K68" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="L68" s="6" t="s">
+        <v>691</v>
+      </c>
+      <c r="M68" s="6" t="s">
+        <v>692</v>
+      </c>
+      <c r="N68" s="6" t="s">
         <v>683</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>684</v>
-      </c>
-      <c r="F68" s="6" t="s">
-        <v>685</v>
-      </c>
-      <c r="G68" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H68" s="6" t="s">
-        <v>686</v>
-      </c>
-      <c r="I68" s="6" t="s">
-        <v>687</v>
-      </c>
-      <c r="J68" s="6" t="s">
-        <v>688</v>
-      </c>
-      <c r="K68" s="6" t="s">
-        <v>689</v>
-      </c>
-      <c r="L68" s="6" t="s">
-        <v>690</v>
-      </c>
-      <c r="M68" s="6" t="s">
-        <v>691</v>
-      </c>
-      <c r="N68" s="6" t="s">
-        <v>692</v>
       </c>
       <c r="O68" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
         <v>693</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D69" s="6" t="s">
         <v>694</v>
@@ -7022,15 +7059,15 @@
         <v>37</v>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
         <v>704</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D70" s="6" t="s">
         <v>705</v>
@@ -7041,8 +7078,8 @@
       <c r="F70" s="6" t="s">
         <v>707</v>
       </c>
-      <c r="G70" s="8" t="s">
-        <v>52</v>
+      <c r="G70" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H70" s="6" t="s">
         <v>708</v>
@@ -7069,15 +7106,15 @@
         <v>37</v>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="5" t="s">
         <v>715</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D71" s="6" t="s">
         <v>716</v>
@@ -7088,76 +7125,76 @@
       <c r="F71" s="6" t="s">
         <v>718</v>
       </c>
-      <c r="G71" s="9" t="s">
-        <v>73</v>
+      <c r="G71" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="H71" s="6" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="J71" s="6" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="K71" s="6" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="L71" s="6" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="M71" s="6" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="N71" s="6" t="s">
-        <v>703</v>
+        <v>725</v>
       </c>
       <c r="O71" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>295</v>
+        <v>727</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>296</v>
+        <v>728</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="G72" s="7" t="s">
-        <v>29</v>
+        <v>729</v>
+      </c>
+      <c r="G72" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H72" s="6" t="s">
-        <v>298</v>
+        <v>719</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>299</v>
+        <v>730</v>
       </c>
       <c r="J72" s="6" t="s">
-        <v>300</v>
+        <v>731</v>
       </c>
       <c r="K72" s="6" t="s">
-        <v>725</v>
+        <v>732</v>
       </c>
       <c r="L72" s="6" t="s">
-        <v>726</v>
+        <v>733</v>
       </c>
       <c r="M72" s="6" t="s">
-        <v>727</v>
+        <v>734</v>
       </c>
       <c r="N72" s="6" t="s">
-        <v>703</v>
+        <v>714</v>
       </c>
       <c r="O72" s="6" t="s">
         <v>37</v>
@@ -7165,169 +7202,169 @@
     </row>
     <row r="73" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>728</v>
+        <v>735</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>729</v>
+        <v>295</v>
       </c>
       <c r="E73" s="6" t="s">
-        <v>730</v>
+        <v>296</v>
       </c>
       <c r="F73" s="6" t="s">
-        <v>731</v>
+        <v>297</v>
       </c>
       <c r="G73" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H73" s="6" t="s">
-        <v>708</v>
+        <v>298</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>732</v>
+        <v>299</v>
       </c>
       <c r="J73" s="6" t="s">
-        <v>733</v>
+        <v>300</v>
       </c>
       <c r="K73" s="6" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="L73" s="6" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="M73" s="6" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="N73" s="6" t="s">
-        <v>737</v>
+        <v>714</v>
       </c>
       <c r="O73" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="5" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>435</v>
+        <v>740</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>665</v>
+        <v>741</v>
       </c>
       <c r="F74" s="6" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="G74" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H74" s="6" t="s">
-        <v>361</v>
+        <v>719</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="J74" s="6" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="K74" s="6" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="M74" s="6" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="N74" s="6" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="O74" s="6" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>729</v>
+        <v>435</v>
       </c>
       <c r="E75" s="6" t="s">
-        <v>747</v>
+        <v>676</v>
       </c>
       <c r="F75" s="6" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="G75" s="7" t="s">
         <v>29</v>
       </c>
       <c r="H75" s="6" t="s">
-        <v>708</v>
+        <v>361</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="J75" s="6" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="K75" s="6" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="L75" s="6" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="M75" s="6" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="N75" s="6" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="O75" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>530</v>
+        <v>541</v>
       </c>
       <c r="D76" s="6" t="s">
-        <v>756</v>
+        <v>740</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="F76" s="6" t="s">
-        <v>758</v>
-      </c>
-      <c r="G76" s="8" t="s">
-        <v>52</v>
+        <v>759</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H76" s="6" t="s">
-        <v>759</v>
+        <v>719</v>
       </c>
       <c r="I76" s="6" t="s">
         <v>760</v>
@@ -7351,15 +7388,15 @@
         <v>37</v>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="5" t="s">
         <v>766</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>25</v>
+        <v>541</v>
       </c>
       <c r="D77" s="6" t="s">
         <v>767</v>
@@ -7374,166 +7411,166 @@
         <v>52</v>
       </c>
       <c r="H77" s="6" t="s">
-        <v>255</v>
+        <v>770</v>
       </c>
       <c r="I77" s="6" t="s">
-        <v>770</v>
+        <v>771</v>
       </c>
       <c r="J77" s="6" t="s">
-        <v>771</v>
+        <v>772</v>
       </c>
       <c r="K77" s="6" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="L77" s="6" t="s">
-        <v>773</v>
+        <v>774</v>
       </c>
       <c r="M77" s="6" t="s">
-        <v>774</v>
+        <v>775</v>
       </c>
       <c r="N77" s="6" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
       <c r="O77" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C78" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D78" s="6" t="s">
+        <v>778</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>779</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>780</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H78" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>781</v>
+      </c>
+      <c r="J78" s="6" t="s">
+        <v>782</v>
+      </c>
+      <c r="K78" s="6" t="s">
+        <v>783</v>
+      </c>
+      <c r="L78" s="6" t="s">
+        <v>784</v>
+      </c>
+      <c r="M78" s="6" t="s">
+        <v>785</v>
+      </c>
+      <c r="N78" s="6" t="s">
         <v>776</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>777</v>
-      </c>
-      <c r="F78" s="6" t="s">
-        <v>778</v>
-      </c>
-      <c r="G78" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="I78" s="6" t="s">
-        <v>779</v>
-      </c>
-      <c r="J78" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="K78" s="6" t="s">
-        <v>780</v>
-      </c>
-      <c r="L78" s="6" t="s">
-        <v>781</v>
-      </c>
-      <c r="M78" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="N78" s="6" t="s">
-        <v>765</v>
       </c>
       <c r="O78" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="5" t="s">
-        <v>782</v>
+        <v>786</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C79" s="6" t="s">
-        <v>530</v>
+        <v>25</v>
       </c>
       <c r="D79" s="6" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="F79" s="6" t="s">
-        <v>785</v>
-      </c>
-      <c r="G79" s="7" t="s">
-        <v>29</v>
+        <v>789</v>
+      </c>
+      <c r="G79" s="9" t="s">
+        <v>73</v>
       </c>
       <c r="H79" s="6" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="I79" s="6" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="J79" s="6" t="s">
-        <v>787</v>
+        <v>268</v>
       </c>
       <c r="K79" s="6" t="s">
-        <v>788</v>
+        <v>791</v>
       </c>
       <c r="L79" s="6" t="s">
-        <v>789</v>
+        <v>792</v>
       </c>
       <c r="M79" s="6" t="s">
-        <v>790</v>
+        <v>271</v>
       </c>
       <c r="N79" s="6" t="s">
-        <v>765</v>
+        <v>776</v>
       </c>
       <c r="O79" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>25</v>
+        <v>541</v>
       </c>
       <c r="D80" s="6" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="F80" s="6" t="s">
-        <v>794</v>
-      </c>
-      <c r="G80" s="8" t="s">
-        <v>52</v>
+        <v>796</v>
+      </c>
+      <c r="G80" s="7" t="s">
+        <v>29</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>330</v>
+        <v>276</v>
       </c>
       <c r="I80" s="6" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="J80" s="6" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="K80" s="6" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="L80" s="6" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="M80" s="6" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>800</v>
+        <v>776</v>
       </c>
       <c r="O80" s="6" t="s">
         <v>37</v>
@@ -7541,48 +7578,95 @@
     </row>
     <row r="81" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="s">
-        <v>801</v>
+        <v>802</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>517</v>
+        <v>528</v>
       </c>
       <c r="C81" s="6" t="s">
         <v>25</v>
       </c>
       <c r="D81" s="6" t="s">
+        <v>803</v>
+      </c>
+      <c r="E81" s="6" t="s">
+        <v>804</v>
+      </c>
+      <c r="F81" s="6" t="s">
+        <v>805</v>
+      </c>
+      <c r="G81" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H81" s="6" t="s">
+        <v>330</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>806</v>
+      </c>
+      <c r="J81" s="6" t="s">
+        <v>807</v>
+      </c>
+      <c r="K81" s="6" t="s">
+        <v>808</v>
+      </c>
+      <c r="L81" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="M81" s="6" t="s">
+        <v>810</v>
+      </c>
+      <c r="N81" s="6" t="s">
+        <v>811</v>
+      </c>
+      <c r="O81" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>528</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D82" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E81" s="6" t="s">
-        <v>802</v>
-      </c>
-      <c r="F81" s="6" t="s">
-        <v>803</v>
-      </c>
-      <c r="G81" s="7" t="s">
+      <c r="E82" s="6" t="s">
+        <v>813</v>
+      </c>
+      <c r="F82" s="6" t="s">
+        <v>814</v>
+      </c>
+      <c r="G82" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="H81" s="6" t="s">
+      <c r="H82" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="I81" s="6" t="s">
-        <v>804</v>
-      </c>
-      <c r="J81" s="6" t="s">
-        <v>805</v>
-      </c>
-      <c r="K81" s="6" t="s">
-        <v>806</v>
-      </c>
-      <c r="L81" s="6" t="s">
-        <v>807</v>
-      </c>
-      <c r="M81" s="6" t="s">
-        <v>808</v>
-      </c>
-      <c r="N81" s="6" t="s">
-        <v>800</v>
-      </c>
-      <c r="O81" s="6" t="s">
+      <c r="I82" s="6" t="s">
+        <v>815</v>
+      </c>
+      <c r="J82" s="6" t="s">
+        <v>816</v>
+      </c>
+      <c r="K82" s="6" t="s">
+        <v>817</v>
+      </c>
+      <c r="L82" s="6" t="s">
+        <v>818</v>
+      </c>
+      <c r="M82" s="6" t="s">
+        <v>819</v>
+      </c>
+      <c r="N82" s="6" t="s">
+        <v>811</v>
+      </c>
+      <c r="O82" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7619,7 +7703,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -7640,7 +7724,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>809</v>
+        <v>820</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7687,7 +7771,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>552</v>
+        <v>563</v>
       </c>
       <c r="B4" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A4,'Bug List'!$G:$G,"Cao")</f>
@@ -7708,7 +7792,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>597</v>
+        <v>608</v>
       </c>
       <c r="B5" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A5,'Bug List'!$G:$G,"Cao")</f>
@@ -7729,7 +7813,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="s">
-        <v>686</v>
+        <v>697</v>
       </c>
       <c r="B6" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A6,'Bug List'!$G:$G,"Cao")</f>
@@ -7813,7 +7897,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>522</v>
+        <v>533</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A10,'Bug List'!$G:$G,"Cao")</f>
@@ -7876,7 +7960,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>759</v>
+        <v>770</v>
       </c>
       <c r="B13" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A13,'Bug List'!$G:$G,"Cao")</f>
@@ -7939,7 +8023,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>697</v>
+        <v>708</v>
       </c>
       <c r="B16" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A16,'Bug List'!$G:$G,"Cao")</f>
@@ -8065,7 +8149,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
       <c r="B22" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A22,'Bug List'!$G:$G,"Cao")</f>
@@ -8275,7 +8359,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
@@ -8338,7 +8422,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>222</v>
+        <v>520</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Cao")</f>
@@ -8359,15 +8443,15 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Thấp")</f>
@@ -8380,7 +8464,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Cao")</f>
@@ -8388,7 +8472,7 @@
       </c>
       <c r="C37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Thấp")</f>
@@ -8396,16 +8480,16 @@
       </c>
       <c r="E37" s="12" t="n">
         <f aca="false">SUM(B37:D37)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>276</v>
+        <v>160</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C38" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Trung")</f>
@@ -8417,79 +8501,100 @@
       </c>
       <c r="E38" s="12" t="n">
         <f aca="false">SUM(B38:D38)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B39" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="12" t="s">
-        <v>809</v>
-      </c>
-      <c r="B39" s="12" t="n">
-        <f aca="false">SUM(B2:B38)</f>
+      <c r="D39" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="12" t="n">
+        <f aca="false">SUM(B39:D39)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="12" t="s">
+        <v>820</v>
+      </c>
+      <c r="B40" s="12" t="n">
+        <f aca="false">SUM(B2:B39)</f>
         <v>24</v>
       </c>
-      <c r="C39" s="12" t="n">
-        <f aca="false">SUM(C2:C38)</f>
-        <v>35</v>
-      </c>
-      <c r="D39" s="12" t="n">
-        <f aca="false">SUM(D2:D38)</f>
+      <c r="C40" s="12" t="n">
+        <f aca="false">SUM(C2:C39)</f>
+        <v>36</v>
+      </c>
+      <c r="D40" s="12" t="n">
+        <f aca="false">SUM(D2:D39)</f>
         <v>21</v>
       </c>
-      <c r="E39" s="12" t="n">
-        <f aca="false">SUM(E2:E38)</f>
-        <v>80</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12" t="s">
+      <c r="E40" s="12" t="n">
+        <f aca="false">SUM(E2:E39)</f>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B41" s="12" t="s">
-        <v>810</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="11" t="s">
-        <v>811</v>
-      </c>
-      <c r="B42" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A42)</f>
-        <v>0</v>
+      <c r="B42" s="12" t="s">
+        <v>821</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>444</v>
+        <v>822</v>
       </c>
       <c r="B43" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
       <c r="B44" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A44)</f>
-        <v>77</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>812</v>
+        <v>37</v>
       </c>
       <c r="B45" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A45)</f>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="11" t="s">
+        <v>823</v>
+      </c>
+      <c r="B46" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A46)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="13" t="s">
-        <v>813</v>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="13" t="s">
+        <v>824</v>
       </c>
     </row>
   </sheetData>
@@ -8517,170 +8622,170 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>814</v>
+        <v>825</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>815</v>
+        <v>826</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>816</v>
+        <v>827</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>817</v>
+        <v>828</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>818</v>
+      <c r="A4" s="14" t="s">
+        <v>829</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>819</v>
+        <v>830</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="14" t="s">
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>821</v>
+      <c r="A6" s="14" t="s">
+        <v>832</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>822</v>
+        <v>833</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>823</v>
+      <c r="A7" s="14" t="s">
+        <v>834</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>824</v>
+        <v>835</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="s">
-        <v>825</v>
+      <c r="A8" s="14" t="s">
+        <v>836</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>827</v>
+      <c r="A9" s="14" t="s">
+        <v>838</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>828</v>
+        <v>839</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
-        <v>829</v>
+      <c r="A10" s="14" t="s">
+        <v>840</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>830</v>
+        <v>841</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>831</v>
+      <c r="A11" s="14" t="s">
+        <v>842</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>832</v>
+        <v>843</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>833</v>
+      <c r="A12" s="14" t="s">
+        <v>844</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>834</v>
+        <v>845</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>835</v>
+      <c r="A13" s="14" t="s">
+        <v>846</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>836</v>
+        <v>847</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
-        <v>837</v>
+      <c r="A14" s="14" t="s">
+        <v>848</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>838</v>
+        <v>849</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>839</v>
+      <c r="A15" s="14" t="s">
+        <v>850</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>840</v>
+        <v>851</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>841</v>
+      <c r="A16" s="14" t="s">
+        <v>852</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>842</v>
+        <v>853</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="14" t="s">
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>843</v>
+        <v>854</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="s">
-        <v>844</v>
+      <c r="A18" s="14" t="s">
+        <v>855</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>845</v>
+        <v>856</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>846</v>
+      <c r="A19" s="14" t="s">
+        <v>857</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>847</v>
+        <v>858</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="s">
-        <v>848</v>
+      <c r="A20" s="14" t="s">
+        <v>859</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>849</v>
+        <v>860</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="14" t="s">
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>850</v>
+        <v>861</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-50 stale read after a write (flaky E2E on report shifts)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1331" uniqueCount="862">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="873">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -3061,6 +3061,39 @@
   </si>
   <si>
     <t xml:space="preserve">Chữ trên giấy in là cam kết với khách và thuế: đặt ở một nơi (payload), các máy in chỉ trình bày.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Báo cáo / API client</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js (api, apiReads)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI (E2E chập chờn) — có thể gặp trên SUNMI 4G chậm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đồng bộ / bộ nhớ đệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vừa mở Báo cáo đã lưu ca mới: danh sách ca không có ca vừa lưu tới khi tải lại; E2E 'a printer report while typing…' đỏ một lần (bấm 'Ca cả ngày' quá 15 s), chạy lại thì xanh.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">api() gộp các lệnh GET trùng đường dẫn đang bay (apiReads). Lệnh GET /report-shifts lúc mở trang còn đang bay khi chủ tiệm bấm Lưu; loadReportShifts sau PUT gộp vào lệnh GET cũ nên nhận dữ liệu trước khi lưu và ghi đè st.reportTemplates.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mọi lệnh ghi (khác GET) xóa apiReads lúc bắt đầu và lúc xong, nên lệnh đọc sau đó luôn gửi yêu cầu mới; lệnh đọc cũ xong muộn chỉ xóa đúng mục của chính nó.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tests/phattai-v185-read-after-write.test.mjs ('API a read after a write starts its own request instead of joining an older one', +3 test); scripts/e2e-staff.mjs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bộ nhớ đệm/gộp yêu cầu có bị vô hiệu sau mỗi lần ghi không? Lệnh đọc sau khi ghi có thể nhận câu trả lời của lệnh đọc gửi trước khi ghi không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7ff99ca</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -3532,8 +3565,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O82" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O82"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O83"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3796,7 +3829,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O82"/>
+  <dimension ref="A1:O83"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -6119,7 +6152,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>516</v>
       </c>
@@ -7667,6 +7700,53 @@
         <v>811</v>
       </c>
       <c r="O82" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="5" t="s">
+        <v>820</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D83" s="6" t="s">
+        <v>821</v>
+      </c>
+      <c r="E83" s="6" t="s">
+        <v>822</v>
+      </c>
+      <c r="F83" s="6" t="s">
+        <v>823</v>
+      </c>
+      <c r="G83" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="H83" s="6" t="s">
+        <v>824</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>825</v>
+      </c>
+      <c r="J83" s="6" t="s">
+        <v>826</v>
+      </c>
+      <c r="K83" s="6" t="s">
+        <v>827</v>
+      </c>
+      <c r="L83" s="6" t="s">
+        <v>828</v>
+      </c>
+      <c r="M83" s="6" t="s">
+        <v>829</v>
+      </c>
+      <c r="N83" s="6" t="s">
+        <v>830</v>
+      </c>
+      <c r="O83" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7703,7 +7783,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -7724,7 +7804,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>820</v>
+        <v>831</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8506,7 +8586,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>276</v>
+        <v>824</v>
       </c>
       <c r="B39" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Cao")</f>
@@ -8514,87 +8594,108 @@
       </c>
       <c r="C39" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D39" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E39" s="12" t="n">
         <f aca="false">SUM(B39:D39)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B40" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A40,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A40,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="12" t="s">
-        <v>820</v>
-      </c>
-      <c r="B40" s="12" t="n">
-        <f aca="false">SUM(B2:B39)</f>
+      <c r="D40" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A40,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="12" t="n">
+        <f aca="false">SUM(B40:D40)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="12" t="s">
+        <v>831</v>
+      </c>
+      <c r="B41" s="12" t="n">
+        <f aca="false">SUM(B2:B40)</f>
         <v>24</v>
       </c>
-      <c r="C40" s="12" t="n">
-        <f aca="false">SUM(C2:C39)</f>
+      <c r="C41" s="12" t="n">
+        <f aca="false">SUM(C2:C40)</f>
         <v>36</v>
       </c>
-      <c r="D40" s="12" t="n">
-        <f aca="false">SUM(D2:D39)</f>
-        <v>21</v>
-      </c>
-      <c r="E40" s="12" t="n">
-        <f aca="false">SUM(E2:E39)</f>
-        <v>81</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="12" t="s">
+      <c r="D41" s="12" t="n">
+        <f aca="false">SUM(D2:D40)</f>
         <v>22</v>
       </c>
-      <c r="B42" s="12" t="s">
-        <v>821</v>
-      </c>
-    </row>
+      <c r="E41" s="12" t="n">
+        <f aca="false">SUM(E2:E40)</f>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="11" t="s">
-        <v>822</v>
-      </c>
-      <c r="B43" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A43)</f>
-        <v>0</v>
+      <c r="A43" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B43" s="12" t="s">
+        <v>832</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="11" t="s">
-        <v>444</v>
+        <v>833</v>
       </c>
       <c r="B44" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A44)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
       <c r="B45" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A45)</f>
-        <v>79</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>823</v>
+        <v>37</v>
       </c>
       <c r="B46" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A46)</f>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11" t="s">
+        <v>834</v>
+      </c>
+      <c r="B47" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A47)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13" t="s">
-        <v>824</v>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="13" t="s">
+        <v>835</v>
       </c>
     </row>
   </sheetData>
@@ -8622,10 +8723,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>825</v>
+        <v>836</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>826</v>
+        <v>837</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8633,7 +8734,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>827</v>
+        <v>838</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8641,15 +8742,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>828</v>
+        <v>839</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>829</v>
+        <v>840</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>830</v>
+        <v>841</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8657,95 +8758,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>831</v>
+        <v>842</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>832</v>
+        <v>843</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>833</v>
+        <v>844</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>834</v>
+        <v>845</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>835</v>
+        <v>846</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>836</v>
+        <v>847</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>837</v>
+        <v>848</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>838</v>
+        <v>849</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>839</v>
+        <v>850</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>840</v>
+        <v>851</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>841</v>
+        <v>852</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>842</v>
+        <v>853</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>843</v>
+        <v>854</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>844</v>
+        <v>855</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>845</v>
+        <v>856</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>846</v>
+        <v>857</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>847</v>
+        <v>858</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>848</v>
+        <v>859</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>849</v>
+        <v>860</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>850</v>
+        <v>861</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>851</v>
+        <v>862</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>852</v>
+        <v>863</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8753,31 +8854,31 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>854</v>
+        <v>865</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>855</v>
+        <v>866</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>856</v>
+        <v>867</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>858</v>
+        <v>869</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>859</v>
+        <v>870</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>860</v>
+        <v>871</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8785,7 +8886,7 @@
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>861</v>
+        <v>872</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug list: PT-51 redraw unticked a person in the fixed-shift form
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6iJ6JkZZiX5XUHPZcWHTL
</commit_message>
<xml_diff>
--- a/docs/LotusPOS_BugList.xlsx
+++ b/docs/LotusPOS_BugList.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="873">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1363" uniqueCount="884">
   <si>
     <t xml:space="preserve">Kho kinh nghiệm lỗi của Lotus POS. Mỗi lỗi phát hiện hoặc sửa (kể cả do AI khác sửa) thêm MỘT dòng vào sheet Bug List.</t>
   </si>
@@ -3094,6 +3094,39 @@
   </si>
   <si>
     <t xml:space="preserve">7ff99ca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PT-51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Xếp ca / Form</t>
+  </si>
+  <si>
+    <t xml:space="preserve">public/staff/staff.js (keepDrafts, rememberField)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI (mô phỏng chập chờn) — gặp được trên SUNMI khi mạng chậm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Render xóa dữ liệu nhập</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ca cố định lưu thiếu người đã tick: mô phỏng 'Ca sáng' mất linh (người tick đầu tiên) một lần trên CI, chạy lại thì xanh.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bản nháp form (PT-32) chỉ giữ ô chữ và ô chọn; checkbox bị loại khỏi draftable. Bấm vào Xếp ca chạy render() rồi refresh(); khi refresh còn đang chờ mạng mà người dùng đã tick, render() ở cuối refresh vẽ lại form và bỏ tick, rồi bấm Lưu gửi thiếu người.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Giữ cả trạng thái checkbox trong bản nháp (khóa tên=giá trị), nghe cả sự kiện input và change; keepDrafts đặt lại checked sau mỗi render. Bản nháp vẫn bị xóa khi lưu thành công hoặc đổi màn hình.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scripts/sim-browser.mjs ('Handheld: a person ticked in the fixed-shift form stays ticked when the screen redraws (PT-51)'); tests/phattai-v178-buglist.test.mjs (PT-32)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Render có giữ MỌI loại ô (chữ, chọn, checkbox, radio) người dùng vừa đổi không? Có test nào tick/gõ rồi ép render lại không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">368145f</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng</t>
@@ -3565,8 +3598,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O83" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:O83"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Bugs" displayName="Bugs" ref="A1:O84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:O84"/>
   <tableColumns count="15">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Ngày phát hiện"/>
@@ -3829,7 +3862,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O83"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
@@ -7703,7 +7736,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="5" t="s">
         <v>820</v>
       </c>
@@ -7747,6 +7780,53 @@
         <v>830</v>
       </c>
       <c r="O83" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>832</v>
+      </c>
+      <c r="E84" s="6" t="s">
+        <v>833</v>
+      </c>
+      <c r="F84" s="6" t="s">
+        <v>834</v>
+      </c>
+      <c r="G84" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="H84" s="6" t="s">
+        <v>835</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>836</v>
+      </c>
+      <c r="J84" s="6" t="s">
+        <v>837</v>
+      </c>
+      <c r="K84" s="6" t="s">
+        <v>838</v>
+      </c>
+      <c r="L84" s="6" t="s">
+        <v>839</v>
+      </c>
+      <c r="M84" s="6" t="s">
+        <v>840</v>
+      </c>
+      <c r="N84" s="6" t="s">
+        <v>841</v>
+      </c>
+      <c r="O84" s="6" t="s">
         <v>37</v>
       </c>
     </row>
@@ -7783,7 +7863,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -7804,7 +7884,7 @@
         <v>73</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>831</v>
+        <v>842</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8439,7 +8519,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="11" t="s">
-        <v>644</v>
+        <v>835</v>
       </c>
       <c r="B32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Cao")</f>
@@ -8447,11 +8527,11 @@
       </c>
       <c r="C32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A32,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">SUM(B32:D32)</f>
@@ -8460,7 +8540,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>478</v>
+        <v>644</v>
       </c>
       <c r="B33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Cao")</f>
@@ -8472,16 +8552,16 @@
       </c>
       <c r="D33" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A33,'Bug List'!$G:$G,"Thấp")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="12" t="n">
         <f aca="false">SUM(B33:D33)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="11" t="s">
-        <v>509</v>
+        <v>478</v>
       </c>
       <c r="B34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Cao")</f>
@@ -8489,20 +8569,20 @@
       </c>
       <c r="C34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Trung")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A34,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E34" s="12" t="n">
         <f aca="false">SUM(B34:D34)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>520</v>
+        <v>509</v>
       </c>
       <c r="B35" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A35,'Bug List'!$G:$G,"Cao")</f>
@@ -8523,7 +8603,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="s">
-        <v>222</v>
+        <v>520</v>
       </c>
       <c r="B36" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A36,'Bug List'!$G:$G,"Cao")</f>
@@ -8544,15 +8624,15 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>94</v>
+        <v>222</v>
       </c>
       <c r="B37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Cao")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D37" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A37,'Bug List'!$G:$G,"Thấp")</f>
@@ -8565,7 +8645,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="s">
-        <v>160</v>
+        <v>94</v>
       </c>
       <c r="B38" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Cao")</f>
@@ -8573,7 +8653,7 @@
       </c>
       <c r="C38" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D38" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A38,'Bug List'!$G:$G,"Thấp")</f>
@@ -8581,33 +8661,33 @@
       </c>
       <c r="E38" s="12" t="n">
         <f aca="false">SUM(B38:D38)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>824</v>
+        <v>160</v>
       </c>
       <c r="B39" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Cao")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C39" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Trung")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D39" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A39,'Bug List'!$G:$G,"Thấp")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E39" s="12" t="n">
         <f aca="false">SUM(B39:D39)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="s">
-        <v>276</v>
+        <v>824</v>
       </c>
       <c r="B40" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A40,'Bug List'!$G:$G,"Cao")</f>
@@ -8615,87 +8695,108 @@
       </c>
       <c r="C40" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A40,'Bug List'!$G:$G,"Trung")</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D40" s="11" t="n">
         <f aca="false">COUNTIFS('Bug List'!$H:$H,$A40,'Bug List'!$G:$G,"Thấp")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E40" s="12" t="n">
         <f aca="false">SUM(B40:D40)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="11" t="s">
+        <v>276</v>
+      </c>
+      <c r="B41" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A41,'Bug List'!$G:$G,"Cao")</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A41,'Bug List'!$G:$G,"Trung")</f>
         <v>2</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="12" t="s">
-        <v>831</v>
-      </c>
-      <c r="B41" s="12" t="n">
-        <f aca="false">SUM(B2:B40)</f>
+      <c r="D41" s="11" t="n">
+        <f aca="false">COUNTIFS('Bug List'!$H:$H,$A41,'Bug List'!$G:$G,"Thấp")</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="12" t="n">
+        <f aca="false">SUM(B41:D41)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="12" t="s">
+        <v>842</v>
+      </c>
+      <c r="B42" s="12" t="n">
+        <f aca="false">SUM(B2:B41)</f>
         <v>24</v>
       </c>
-      <c r="C41" s="12" t="n">
-        <f aca="false">SUM(C2:C40)</f>
-        <v>36</v>
-      </c>
-      <c r="D41" s="12" t="n">
-        <f aca="false">SUM(D2:D40)</f>
+      <c r="C42" s="12" t="n">
+        <f aca="false">SUM(C2:C41)</f>
+        <v>37</v>
+      </c>
+      <c r="D42" s="12" t="n">
+        <f aca="false">SUM(D2:D41)</f>
         <v>22</v>
       </c>
-      <c r="E41" s="12" t="n">
-        <f aca="false">SUM(E2:E40)</f>
-        <v>82</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="12" t="s">
+      <c r="E42" s="12" t="n">
+        <f aca="false">SUM(E2:E41)</f>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B43" s="12" t="s">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="11" t="s">
-        <v>833</v>
-      </c>
-      <c r="B44" s="11" t="n">
-        <f aca="false">COUNTIF('Bug List'!$O:$O,A44)</f>
-        <v>0</v>
+      <c r="B44" s="12" t="s">
+        <v>843</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>444</v>
+        <v>844</v>
       </c>
       <c r="B45" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A45)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="s">
-        <v>37</v>
+        <v>444</v>
       </c>
       <c r="B46" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A46)</f>
-        <v>80</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>834</v>
+        <v>37</v>
       </c>
       <c r="B47" s="11" t="n">
         <f aca="false">COUNTIF('Bug List'!$O:$O,A47)</f>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="11" t="s">
+        <v>845</v>
+      </c>
+      <c r="B48" s="11" t="n">
+        <f aca="false">COUNTIF('Bug List'!$O:$O,A48)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="13" t="s">
-        <v>835</v>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="13" t="s">
+        <v>846</v>
       </c>
     </row>
   </sheetData>
@@ -8723,10 +8824,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>836</v>
+        <v>847</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>837</v>
+        <v>848</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8734,7 +8835,7 @@
         <v>149</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>838</v>
+        <v>849</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8742,15 +8843,15 @@
         <v>53</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>839</v>
+        <v>850</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>840</v>
+        <v>851</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>841</v>
+        <v>852</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8758,95 +8859,95 @@
         <v>115</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>842</v>
+        <v>853</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>843</v>
+        <v>854</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>844</v>
+        <v>855</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>845</v>
+        <v>856</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>846</v>
+        <v>857</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>847</v>
+        <v>858</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>848</v>
+        <v>859</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>849</v>
+        <v>860</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>850</v>
+        <v>861</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>851</v>
+        <v>862</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>852</v>
+        <v>863</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>853</v>
+        <v>864</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>854</v>
+        <v>865</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>855</v>
+        <v>866</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>856</v>
+        <v>867</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>857</v>
+        <v>868</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>858</v>
+        <v>869</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>859</v>
+        <v>870</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>860</v>
+        <v>871</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>861</v>
+        <v>872</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>862</v>
+        <v>873</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>863</v>
+        <v>874</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>864</v>
+        <v>875</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8854,31 +8955,31 @@
         <v>287</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>865</v>
+        <v>876</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>866</v>
+        <v>877</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>867</v>
+        <v>878</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>868</v>
+        <v>879</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>869</v>
+        <v>880</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>870</v>
+        <v>881</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>871</v>
+        <v>882</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8886,7 +8987,7 @@
         <v>428</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>872</v>
+        <v>883</v>
       </c>
     </row>
   </sheetData>

</xml_diff>